<commit_message>
Actualización automática ERP - Pedidos Transmicion - 21/09/2026 06:06:16
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32651B99-BD7A-4965-A433-19B9A34D9B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C637227-1A6A-4661-AABC-91BCCD4F390E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{AA43A1BD-2EBC-4E6B-A8C0-B06F38CB813E}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A920312E-E1EC-41E0-BA63-71AD203645D7}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -4510,7 +4510,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46B58B86-13CC-4B56-BCB8-3994B39D6CEE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C027D2E-1035-4ECD-AF9F-77E6C835F9D2}">
   <dimension ref="A1:G742"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 28/09/2026 06:12:51
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC35C15E-CEF6-4CD9-874B-301CA3196F6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6025169-11E7-424F-BDE5-C5E0874C5066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{43C0AF68-44A9-44DD-B3B4-D244A6EA0A61}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{386BEF06-9D30-4982-9932-AAD1C352A85A}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -4468,7 +4468,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26AA8AD9-1316-498E-AEC1-3BB3967F5A69}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C499A68-4AD1-4B16-A9E9-40FD10C7A706}">
   <dimension ref="A1:G716"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 02/10/2026 10:46:31
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB124B78-91C8-45CE-8A9B-E5A31D937093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{59A825F2-9151-4107-AA5E-81FF6269FF3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{10659DCE-AFA0-42E0-A2F0-BEF5F2A0F442}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{59BFD859-169D-4D95-8EF9-465B517AD1D0}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3037" uniqueCount="1160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3142" uniqueCount="1187">
   <si>
     <t>0001</t>
   </si>
@@ -3223,6 +3223,9 @@
     <t xml:space="preserve">  216822</t>
   </si>
   <si>
+    <t xml:space="preserve">  216823</t>
+  </si>
+  <si>
     <t xml:space="preserve">  216824</t>
   </si>
   <si>
@@ -3244,6 +3247,90 @@
     <t xml:space="preserve">  216828</t>
   </si>
   <si>
+    <t xml:space="preserve">  216830</t>
+  </si>
+  <si>
+    <t>VC09</t>
+  </si>
+  <si>
+    <t>VICENTELLI CARLOS ROBERTO - CASA DIVI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216831</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216832</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216833</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216835</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216837</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216838</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216839</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216840</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216841</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216842</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216843</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216844</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216845</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216846</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216847</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216848</t>
+  </si>
+  <si>
+    <t>MF13</t>
+  </si>
+  <si>
+    <t>MAS FERRETERIAS S.A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216849</t>
+  </si>
+  <si>
+    <t>HC03</t>
+  </si>
+  <si>
+    <t>HIJOS DE RAFAEL CONTI S.A. - CONTI MATERIALES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216850</t>
+  </si>
+  <si>
+    <t>GL08</t>
+  </si>
+  <si>
+    <t>GUTIERREZ LUIS ENRIQUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  216851</t>
+  </si>
+  <si>
     <t>0004</t>
   </si>
   <si>
@@ -3310,9 +3397,6 @@
     <t xml:space="preserve">    2959</t>
   </si>
   <si>
-    <t xml:space="preserve">    2974</t>
-  </si>
-  <si>
     <t xml:space="preserve">    2977</t>
   </si>
   <si>
@@ -3325,13 +3409,7 @@
     <t xml:space="preserve">    2992</t>
   </si>
   <si>
-    <t xml:space="preserve">    2994</t>
-  </si>
-  <si>
-    <t>PA01</t>
-  </si>
-  <si>
-    <t>VARIOS</t>
+    <t xml:space="preserve">    2996</t>
   </si>
   <si>
     <t>4444</t>
@@ -3418,10 +3496,13 @@
     <t xml:space="preserve">    2644</t>
   </si>
   <si>
-    <t xml:space="preserve">    2674</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2675</t>
+    <t xml:space="preserve">    2686</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    2688</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    2689</t>
   </si>
   <si>
     <t>9999</t>
@@ -3949,31 +4030,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C06B3F2-EB6E-462E-BBD0-666D451C5748}">
-  <dimension ref="A1:G607"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DDFE0BE-7CA2-47A9-9B7D-D36B993F240A}">
+  <dimension ref="A1:G628"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>1153</v>
+        <v>1180</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1154</v>
+        <v>1181</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1155</v>
+        <v>1182</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>1156</v>
+        <v>1183</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>1157</v>
+        <v>1184</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>1158</v>
+        <v>1185</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>1159</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -5847,7 +5928,7 @@
         <v>206</v>
       </c>
       <c r="C83" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D83" t="s">
         <v>37</v>
@@ -5985,7 +6066,7 @@
         <v>220</v>
       </c>
       <c r="C89" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D89" t="s">
         <v>37</v>
@@ -6238,7 +6319,7 @@
         <v>241</v>
       </c>
       <c r="C100" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D100" t="s">
         <v>37</v>
@@ -6284,7 +6365,7 @@
         <v>243</v>
       </c>
       <c r="C102" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D102" t="s">
         <v>16</v>
@@ -6491,7 +6572,7 @@
         <v>264</v>
       </c>
       <c r="C111" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D111" t="s">
         <v>140</v>
@@ -6652,7 +6733,7 @@
         <v>281</v>
       </c>
       <c r="C118" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D118" t="s">
         <v>140</v>
@@ -6721,7 +6802,7 @@
         <v>288</v>
       </c>
       <c r="C121" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D121" t="s">
         <v>289</v>
@@ -6836,7 +6917,7 @@
         <v>297</v>
       </c>
       <c r="C126" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D126" t="s">
         <v>298</v>
@@ -6859,7 +6940,7 @@
         <v>300</v>
       </c>
       <c r="C127" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D127" t="s">
         <v>140</v>
@@ -6882,7 +6963,7 @@
         <v>301</v>
       </c>
       <c r="C128" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D128" t="s">
         <v>140</v>
@@ -7503,7 +7584,7 @@
         <v>340</v>
       </c>
       <c r="C155" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D155" t="s">
         <v>37</v>
@@ -7572,7 +7653,7 @@
         <v>347</v>
       </c>
       <c r="C158" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D158" t="s">
         <v>348</v>
@@ -7710,7 +7791,7 @@
         <v>361</v>
       </c>
       <c r="C164" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D164" t="s">
         <v>16</v>
@@ -7756,7 +7837,7 @@
         <v>365</v>
       </c>
       <c r="C166" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D166" t="s">
         <v>223</v>
@@ -8193,7 +8274,7 @@
         <v>400</v>
       </c>
       <c r="C185" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D185" t="s">
         <v>37</v>
@@ -8699,7 +8780,7 @@
         <v>452</v>
       </c>
       <c r="C207" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D207" t="s">
         <v>185</v>
@@ -8860,7 +8941,7 @@
         <v>469</v>
       </c>
       <c r="C214" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D214" t="s">
         <v>470</v>
@@ -8952,7 +9033,7 @@
         <v>477</v>
       </c>
       <c r="C218" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D218" t="s">
         <v>37</v>
@@ -9343,7 +9424,7 @@
         <v>516</v>
       </c>
       <c r="C235" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D235" t="s">
         <v>517</v>
@@ -9527,7 +9608,7 @@
         <v>532</v>
       </c>
       <c r="C243" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D243" t="s">
         <v>140</v>
@@ -9803,7 +9884,7 @@
         <v>548</v>
       </c>
       <c r="C255" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D255" t="s">
         <v>37</v>
@@ -10148,7 +10229,7 @@
         <v>585</v>
       </c>
       <c r="C270" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D270" t="s">
         <v>586</v>
@@ -10240,7 +10321,7 @@
         <v>593</v>
       </c>
       <c r="C274" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D274" t="s">
         <v>48</v>
@@ -10378,7 +10459,7 @@
         <v>603</v>
       </c>
       <c r="C280" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D280" t="s">
         <v>604</v>
@@ -10401,7 +10482,7 @@
         <v>606</v>
       </c>
       <c r="C281" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D281" t="s">
         <v>604</v>
@@ -10424,7 +10505,7 @@
         <v>607</v>
       </c>
       <c r="C282" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D282" t="s">
         <v>608</v>
@@ -10516,7 +10597,7 @@
         <v>615</v>
       </c>
       <c r="C286" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D286" t="s">
         <v>616</v>
@@ -10608,7 +10689,7 @@
         <v>627</v>
       </c>
       <c r="C290" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D290" t="s">
         <v>37</v>
@@ -10631,7 +10712,7 @@
         <v>628</v>
       </c>
       <c r="C291" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D291" t="s">
         <v>37</v>
@@ -10838,7 +10919,7 @@
         <v>641</v>
       </c>
       <c r="C300" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D300" t="s">
         <v>642</v>
@@ -10861,7 +10942,7 @@
         <v>644</v>
       </c>
       <c r="C301" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D301" t="s">
         <v>517</v>
@@ -11275,7 +11356,7 @@
         <v>690</v>
       </c>
       <c r="C319" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D319" t="s">
         <v>691</v>
@@ -11321,7 +11402,7 @@
         <v>696</v>
       </c>
       <c r="C321" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D321" t="s">
         <v>81</v>
@@ -11620,7 +11701,7 @@
         <v>711</v>
       </c>
       <c r="C334" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D334" t="s">
         <v>712</v>
@@ -11643,7 +11724,7 @@
         <v>714</v>
       </c>
       <c r="C335" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D335" t="s">
         <v>715</v>
@@ -11758,7 +11839,7 @@
         <v>727</v>
       </c>
       <c r="C340" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D340" t="s">
         <v>172</v>
@@ -11804,7 +11885,7 @@
         <v>731</v>
       </c>
       <c r="C342" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D342" t="s">
         <v>200</v>
@@ -11896,7 +11977,7 @@
         <v>735</v>
       </c>
       <c r="C346" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D346" t="s">
         <v>179</v>
@@ -11942,7 +12023,7 @@
         <v>737</v>
       </c>
       <c r="C348" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D348" t="s">
         <v>16</v>
@@ -11988,7 +12069,7 @@
         <v>741</v>
       </c>
       <c r="C350" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D350" t="s">
         <v>172</v>
@@ -12011,7 +12092,7 @@
         <v>742</v>
       </c>
       <c r="C351" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D351" t="s">
         <v>172</v>
@@ -12034,7 +12115,7 @@
         <v>743</v>
       </c>
       <c r="C352" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D352" t="s">
         <v>223</v>
@@ -12195,7 +12276,7 @@
         <v>754</v>
       </c>
       <c r="C359" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D359" t="s">
         <v>81</v>
@@ -12287,7 +12368,7 @@
         <v>760</v>
       </c>
       <c r="C363" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D363" t="s">
         <v>761</v>
@@ -12402,7 +12483,7 @@
         <v>767</v>
       </c>
       <c r="C368" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D368" t="s">
         <v>37</v>
@@ -12471,7 +12552,7 @@
         <v>772</v>
       </c>
       <c r="C371" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D371" t="s">
         <v>87</v>
@@ -12517,7 +12598,7 @@
         <v>774</v>
       </c>
       <c r="C373" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D373" t="s">
         <v>87</v>
@@ -12563,7 +12644,7 @@
         <v>776</v>
       </c>
       <c r="C375" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D375" t="s">
         <v>87</v>
@@ -13368,7 +13449,7 @@
         <v>839</v>
       </c>
       <c r="C410" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D410" t="s">
         <v>840</v>
@@ -13414,7 +13495,7 @@
         <v>843</v>
       </c>
       <c r="C412" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D412" t="s">
         <v>844</v>
@@ -13552,7 +13633,7 @@
         <v>859</v>
       </c>
       <c r="C418" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D418" t="s">
         <v>185</v>
@@ -13667,7 +13748,7 @@
         <v>868</v>
       </c>
       <c r="C423" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D423" t="s">
         <v>869</v>
@@ -13736,7 +13817,7 @@
         <v>875</v>
       </c>
       <c r="C426" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D426" t="s">
         <v>876</v>
@@ -13782,7 +13863,7 @@
         <v>879</v>
       </c>
       <c r="C428" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D428" t="s">
         <v>16</v>
@@ -14265,7 +14346,7 @@
         <v>916</v>
       </c>
       <c r="C449" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D449" t="s">
         <v>185</v>
@@ -14334,7 +14415,7 @@
         <v>921</v>
       </c>
       <c r="C452" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D452" t="s">
         <v>922</v>
@@ -14380,7 +14461,7 @@
         <v>927</v>
       </c>
       <c r="C454" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D454" t="s">
         <v>470</v>
@@ -14449,7 +14530,7 @@
         <v>934</v>
       </c>
       <c r="C457" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D457" t="s">
         <v>935</v>
@@ -14495,7 +14576,7 @@
         <v>938</v>
       </c>
       <c r="C459" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D459" t="s">
         <v>939</v>
@@ -14518,7 +14599,7 @@
         <v>941</v>
       </c>
       <c r="C460" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D460" t="s">
         <v>942</v>
@@ -14541,7 +14622,7 @@
         <v>944</v>
       </c>
       <c r="C461" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D461" t="s">
         <v>945</v>
@@ -14564,7 +14645,7 @@
         <v>947</v>
       </c>
       <c r="C462" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D462" t="s">
         <v>948</v>
@@ -14587,7 +14668,7 @@
         <v>950</v>
       </c>
       <c r="C463" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D463" t="s">
         <v>655</v>
@@ -14633,7 +14714,7 @@
         <v>952</v>
       </c>
       <c r="C465" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D465" t="s">
         <v>953</v>
@@ -14656,7 +14737,7 @@
         <v>955</v>
       </c>
       <c r="C466" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D466" t="s">
         <v>945</v>
@@ -14702,7 +14783,7 @@
         <v>957</v>
       </c>
       <c r="C468" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D468" t="s">
         <v>140</v>
@@ -14771,7 +14852,7 @@
         <v>960</v>
       </c>
       <c r="C471" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D471" t="s">
         <v>140</v>
@@ -14794,7 +14875,7 @@
         <v>961</v>
       </c>
       <c r="C472" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D472" t="s">
         <v>140</v>
@@ -14817,7 +14898,7 @@
         <v>962</v>
       </c>
       <c r="C473" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D473" t="s">
         <v>608</v>
@@ -14840,7 +14921,7 @@
         <v>963</v>
       </c>
       <c r="C474" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D474" t="s">
         <v>608</v>
@@ -14863,7 +14944,7 @@
         <v>964</v>
       </c>
       <c r="C475" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D475" t="s">
         <v>608</v>
@@ -14886,7 +14967,7 @@
         <v>965</v>
       </c>
       <c r="C476" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D476" t="s">
         <v>608</v>
@@ -14909,7 +14990,7 @@
         <v>966</v>
       </c>
       <c r="C477" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D477" t="s">
         <v>967</v>
@@ -15208,7 +15289,7 @@
         <v>983</v>
       </c>
       <c r="C490" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D490" t="s">
         <v>45</v>
@@ -15231,7 +15312,7 @@
         <v>984</v>
       </c>
       <c r="C491" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D491" t="s">
         <v>45</v>
@@ -16220,7 +16301,7 @@
         <v>1045</v>
       </c>
       <c r="C534" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D534" t="s">
         <v>608</v>
@@ -16499,16 +16580,16 @@
         <v>80</v>
       </c>
       <c r="D546" t="s">
-        <v>918</v>
+        <v>608</v>
       </c>
       <c r="E546" t="s">
-        <v>919</v>
+        <v>609</v>
       </c>
       <c r="F546" s="1">
         <v>46296</v>
       </c>
       <c r="G546" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="547" spans="1:7" x14ac:dyDescent="0.2">
@@ -16522,10 +16603,10 @@
         <v>80</v>
       </c>
       <c r="D547" t="s">
-        <v>847</v>
+        <v>918</v>
       </c>
       <c r="E547" t="s">
-        <v>848</v>
+        <v>919</v>
       </c>
       <c r="F547" s="1">
         <v>46296</v>
@@ -16568,10 +16649,10 @@
         <v>80</v>
       </c>
       <c r="D549" t="s">
-        <v>1071</v>
+        <v>847</v>
       </c>
       <c r="E549" t="s">
-        <v>1072</v>
+        <v>848</v>
       </c>
       <c r="F549" s="1">
         <v>46296</v>
@@ -16585,16 +16666,16 @@
         <v>0</v>
       </c>
       <c r="B550" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C550" t="s">
+        <v>80</v>
+      </c>
+      <c r="D550" t="s">
+        <v>1072</v>
+      </c>
+      <c r="E550" t="s">
         <v>1073</v>
-      </c>
-      <c r="C550" t="s">
-        <v>80</v>
-      </c>
-      <c r="D550" t="s">
-        <v>1071</v>
-      </c>
-      <c r="E550" t="s">
-        <v>1072</v>
       </c>
       <c r="F550" s="1">
         <v>46296</v>
@@ -16605,122 +16686,122 @@
     </row>
     <row r="551" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A551" t="s">
+        <v>0</v>
+      </c>
+      <c r="B551" t="s">
         <v>1074</v>
       </c>
-      <c r="B551" t="s">
-        <v>1075</v>
-      </c>
       <c r="C551" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D551" t="s">
-        <v>200</v>
+        <v>1072</v>
       </c>
       <c r="E551" t="s">
-        <v>201</v>
+        <v>1073</v>
       </c>
       <c r="F551" s="1">
-        <v>46148</v>
+        <v>46296</v>
       </c>
       <c r="G551" s="1">
-        <v>46149</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="552" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A552" t="s">
-        <v>1074</v>
+        <v>0</v>
       </c>
       <c r="B552" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C552" t="s">
+        <v>80</v>
+      </c>
+      <c r="D552" t="s">
         <v>1076</v>
       </c>
-      <c r="C552" t="s">
-        <v>2</v>
-      </c>
-      <c r="D552" t="s">
-        <v>112</v>
-      </c>
       <c r="E552" t="s">
-        <v>113</v>
+        <v>1077</v>
       </c>
       <c r="F552" s="1">
-        <v>46268</v>
+        <v>46296</v>
       </c>
       <c r="G552" s="1">
-        <v>46268</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="553" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A553" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B553" t="s">
         <v>1078</v>
       </c>
       <c r="C553" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D553" t="s">
-        <v>41</v>
+        <v>761</v>
       </c>
       <c r="E553" t="s">
-        <v>42</v>
+        <v>762</v>
       </c>
       <c r="F553" s="1">
-        <v>46133</v>
+        <v>46296</v>
       </c>
       <c r="G553" s="1">
-        <v>46134</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="554" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A554" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B554" t="s">
         <v>1079</v>
       </c>
       <c r="C554" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D554" t="s">
-        <v>41</v>
+        <v>1061</v>
       </c>
       <c r="E554" t="s">
-        <v>42</v>
+        <v>1062</v>
       </c>
       <c r="F554" s="1">
-        <v>46134</v>
+        <v>46296</v>
       </c>
       <c r="G554" s="1">
-        <v>46134</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="555" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A555" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B555" t="s">
         <v>1080</v>
       </c>
       <c r="C555" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D555" t="s">
-        <v>19</v>
+        <v>1022</v>
       </c>
       <c r="E555" t="s">
-        <v>20</v>
+        <v>1023</v>
       </c>
       <c r="F555" s="1">
-        <v>46156</v>
+        <v>46296</v>
       </c>
       <c r="G555" s="1">
-        <v>46156</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="556" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A556" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B556" t="s">
         <v>1081</v>
@@ -16729,832 +16810,832 @@
         <v>80</v>
       </c>
       <c r="D556" t="s">
-        <v>1001</v>
+        <v>146</v>
       </c>
       <c r="E556" t="s">
-        <v>1002</v>
+        <v>147</v>
       </c>
       <c r="F556" s="1">
-        <v>46195</v>
+        <v>46296</v>
       </c>
       <c r="G556" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="557" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A557" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B557" t="s">
         <v>1082</v>
       </c>
       <c r="C557" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="D557" t="s">
-        <v>1083</v>
+        <v>304</v>
       </c>
       <c r="E557" t="s">
-        <v>1084</v>
+        <v>305</v>
       </c>
       <c r="F557" s="1">
-        <v>46209</v>
+        <v>46297</v>
       </c>
       <c r="G557" s="1">
-        <v>46218</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="558" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A558" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B558" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
       <c r="C558" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D558" t="s">
-        <v>939</v>
+        <v>807</v>
       </c>
       <c r="E558" t="s">
-        <v>940</v>
+        <v>808</v>
       </c>
       <c r="F558" s="1">
-        <v>46213</v>
+        <v>46297</v>
       </c>
       <c r="G558" s="1">
-        <v>46213</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="559" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A559" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B559" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
       <c r="C559" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="D559" t="s">
-        <v>1087</v>
+        <v>460</v>
       </c>
       <c r="E559" t="s">
-        <v>1088</v>
+        <v>461</v>
       </c>
       <c r="F559" s="1">
-        <v>46213</v>
+        <v>46297</v>
       </c>
       <c r="G559" s="1">
-        <v>46216</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="560" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A560" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B560" t="s">
-        <v>1089</v>
+        <v>1085</v>
       </c>
       <c r="C560" t="s">
         <v>80</v>
       </c>
       <c r="D560" t="s">
-        <v>1001</v>
+        <v>25</v>
       </c>
       <c r="E560" t="s">
-        <v>1002</v>
+        <v>26</v>
       </c>
       <c r="F560" s="1">
-        <v>46223</v>
+        <v>46297</v>
       </c>
       <c r="G560" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="561" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A561" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B561" t="s">
-        <v>1090</v>
+        <v>1086</v>
       </c>
       <c r="C561" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="D561" t="s">
-        <v>1087</v>
+        <v>37</v>
       </c>
       <c r="E561" t="s">
-        <v>1088</v>
+        <v>38</v>
       </c>
       <c r="F561" s="1">
-        <v>46224</v>
+        <v>46297</v>
       </c>
       <c r="G561" s="1">
-        <v>46224</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="562" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A562" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B562" t="s">
-        <v>1091</v>
+        <v>1087</v>
       </c>
       <c r="C562" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D562" t="s">
-        <v>1092</v>
+        <v>37</v>
       </c>
       <c r="E562" t="s">
-        <v>1093</v>
+        <v>38</v>
       </c>
       <c r="F562" s="1">
-        <v>46253</v>
+        <v>46297</v>
       </c>
       <c r="G562" s="1">
-        <v>46253</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="563" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A563" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B563" t="s">
-        <v>1094</v>
+        <v>1088</v>
       </c>
       <c r="C563" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D563" t="s">
-        <v>212</v>
+        <v>492</v>
       </c>
       <c r="E563" t="s">
-        <v>213</v>
+        <v>493</v>
       </c>
       <c r="F563" s="1">
-        <v>46273</v>
+        <v>46297</v>
       </c>
       <c r="G563" s="1">
-        <v>46274</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="564" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A564" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B564" t="s">
-        <v>1095</v>
+        <v>1089</v>
       </c>
       <c r="C564" t="s">
         <v>80</v>
       </c>
       <c r="D564" t="s">
-        <v>354</v>
+        <v>492</v>
       </c>
       <c r="E564" t="s">
-        <v>355</v>
+        <v>493</v>
       </c>
       <c r="F564" s="1">
-        <v>46284</v>
+        <v>46297</v>
       </c>
       <c r="G564" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="565" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A565" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B565" t="s">
-        <v>1096</v>
+        <v>1090</v>
       </c>
       <c r="C565" t="s">
         <v>80</v>
       </c>
       <c r="D565" t="s">
-        <v>1087</v>
+        <v>143</v>
       </c>
       <c r="E565" t="s">
-        <v>1088</v>
+        <v>144</v>
       </c>
       <c r="F565" s="1">
-        <v>46289</v>
+        <v>46297</v>
       </c>
       <c r="G565" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="566" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A566" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B566" t="s">
-        <v>1097</v>
+        <v>1091</v>
       </c>
       <c r="C566" t="s">
         <v>80</v>
       </c>
       <c r="D566" t="s">
-        <v>41</v>
+        <v>133</v>
       </c>
       <c r="E566" t="s">
-        <v>42</v>
+        <v>134</v>
       </c>
       <c r="F566" s="1">
-        <v>46289</v>
+        <v>46297</v>
       </c>
       <c r="G566" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="567" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A567" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B567" t="s">
-        <v>1098</v>
+        <v>1092</v>
       </c>
       <c r="C567" t="s">
         <v>80</v>
       </c>
       <c r="D567" t="s">
-        <v>304</v>
+        <v>48</v>
       </c>
       <c r="E567" t="s">
-        <v>305</v>
+        <v>49</v>
       </c>
       <c r="F567" s="1">
-        <v>46293</v>
+        <v>46297</v>
       </c>
       <c r="G567" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="568" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A568" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B568" t="s">
-        <v>1099</v>
+        <v>1093</v>
       </c>
       <c r="C568" t="s">
         <v>80</v>
       </c>
       <c r="D568" t="s">
-        <v>756</v>
+        <v>1094</v>
       </c>
       <c r="E568" t="s">
-        <v>757</v>
+        <v>1095</v>
       </c>
       <c r="F568" s="1">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="G568" s="1">
-        <v>46294</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="569" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A569" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B569" t="s">
-        <v>1100</v>
+        <v>1096</v>
       </c>
       <c r="C569" t="s">
         <v>80</v>
       </c>
       <c r="D569" t="s">
-        <v>1083</v>
+        <v>1097</v>
       </c>
       <c r="E569" t="s">
-        <v>1084</v>
+        <v>1098</v>
       </c>
       <c r="F569" s="1">
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="G569" s="1">
-        <v>46295</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="570" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A570" t="s">
-        <v>1077</v>
+        <v>0</v>
       </c>
       <c r="B570" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C570" t="s">
+        <v>80</v>
+      </c>
+      <c r="D570" t="s">
+        <v>1100</v>
+      </c>
+      <c r="E570" t="s">
         <v>1101</v>
       </c>
-      <c r="C570" t="s">
-        <v>80</v>
-      </c>
-      <c r="D570" t="s">
-        <v>1102</v>
-      </c>
-      <c r="E570" t="s">
-        <v>1103</v>
-      </c>
       <c r="F570" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="G570" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="571" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A571" t="s">
-        <v>1104</v>
+        <v>0</v>
       </c>
       <c r="B571" t="s">
-        <v>1105</v>
+        <v>1102</v>
       </c>
       <c r="C571" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="D571" t="s">
-        <v>1106</v>
+        <v>16</v>
       </c>
       <c r="E571" t="s">
-        <v>1107</v>
+        <v>17</v>
       </c>
       <c r="F571" s="1">
-        <v>46063</v>
+        <v>46297</v>
       </c>
       <c r="G571" s="1">
-        <v>46064</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="572" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A572" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B572" t="s">
         <v>1104</v>
       </c>
-      <c r="B572" t="s">
-        <v>1108</v>
-      </c>
       <c r="C572" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D572" t="s">
-        <v>57</v>
+        <v>200</v>
       </c>
       <c r="E572" t="s">
-        <v>58</v>
+        <v>201</v>
       </c>
       <c r="F572" s="1">
-        <v>46113</v>
+        <v>46148</v>
       </c>
       <c r="G572" s="1">
-        <v>46125</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="573" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A573" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="B573" t="s">
-        <v>1109</v>
+        <v>1105</v>
       </c>
       <c r="C573" t="s">
         <v>2</v>
       </c>
       <c r="D573" t="s">
-        <v>57</v>
+        <v>112</v>
       </c>
       <c r="E573" t="s">
-        <v>58</v>
+        <v>113</v>
       </c>
       <c r="F573" s="1">
-        <v>46125</v>
+        <v>46268</v>
       </c>
       <c r="G573" s="1">
-        <v>46125</v>
+        <v>46268</v>
       </c>
     </row>
     <row r="574" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A574" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B574" t="s">
-        <v>1110</v>
+        <v>1107</v>
       </c>
       <c r="C574" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D574" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="E574" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="F574" s="1">
-        <v>46126</v>
+        <v>46133</v>
       </c>
       <c r="G574" s="1">
-        <v>46126</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="575" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A575" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B575" t="s">
-        <v>1111</v>
+        <v>1108</v>
       </c>
       <c r="C575" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D575" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="E575" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="F575" s="1">
-        <v>46126</v>
+        <v>46134</v>
       </c>
       <c r="G575" s="1">
-        <v>46126</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="576" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A576" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B576" t="s">
-        <v>1112</v>
+        <v>1109</v>
       </c>
       <c r="C576" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D576" t="s">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="E576" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="F576" s="1">
-        <v>46128</v>
+        <v>46156</v>
       </c>
       <c r="G576" s="1">
-        <v>46128</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="577" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A577" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B577" t="s">
-        <v>1113</v>
+        <v>1110</v>
       </c>
       <c r="C577" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D577" t="s">
-        <v>57</v>
+        <v>1001</v>
       </c>
       <c r="E577" t="s">
-        <v>58</v>
+        <v>1002</v>
       </c>
       <c r="F577" s="1">
-        <v>46132</v>
+        <v>46195</v>
       </c>
       <c r="G577" s="1">
-        <v>46132</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="578" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A578" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B578" t="s">
-        <v>1114</v>
+        <v>1111</v>
       </c>
       <c r="C578" t="s">
-        <v>2</v>
+        <v>96</v>
       </c>
       <c r="D578" t="s">
-        <v>57</v>
+        <v>1112</v>
       </c>
       <c r="E578" t="s">
-        <v>58</v>
+        <v>1113</v>
       </c>
       <c r="F578" s="1">
-        <v>46161</v>
+        <v>46209</v>
       </c>
       <c r="G578" s="1">
-        <v>46161</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="579" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A579" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B579" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="C579" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D579" t="s">
-        <v>57</v>
+        <v>939</v>
       </c>
       <c r="E579" t="s">
-        <v>58</v>
+        <v>940</v>
       </c>
       <c r="F579" s="1">
-        <v>46174</v>
+        <v>46213</v>
       </c>
       <c r="G579" s="1">
-        <v>46174</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="580" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A580" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B580" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C580" t="s">
+        <v>96</v>
+      </c>
+      <c r="D580" t="s">
         <v>1116</v>
       </c>
-      <c r="C580" t="s">
-        <v>2</v>
-      </c>
-      <c r="D580" t="s">
-        <v>57</v>
-      </c>
       <c r="E580" t="s">
-        <v>58</v>
+        <v>1117</v>
       </c>
       <c r="F580" s="1">
-        <v>46174</v>
+        <v>46213</v>
       </c>
       <c r="G580" s="1">
-        <v>46174</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="581" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A581" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B581" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="C581" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D581" t="s">
-        <v>57</v>
+        <v>1001</v>
       </c>
       <c r="E581" t="s">
-        <v>58</v>
+        <v>1002</v>
       </c>
       <c r="F581" s="1">
-        <v>46195</v>
+        <v>46223</v>
       </c>
       <c r="G581" s="1">
-        <v>46252</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="582" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A582" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B582" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="C582" t="s">
-        <v>6</v>
+        <v>96</v>
       </c>
       <c r="D582" t="s">
-        <v>57</v>
+        <v>1116</v>
       </c>
       <c r="E582" t="s">
-        <v>58</v>
+        <v>1117</v>
       </c>
       <c r="F582" s="1">
-        <v>46210</v>
+        <v>46224</v>
       </c>
       <c r="G582" s="1">
-        <v>46210</v>
+        <v>46224</v>
       </c>
     </row>
     <row r="583" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A583" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B583" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="C583" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D583" t="s">
-        <v>57</v>
+        <v>1121</v>
       </c>
       <c r="E583" t="s">
-        <v>58</v>
+        <v>1122</v>
       </c>
       <c r="F583" s="1">
-        <v>46213</v>
+        <v>46253</v>
       </c>
       <c r="G583" s="1">
-        <v>46213</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="584" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A584" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B584" t="s">
-        <v>1120</v>
+        <v>1123</v>
       </c>
       <c r="C584" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D584" t="s">
-        <v>57</v>
+        <v>212</v>
       </c>
       <c r="E584" t="s">
-        <v>58</v>
+        <v>213</v>
       </c>
       <c r="F584" s="1">
-        <v>46218</v>
+        <v>46273</v>
       </c>
       <c r="G584" s="1">
-        <v>46252</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="585" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A585" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B585" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="C585" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D585" t="s">
-        <v>77</v>
+        <v>354</v>
       </c>
       <c r="E585" t="s">
-        <v>78</v>
+        <v>355</v>
       </c>
       <c r="F585" s="1">
-        <v>46226</v>
+        <v>46284</v>
       </c>
       <c r="G585" s="1">
-        <v>46226</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="586" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A586" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B586" t="s">
-        <v>1122</v>
+        <v>1125</v>
       </c>
       <c r="C586" t="s">
         <v>80</v>
       </c>
       <c r="D586" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="E586" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="F586" s="1">
-        <v>46227</v>
+        <v>46289</v>
       </c>
       <c r="G586" s="1">
-        <v>46252</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="587" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A587" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B587" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
       <c r="C587" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D587" t="s">
-        <v>57</v>
+        <v>304</v>
       </c>
       <c r="E587" t="s">
-        <v>58</v>
+        <v>305</v>
       </c>
       <c r="F587" s="1">
-        <v>46227</v>
+        <v>46293</v>
       </c>
       <c r="G587" s="1">
-        <v>46252</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="588" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A588" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B588" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="C588" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D588" t="s">
-        <v>57</v>
+        <v>756</v>
       </c>
       <c r="E588" t="s">
-        <v>58</v>
+        <v>757</v>
       </c>
       <c r="F588" s="1">
-        <v>46227</v>
+        <v>46294</v>
       </c>
       <c r="G588" s="1">
-        <v>46228</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="589" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A589" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B589" t="s">
-        <v>1125</v>
+        <v>1128</v>
       </c>
       <c r="C589" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D589" t="s">
-        <v>77</v>
+        <v>1112</v>
       </c>
       <c r="E589" t="s">
-        <v>78</v>
+        <v>1113</v>
       </c>
       <c r="F589" s="1">
-        <v>46230</v>
+        <v>46295</v>
       </c>
       <c r="G589" s="1">
-        <v>46252</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="590" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A590" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="B590" t="s">
-        <v>1126</v>
+        <v>1129</v>
       </c>
       <c r="C590" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D590" t="s">
-        <v>57</v>
+        <v>1112</v>
       </c>
       <c r="E590" t="s">
-        <v>58</v>
+        <v>1113</v>
       </c>
       <c r="F590" s="1">
-        <v>46231</v>
+        <v>46297</v>
       </c>
       <c r="G590" s="1">
-        <v>46231</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="591" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A591" t="s">
-        <v>1104</v>
+        <v>1130</v>
       </c>
       <c r="B591" t="s">
-        <v>1127</v>
+        <v>1131</v>
       </c>
       <c r="C591" t="s">
-        <v>6</v>
+        <v>96</v>
       </c>
       <c r="D591" t="s">
-        <v>57</v>
+        <v>1132</v>
       </c>
       <c r="E591" t="s">
-        <v>58</v>
+        <v>1133</v>
       </c>
       <c r="F591" s="1">
-        <v>46254</v>
+        <v>46063</v>
       </c>
       <c r="G591" s="1">
-        <v>46254</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="592" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A592" t="s">
-        <v>1104</v>
+        <v>1130</v>
       </c>
       <c r="B592" t="s">
-        <v>1128</v>
+        <v>1134</v>
       </c>
       <c r="C592" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D592" t="s">
         <v>57</v>
@@ -17563,21 +17644,21 @@
         <v>58</v>
       </c>
       <c r="F592" s="1">
-        <v>46255</v>
+        <v>46113</v>
       </c>
       <c r="G592" s="1">
-        <v>46255</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="593" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A593" t="s">
-        <v>1104</v>
+        <v>1130</v>
       </c>
       <c r="B593" t="s">
-        <v>1129</v>
+        <v>1135</v>
       </c>
       <c r="C593" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D593" t="s">
         <v>57</v>
@@ -17586,21 +17667,21 @@
         <v>58</v>
       </c>
       <c r="F593" s="1">
-        <v>46260</v>
+        <v>46125</v>
       </c>
       <c r="G593" s="1">
-        <v>46260</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="594" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A594" t="s">
-        <v>1104</v>
+        <v>1130</v>
       </c>
       <c r="B594" t="s">
-        <v>1130</v>
+        <v>1136</v>
       </c>
       <c r="C594" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D594" t="s">
         <v>57</v>
@@ -17609,21 +17690,21 @@
         <v>58</v>
       </c>
       <c r="F594" s="1">
-        <v>46289</v>
+        <v>46126</v>
       </c>
       <c r="G594" s="1">
-        <v>46289</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="595" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A595" t="s">
-        <v>1104</v>
+        <v>1130</v>
       </c>
       <c r="B595" t="s">
-        <v>1131</v>
+        <v>1137</v>
       </c>
       <c r="C595" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D595" t="s">
         <v>57</v>
@@ -17632,21 +17713,21 @@
         <v>58</v>
       </c>
       <c r="F595" s="1">
-        <v>46294</v>
+        <v>46126</v>
       </c>
       <c r="G595" s="1">
-        <v>46294</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="596" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A596" t="s">
-        <v>1104</v>
+        <v>1130</v>
       </c>
       <c r="B596" t="s">
-        <v>1132</v>
+        <v>1138</v>
       </c>
       <c r="C596" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D596" t="s">
         <v>57</v>
@@ -17655,21 +17736,21 @@
         <v>58</v>
       </c>
       <c r="F596" s="1">
-        <v>46296</v>
+        <v>46128</v>
       </c>
       <c r="G596" s="1">
-        <v>46296</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="597" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A597" t="s">
-        <v>1104</v>
+        <v>1130</v>
       </c>
       <c r="B597" t="s">
-        <v>1133</v>
+        <v>1139</v>
       </c>
       <c r="C597" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D597" t="s">
         <v>57</v>
@@ -17678,239 +17759,722 @@
         <v>58</v>
       </c>
       <c r="F597" s="1">
-        <v>46296</v>
+        <v>46132</v>
       </c>
       <c r="G597" s="1">
-        <v>46296</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="598" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A598" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B598" t="s">
-        <v>1135</v>
+        <v>1140</v>
       </c>
       <c r="C598" t="s">
         <v>2</v>
       </c>
       <c r="D598" t="s">
-        <v>1136</v>
+        <v>57</v>
       </c>
       <c r="E598" t="s">
-        <v>1137</v>
+        <v>58</v>
       </c>
       <c r="F598" s="1">
-        <v>46157</v>
+        <v>46161</v>
       </c>
       <c r="G598" s="1">
-        <v>46157</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="599" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A599" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B599" t="s">
-        <v>1138</v>
+        <v>1141</v>
       </c>
       <c r="C599" t="s">
         <v>2</v>
       </c>
       <c r="D599" t="s">
-        <v>1139</v>
+        <v>57</v>
       </c>
       <c r="E599" t="s">
-        <v>1140</v>
+        <v>58</v>
       </c>
       <c r="F599" s="1">
-        <v>46168</v>
+        <v>46174</v>
       </c>
       <c r="G599" s="1">
-        <v>46170</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="600" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A600" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B600" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="C600" t="s">
         <v>2</v>
       </c>
       <c r="D600" t="s">
-        <v>1136</v>
+        <v>57</v>
       </c>
       <c r="E600" t="s">
-        <v>1137</v>
+        <v>58</v>
       </c>
       <c r="F600" s="1">
-        <v>46244</v>
+        <v>46174</v>
       </c>
       <c r="G600" s="1">
-        <v>46244</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="601" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A601" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B601" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="C601" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D601" t="s">
-        <v>1136</v>
+        <v>57</v>
       </c>
       <c r="E601" t="s">
-        <v>1137</v>
+        <v>58</v>
       </c>
       <c r="F601" s="1">
-        <v>46247</v>
+        <v>46195</v>
       </c>
       <c r="G601" s="1">
-        <v>46247</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="602" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A602" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B602" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="C602" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D602" t="s">
-        <v>1144</v>
+        <v>57</v>
       </c>
       <c r="E602" t="s">
-        <v>1145</v>
+        <v>58</v>
       </c>
       <c r="F602" s="1">
-        <v>46247</v>
+        <v>46210</v>
       </c>
       <c r="G602" s="1">
-        <v>46247</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="603" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A603" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B603" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="C603" t="s">
         <v>2</v>
       </c>
       <c r="D603" t="s">
-        <v>1136</v>
+        <v>57</v>
       </c>
       <c r="E603" t="s">
-        <v>1137</v>
+        <v>58</v>
       </c>
       <c r="F603" s="1">
-        <v>46255</v>
+        <v>46213</v>
       </c>
       <c r="G603" s="1">
-        <v>46255</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="604" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A604" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B604" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="C604" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D604" t="s">
-        <v>1136</v>
+        <v>57</v>
       </c>
       <c r="E604" t="s">
-        <v>1137</v>
+        <v>58</v>
       </c>
       <c r="F604" s="1">
-        <v>46258</v>
+        <v>46218</v>
       </c>
       <c r="G604" s="1">
-        <v>46258</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="605" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A605" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B605" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="C605" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D605" t="s">
-        <v>1136</v>
+        <v>77</v>
       </c>
       <c r="E605" t="s">
-        <v>1137</v>
+        <v>78</v>
       </c>
       <c r="F605" s="1">
-        <v>46262</v>
+        <v>46226</v>
       </c>
       <c r="G605" s="1">
-        <v>46265</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="606" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A606" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B606" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="C606" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D606" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="E606" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="F606" s="1">
-        <v>46281</v>
+        <v>46227</v>
       </c>
       <c r="G606" s="1">
-        <v>46283</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="607" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A607" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B607" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C607" t="s">
+        <v>6</v>
+      </c>
+      <c r="D607" t="s">
+        <v>57</v>
+      </c>
+      <c r="E607" t="s">
+        <v>58</v>
+      </c>
+      <c r="F607" s="1">
+        <v>46227</v>
+      </c>
+      <c r="G607" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="608" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A608" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B608" t="s">
         <v>1150</v>
       </c>
-      <c r="C607" t="s">
-        <v>80</v>
-      </c>
-      <c r="D607" t="s">
+      <c r="C608" t="s">
+        <v>6</v>
+      </c>
+      <c r="D608" t="s">
+        <v>57</v>
+      </c>
+      <c r="E608" t="s">
+        <v>58</v>
+      </c>
+      <c r="F608" s="1">
+        <v>46227</v>
+      </c>
+      <c r="G608" s="1">
+        <v>46228</v>
+      </c>
+    </row>
+    <row r="609" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A609" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B609" t="s">
         <v>1151</v>
       </c>
-      <c r="E607" t="s">
+      <c r="C609" t="s">
+        <v>6</v>
+      </c>
+      <c r="D609" t="s">
+        <v>77</v>
+      </c>
+      <c r="E609" t="s">
+        <v>78</v>
+      </c>
+      <c r="F609" s="1">
+        <v>46230</v>
+      </c>
+      <c r="G609" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="610" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A610" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B610" t="s">
         <v>1152</v>
       </c>
-      <c r="F607" s="1">
+      <c r="C610" t="s">
+        <v>6</v>
+      </c>
+      <c r="D610" t="s">
+        <v>57</v>
+      </c>
+      <c r="E610" t="s">
+        <v>58</v>
+      </c>
+      <c r="F610" s="1">
+        <v>46231</v>
+      </c>
+      <c r="G610" s="1">
+        <v>46231</v>
+      </c>
+    </row>
+    <row r="611" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A611" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B611" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C611" t="s">
+        <v>6</v>
+      </c>
+      <c r="D611" t="s">
+        <v>57</v>
+      </c>
+      <c r="E611" t="s">
+        <v>58</v>
+      </c>
+      <c r="F611" s="1">
+        <v>46254</v>
+      </c>
+      <c r="G611" s="1">
+        <v>46254</v>
+      </c>
+    </row>
+    <row r="612" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A612" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B612" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C612" t="s">
+        <v>2</v>
+      </c>
+      <c r="D612" t="s">
+        <v>57</v>
+      </c>
+      <c r="E612" t="s">
+        <v>58</v>
+      </c>
+      <c r="F612" s="1">
+        <v>46255</v>
+      </c>
+      <c r="G612" s="1">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="613" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A613" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B613" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C613" t="s">
+        <v>6</v>
+      </c>
+      <c r="D613" t="s">
+        <v>57</v>
+      </c>
+      <c r="E613" t="s">
+        <v>58</v>
+      </c>
+      <c r="F613" s="1">
+        <v>46260</v>
+      </c>
+      <c r="G613" s="1">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="614" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A614" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B614" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C614" t="s">
+        <v>6</v>
+      </c>
+      <c r="D614" t="s">
+        <v>57</v>
+      </c>
+      <c r="E614" t="s">
+        <v>58</v>
+      </c>
+      <c r="F614" s="1">
+        <v>46289</v>
+      </c>
+      <c r="G614" s="1">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="615" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A615" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B615" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C615" t="s">
+        <v>6</v>
+      </c>
+      <c r="D615" t="s">
+        <v>57</v>
+      </c>
+      <c r="E615" t="s">
+        <v>58</v>
+      </c>
+      <c r="F615" s="1">
+        <v>46294</v>
+      </c>
+      <c r="G615" s="1">
+        <v>46294</v>
+      </c>
+    </row>
+    <row r="616" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A616" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B616" t="s">
+        <v>1158</v>
+      </c>
+      <c r="C616" t="s">
+        <v>80</v>
+      </c>
+      <c r="D616" t="s">
+        <v>57</v>
+      </c>
+      <c r="E616" t="s">
+        <v>58</v>
+      </c>
+      <c r="F616" s="1">
+        <v>46297</v>
+      </c>
+      <c r="G616" s="1">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="617" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A617" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B617" t="s">
+        <v>1159</v>
+      </c>
+      <c r="C617" t="s">
+        <v>80</v>
+      </c>
+      <c r="D617" t="s">
+        <v>57</v>
+      </c>
+      <c r="E617" t="s">
+        <v>58</v>
+      </c>
+      <c r="F617" s="1">
+        <v>46297</v>
+      </c>
+      <c r="G617" s="1">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="618" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A618" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B618" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C618" t="s">
+        <v>80</v>
+      </c>
+      <c r="D618" t="s">
+        <v>57</v>
+      </c>
+      <c r="E618" t="s">
+        <v>58</v>
+      </c>
+      <c r="F618" s="1">
+        <v>46297</v>
+      </c>
+      <c r="G618" s="1">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="619" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A619" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B619" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C619" t="s">
+        <v>2</v>
+      </c>
+      <c r="D619" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E619" t="s">
+        <v>1164</v>
+      </c>
+      <c r="F619" s="1">
+        <v>46157</v>
+      </c>
+      <c r="G619" s="1">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="620" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A620" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B620" t="s">
+        <v>1165</v>
+      </c>
+      <c r="C620" t="s">
+        <v>2</v>
+      </c>
+      <c r="D620" t="s">
+        <v>1166</v>
+      </c>
+      <c r="E620" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F620" s="1">
+        <v>46168</v>
+      </c>
+      <c r="G620" s="1">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="621" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A621" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B621" t="s">
+        <v>1168</v>
+      </c>
+      <c r="C621" t="s">
+        <v>2</v>
+      </c>
+      <c r="D621" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E621" t="s">
+        <v>1164</v>
+      </c>
+      <c r="F621" s="1">
+        <v>46244</v>
+      </c>
+      <c r="G621" s="1">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="622" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A622" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B622" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C622" t="s">
+        <v>2</v>
+      </c>
+      <c r="D622" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E622" t="s">
+        <v>1164</v>
+      </c>
+      <c r="F622" s="1">
+        <v>46247</v>
+      </c>
+      <c r="G622" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="623" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A623" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B623" t="s">
+        <v>1170</v>
+      </c>
+      <c r="C623" t="s">
+        <v>2</v>
+      </c>
+      <c r="D623" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E623" t="s">
+        <v>1172</v>
+      </c>
+      <c r="F623" s="1">
+        <v>46247</v>
+      </c>
+      <c r="G623" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="624" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A624" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B624" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C624" t="s">
+        <v>2</v>
+      </c>
+      <c r="D624" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E624" t="s">
+        <v>1164</v>
+      </c>
+      <c r="F624" s="1">
+        <v>46255</v>
+      </c>
+      <c r="G624" s="1">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="625" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A625" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B625" t="s">
+        <v>1174</v>
+      </c>
+      <c r="C625" t="s">
+        <v>2</v>
+      </c>
+      <c r="D625" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E625" t="s">
+        <v>1164</v>
+      </c>
+      <c r="F625" s="1">
+        <v>46258</v>
+      </c>
+      <c r="G625" s="1">
+        <v>46258</v>
+      </c>
+    </row>
+    <row r="626" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A626" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B626" t="s">
+        <v>1175</v>
+      </c>
+      <c r="C626" t="s">
+        <v>2</v>
+      </c>
+      <c r="D626" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E626" t="s">
+        <v>1164</v>
+      </c>
+      <c r="F626" s="1">
+        <v>46262</v>
+      </c>
+      <c r="G626" s="1">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="627" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A627" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B627" t="s">
+        <v>1176</v>
+      </c>
+      <c r="C627" t="s">
+        <v>6</v>
+      </c>
+      <c r="D627" t="s">
+        <v>13</v>
+      </c>
+      <c r="E627" t="s">
+        <v>14</v>
+      </c>
+      <c r="F627" s="1">
+        <v>46281</v>
+      </c>
+      <c r="G627" s="1">
+        <v>46283</v>
+      </c>
+    </row>
+    <row r="628" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A628" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B628" t="s">
+        <v>1177</v>
+      </c>
+      <c r="C628" t="s">
+        <v>80</v>
+      </c>
+      <c r="D628" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E628" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F628" s="1">
         <v>46296</v>
       </c>
-      <c r="G607" s="1">
+      <c r="G628" s="1">
         <v>46296</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 05/10/2026 06:02:42
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79D2DE02-734B-41C8-8A01-ECD818F10DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DB71B2E-2DDA-48DC-83A1-A73DE924BB67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3F782A1E-2DE1-4C43-A05B-9504CDFDF93D}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F6ABC71F-A7F9-4D66-AD6E-1BB0243FA047}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2982" uniqueCount="1135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="1133">
   <si>
     <t>0001</t>
   </si>
@@ -3226,13 +3226,7 @@
     <t xml:space="preserve">    2912</t>
   </si>
   <si>
-    <t xml:space="preserve">    2959</t>
-  </si>
-  <si>
     <t xml:space="preserve">    2977</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2984</t>
   </si>
   <si>
     <t xml:space="preserve">    2989</t>
@@ -3874,31 +3868,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4EBB095-BFE9-4105-AD13-1A86A742EC8E}">
-  <dimension ref="A1:G596"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D936D12B-A57F-41E8-914C-0CDC702B4F18}">
+  <dimension ref="A1:G594"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>1126</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1128</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>1129</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>1130</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>1131</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>1132</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>1133</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>1134</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -6232,7 +6226,7 @@
         <v>246</v>
       </c>
       <c r="C103" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D103" t="s">
         <v>247</v>
@@ -6301,7 +6295,7 @@
         <v>253</v>
       </c>
       <c r="C106" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D106" t="s">
         <v>254</v>
@@ -6439,7 +6433,7 @@
         <v>269</v>
       </c>
       <c r="C112" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D112" t="s">
         <v>37</v>
@@ -6508,7 +6502,7 @@
         <v>274</v>
       </c>
       <c r="C115" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D115" t="s">
         <v>37</v>
@@ -6646,7 +6640,7 @@
         <v>286</v>
       </c>
       <c r="C121" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D121" t="s">
         <v>37</v>
@@ -6692,7 +6686,7 @@
         <v>288</v>
       </c>
       <c r="C123" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D123" t="s">
         <v>37</v>
@@ -6715,7 +6709,7 @@
         <v>289</v>
       </c>
       <c r="C124" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D124" t="s">
         <v>37</v>
@@ -6738,7 +6732,7 @@
         <v>290</v>
       </c>
       <c r="C125" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D125" t="s">
         <v>37</v>
@@ -6807,7 +6801,7 @@
         <v>293</v>
       </c>
       <c r="C128" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D128" t="s">
         <v>37</v>
@@ -6853,7 +6847,7 @@
         <v>295</v>
       </c>
       <c r="C130" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D130" t="s">
         <v>37</v>
@@ -6968,7 +6962,7 @@
         <v>304</v>
       </c>
       <c r="C135" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D135" t="s">
         <v>305</v>
@@ -7175,7 +7169,7 @@
         <v>321</v>
       </c>
       <c r="C144" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D144" t="s">
         <v>322</v>
@@ -8279,7 +8273,7 @@
         <v>429</v>
       </c>
       <c r="C192" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D192" t="s">
         <v>427</v>
@@ -8486,7 +8480,7 @@
         <v>446</v>
       </c>
       <c r="C201" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D201" t="s">
         <v>447</v>
@@ -8601,7 +8595,7 @@
         <v>461</v>
       </c>
       <c r="C206" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D206" t="s">
         <v>462</v>
@@ -8624,7 +8618,7 @@
         <v>464</v>
       </c>
       <c r="C207" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D207" t="s">
         <v>462</v>
@@ -8647,7 +8641,7 @@
         <v>465</v>
       </c>
       <c r="C208" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D208" t="s">
         <v>462</v>
@@ -9475,7 +9469,7 @@
         <v>535</v>
       </c>
       <c r="C244" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D244" t="s">
         <v>536</v>
@@ -10694,7 +10688,7 @@
         <v>642</v>
       </c>
       <c r="C297" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D297" t="s">
         <v>462</v>
@@ -10970,7 +10964,7 @@
         <v>662</v>
       </c>
       <c r="C309" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D309" t="s">
         <v>37</v>
@@ -11039,7 +11033,7 @@
         <v>665</v>
       </c>
       <c r="C312" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D312" t="s">
         <v>37</v>
@@ -11982,7 +11976,7 @@
         <v>738</v>
       </c>
       <c r="C353" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D353" t="s">
         <v>322</v>
@@ -12051,7 +12045,7 @@
         <v>745</v>
       </c>
       <c r="C356" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D356" t="s">
         <v>746</v>
@@ -12235,7 +12229,7 @@
         <v>759</v>
       </c>
       <c r="C364" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D364" t="s">
         <v>760</v>
@@ -12373,7 +12367,7 @@
         <v>769</v>
       </c>
       <c r="C370" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D370" t="s">
         <v>770</v>
@@ -12396,7 +12390,7 @@
         <v>772</v>
       </c>
       <c r="C371" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D371" t="s">
         <v>773</v>
@@ -12419,7 +12413,7 @@
         <v>775</v>
       </c>
       <c r="C372" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D372" t="s">
         <v>773</v>
@@ -12488,7 +12482,7 @@
         <v>780</v>
       </c>
       <c r="C375" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D375" t="s">
         <v>322</v>
@@ -12511,7 +12505,7 @@
         <v>781</v>
       </c>
       <c r="C376" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D376" t="s">
         <v>782</v>
@@ -12603,7 +12597,7 @@
         <v>789</v>
       </c>
       <c r="C380" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D380" t="s">
         <v>254</v>
@@ -12718,7 +12712,7 @@
         <v>800</v>
       </c>
       <c r="C385" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D385" t="s">
         <v>68</v>
@@ -12741,7 +12735,7 @@
         <v>801</v>
       </c>
       <c r="C386" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D386" t="s">
         <v>19</v>
@@ -13247,7 +13241,7 @@
         <v>829</v>
       </c>
       <c r="C408" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D408" t="s">
         <v>81</v>
@@ -13316,7 +13310,7 @@
         <v>832</v>
       </c>
       <c r="C411" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D411" t="s">
         <v>37</v>
@@ -13546,7 +13540,7 @@
         <v>848</v>
       </c>
       <c r="C421" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D421" t="s">
         <v>7</v>
@@ -13845,7 +13839,7 @@
         <v>867</v>
       </c>
       <c r="C434" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D434" t="s">
         <v>19</v>
@@ -13914,7 +13908,7 @@
         <v>870</v>
       </c>
       <c r="C437" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D437" t="s">
         <v>68</v>
@@ -14052,7 +14046,7 @@
         <v>884</v>
       </c>
       <c r="C443" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D443" t="s">
         <v>885</v>
@@ -14075,7 +14069,7 @@
         <v>887</v>
       </c>
       <c r="C444" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D444" t="s">
         <v>885</v>
@@ -14121,7 +14115,7 @@
         <v>891</v>
       </c>
       <c r="C446" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D446" t="s">
         <v>140</v>
@@ -16493,13 +16487,13 @@
         <v>80</v>
       </c>
       <c r="D549" t="s">
-        <v>322</v>
+        <v>41</v>
       </c>
       <c r="E549" t="s">
-        <v>323</v>
+        <v>42</v>
       </c>
       <c r="F549" s="1">
-        <v>46284</v>
+        <v>46289</v>
       </c>
       <c r="G549" s="1">
         <v>46296</v>
@@ -16516,16 +16510,16 @@
         <v>80</v>
       </c>
       <c r="D550" t="s">
-        <v>41</v>
+        <v>657</v>
       </c>
       <c r="E550" t="s">
-        <v>42</v>
+        <v>658</v>
       </c>
       <c r="F550" s="1">
-        <v>46289</v>
+        <v>46294</v>
       </c>
       <c r="G550" s="1">
-        <v>46296</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="551" spans="1:7" x14ac:dyDescent="0.2">
@@ -16539,16 +16533,16 @@
         <v>80</v>
       </c>
       <c r="D551" t="s">
-        <v>276</v>
+        <v>1055</v>
       </c>
       <c r="E551" t="s">
-        <v>277</v>
+        <v>1056</v>
       </c>
       <c r="F551" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="G551" s="1">
-        <v>46296</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="552" spans="1:7" x14ac:dyDescent="0.2">
@@ -16562,16 +16556,16 @@
         <v>80</v>
       </c>
       <c r="D552" t="s">
-        <v>657</v>
+        <v>133</v>
       </c>
       <c r="E552" t="s">
-        <v>658</v>
+        <v>134</v>
       </c>
       <c r="F552" s="1">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="G552" s="1">
-        <v>46294</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="553" spans="1:7" x14ac:dyDescent="0.2">
@@ -16591,10 +16585,10 @@
         <v>1056</v>
       </c>
       <c r="F553" s="1">
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="G553" s="1">
-        <v>46295</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="554" spans="1:7" x14ac:dyDescent="0.2">
@@ -16608,10 +16602,10 @@
         <v>80</v>
       </c>
       <c r="D554" t="s">
-        <v>133</v>
+        <v>1045</v>
       </c>
       <c r="E554" t="s">
-        <v>134</v>
+        <v>1046</v>
       </c>
       <c r="F554" s="1">
         <v>46297</v>
@@ -16622,82 +16616,82 @@
     </row>
     <row r="555" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A555" t="s">
-        <v>1050</v>
+        <v>1074</v>
       </c>
       <c r="B555" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="C555" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D555" t="s">
-        <v>1055</v>
+        <v>1076</v>
       </c>
       <c r="E555" t="s">
-        <v>1056</v>
+        <v>1077</v>
       </c>
       <c r="F555" s="1">
-        <v>46297</v>
+        <v>46063</v>
       </c>
       <c r="G555" s="1">
-        <v>46297</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="556" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A556" t="s">
-        <v>1050</v>
+        <v>1074</v>
       </c>
       <c r="B556" t="s">
-        <v>1075</v>
+        <v>1078</v>
       </c>
       <c r="C556" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D556" t="s">
-        <v>1045</v>
+        <v>57</v>
       </c>
       <c r="E556" t="s">
-        <v>1046</v>
+        <v>58</v>
       </c>
       <c r="F556" s="1">
-        <v>46297</v>
+        <v>46113</v>
       </c>
       <c r="G556" s="1">
-        <v>46297</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="557" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A557" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B557" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="C557" t="s">
-        <v>96</v>
+        <v>2</v>
       </c>
       <c r="D557" t="s">
-        <v>1078</v>
+        <v>57</v>
       </c>
       <c r="E557" t="s">
-        <v>1079</v>
+        <v>58</v>
       </c>
       <c r="F557" s="1">
-        <v>46063</v>
+        <v>46125</v>
       </c>
       <c r="G557" s="1">
-        <v>46064</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="558" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A558" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B558" t="s">
         <v>1080</v>
       </c>
       <c r="C558" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D558" t="s">
         <v>57</v>
@@ -16706,15 +16700,15 @@
         <v>58</v>
       </c>
       <c r="F558" s="1">
-        <v>46113</v>
+        <v>46126</v>
       </c>
       <c r="G558" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="559" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A559" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B559" t="s">
         <v>1081</v>
@@ -16729,15 +16723,15 @@
         <v>58</v>
       </c>
       <c r="F559" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="G559" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="560" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A560" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B560" t="s">
         <v>1082</v>
@@ -16752,21 +16746,21 @@
         <v>58</v>
       </c>
       <c r="F560" s="1">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="G560" s="1">
-        <v>46126</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="561" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A561" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B561" t="s">
         <v>1083</v>
       </c>
       <c r="C561" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D561" t="s">
         <v>57</v>
@@ -16775,15 +16769,15 @@
         <v>58</v>
       </c>
       <c r="F561" s="1">
-        <v>46126</v>
+        <v>46132</v>
       </c>
       <c r="G561" s="1">
-        <v>46126</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="562" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A562" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B562" t="s">
         <v>1084</v>
@@ -16798,21 +16792,21 @@
         <v>58</v>
       </c>
       <c r="F562" s="1">
-        <v>46128</v>
+        <v>46161</v>
       </c>
       <c r="G562" s="1">
-        <v>46128</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="563" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A563" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B563" t="s">
         <v>1085</v>
       </c>
       <c r="C563" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D563" t="s">
         <v>57</v>
@@ -16821,15 +16815,15 @@
         <v>58</v>
       </c>
       <c r="F563" s="1">
-        <v>46132</v>
+        <v>46174</v>
       </c>
       <c r="G563" s="1">
-        <v>46132</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="564" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A564" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B564" t="s">
         <v>1086</v>
@@ -16844,21 +16838,21 @@
         <v>58</v>
       </c>
       <c r="F564" s="1">
-        <v>46161</v>
+        <v>46174</v>
       </c>
       <c r="G564" s="1">
-        <v>46161</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="565" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A565" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B565" t="s">
         <v>1087</v>
       </c>
       <c r="C565" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D565" t="s">
         <v>57</v>
@@ -16867,21 +16861,21 @@
         <v>58</v>
       </c>
       <c r="F565" s="1">
-        <v>46174</v>
+        <v>46195</v>
       </c>
       <c r="G565" s="1">
-        <v>46174</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="566" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A566" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B566" t="s">
         <v>1088</v>
       </c>
       <c r="C566" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D566" t="s">
         <v>57</v>
@@ -16890,21 +16884,21 @@
         <v>58</v>
       </c>
       <c r="F566" s="1">
-        <v>46174</v>
+        <v>46210</v>
       </c>
       <c r="G566" s="1">
-        <v>46174</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="567" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A567" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B567" t="s">
         <v>1089</v>
       </c>
       <c r="C567" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D567" t="s">
         <v>57</v>
@@ -16913,15 +16907,15 @@
         <v>58</v>
       </c>
       <c r="F567" s="1">
-        <v>46195</v>
+        <v>46213</v>
       </c>
       <c r="G567" s="1">
-        <v>46252</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="568" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A568" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B568" t="s">
         <v>1090</v>
@@ -16936,44 +16930,44 @@
         <v>58</v>
       </c>
       <c r="F568" s="1">
-        <v>46210</v>
+        <v>46218</v>
       </c>
       <c r="G568" s="1">
-        <v>46210</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="569" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A569" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B569" t="s">
         <v>1091</v>
       </c>
       <c r="C569" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D569" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="E569" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="F569" s="1">
-        <v>46213</v>
+        <v>46226</v>
       </c>
       <c r="G569" s="1">
-        <v>46213</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="570" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A570" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B570" t="s">
         <v>1092</v>
       </c>
       <c r="C570" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D570" t="s">
         <v>57</v>
@@ -16982,7 +16976,7 @@
         <v>58</v>
       </c>
       <c r="F570" s="1">
-        <v>46218</v>
+        <v>46227</v>
       </c>
       <c r="G570" s="1">
         <v>46252</v>
@@ -16990,7 +16984,7 @@
     </row>
     <row r="571" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A571" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B571" t="s">
         <v>1093</v>
@@ -16999,27 +16993,27 @@
         <v>6</v>
       </c>
       <c r="D571" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="E571" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="F571" s="1">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="G571" s="1">
-        <v>46226</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="572" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A572" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B572" t="s">
         <v>1094</v>
       </c>
       <c r="C572" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D572" t="s">
         <v>57</v>
@@ -17031,12 +17025,12 @@
         <v>46227</v>
       </c>
       <c r="G572" s="1">
-        <v>46252</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="573" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A573" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B573" t="s">
         <v>1095</v>
@@ -17045,13 +17039,13 @@
         <v>6</v>
       </c>
       <c r="D573" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="E573" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="F573" s="1">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="G573" s="1">
         <v>46252</v>
@@ -17059,7 +17053,7 @@
     </row>
     <row r="574" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A574" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B574" t="s">
         <v>1096</v>
@@ -17074,15 +17068,15 @@
         <v>58</v>
       </c>
       <c r="F574" s="1">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="G574" s="1">
-        <v>46228</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="575" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A575" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B575" t="s">
         <v>1097</v>
@@ -17091,27 +17085,27 @@
         <v>6</v>
       </c>
       <c r="D575" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="E575" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="F575" s="1">
-        <v>46230</v>
+        <v>46254</v>
       </c>
       <c r="G575" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="576" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A576" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B576" t="s">
         <v>1098</v>
       </c>
       <c r="C576" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D576" t="s">
         <v>57</v>
@@ -17120,15 +17114,15 @@
         <v>58</v>
       </c>
       <c r="F576" s="1">
-        <v>46231</v>
+        <v>46255</v>
       </c>
       <c r="G576" s="1">
-        <v>46231</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="577" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A577" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B577" t="s">
         <v>1099</v>
@@ -17143,21 +17137,21 @@
         <v>58</v>
       </c>
       <c r="F577" s="1">
-        <v>46254</v>
+        <v>46260</v>
       </c>
       <c r="G577" s="1">
-        <v>46254</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="578" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A578" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B578" t="s">
         <v>1100</v>
       </c>
       <c r="C578" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D578" t="s">
         <v>57</v>
@@ -17166,15 +17160,15 @@
         <v>58</v>
       </c>
       <c r="F578" s="1">
-        <v>46255</v>
+        <v>46289</v>
       </c>
       <c r="G578" s="1">
-        <v>46255</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="579" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A579" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B579" t="s">
         <v>1101</v>
@@ -17189,21 +17183,21 @@
         <v>58</v>
       </c>
       <c r="F579" s="1">
-        <v>46260</v>
+        <v>46294</v>
       </c>
       <c r="G579" s="1">
-        <v>46260</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="580" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A580" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B580" t="s">
         <v>1102</v>
       </c>
       <c r="C580" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D580" t="s">
         <v>57</v>
@@ -17212,21 +17206,21 @@
         <v>58</v>
       </c>
       <c r="F580" s="1">
-        <v>46289</v>
+        <v>46297</v>
       </c>
       <c r="G580" s="1">
-        <v>46289</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="581" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A581" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B581" t="s">
         <v>1103</v>
       </c>
       <c r="C581" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D581" t="s">
         <v>57</v>
@@ -17235,15 +17229,15 @@
         <v>58</v>
       </c>
       <c r="F581" s="1">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="G581" s="1">
-        <v>46294</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="582" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A582" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B582" t="s">
         <v>1104</v>
@@ -17266,7 +17260,7 @@
     </row>
     <row r="583" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A583" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B583" t="s">
         <v>1105</v>
@@ -17289,99 +17283,99 @@
     </row>
     <row r="584" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A584" t="s">
-        <v>1076</v>
+        <v>1106</v>
       </c>
       <c r="B584" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="C584" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D584" t="s">
-        <v>57</v>
+        <v>1108</v>
       </c>
       <c r="E584" t="s">
-        <v>58</v>
+        <v>1109</v>
       </c>
       <c r="F584" s="1">
-        <v>46297</v>
+        <v>46157</v>
       </c>
       <c r="G584" s="1">
-        <v>46297</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="585" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A585" t="s">
-        <v>1076</v>
+        <v>1106</v>
       </c>
       <c r="B585" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="C585" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D585" t="s">
-        <v>57</v>
+        <v>1111</v>
       </c>
       <c r="E585" t="s">
-        <v>58</v>
+        <v>1112</v>
       </c>
       <c r="F585" s="1">
-        <v>46297</v>
+        <v>46168</v>
       </c>
       <c r="G585" s="1">
-        <v>46297</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="586" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A586" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B586" t="s">
-        <v>1109</v>
+        <v>1113</v>
       </c>
       <c r="C586" t="s">
         <v>2</v>
       </c>
       <c r="D586" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="E586" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="F586" s="1">
-        <v>46157</v>
+        <v>46218</v>
       </c>
       <c r="G586" s="1">
-        <v>46157</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="587" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A587" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B587" t="s">
-        <v>1112</v>
+        <v>1114</v>
       </c>
       <c r="C587" t="s">
         <v>2</v>
       </c>
       <c r="D587" t="s">
-        <v>1113</v>
+        <v>1108</v>
       </c>
       <c r="E587" t="s">
-        <v>1114</v>
+        <v>1109</v>
       </c>
       <c r="F587" s="1">
-        <v>46168</v>
+        <v>46244</v>
       </c>
       <c r="G587" s="1">
-        <v>46170</v>
+        <v>46244</v>
       </c>
     </row>
     <row r="588" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A588" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B588" t="s">
         <v>1115</v>
@@ -17390,21 +17384,21 @@
         <v>2</v>
       </c>
       <c r="D588" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="E588" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="F588" s="1">
-        <v>46218</v>
+        <v>46247</v>
       </c>
       <c r="G588" s="1">
-        <v>46218</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="589" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A589" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B589" t="s">
         <v>1116</v>
@@ -17413,67 +17407,67 @@
         <v>2</v>
       </c>
       <c r="D589" t="s">
-        <v>1110</v>
+        <v>1117</v>
       </c>
       <c r="E589" t="s">
-        <v>1111</v>
+        <v>1118</v>
       </c>
       <c r="F589" s="1">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="G589" s="1">
-        <v>46244</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="590" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A590" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B590" t="s">
-        <v>1117</v>
+        <v>1119</v>
       </c>
       <c r="C590" t="s">
         <v>2</v>
       </c>
       <c r="D590" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="E590" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="F590" s="1">
-        <v>46247</v>
+        <v>46255</v>
       </c>
       <c r="G590" s="1">
-        <v>46247</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="591" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A591" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B591" t="s">
-        <v>1118</v>
+        <v>1120</v>
       </c>
       <c r="C591" t="s">
         <v>2</v>
       </c>
       <c r="D591" t="s">
-        <v>1119</v>
+        <v>1108</v>
       </c>
       <c r="E591" t="s">
-        <v>1120</v>
+        <v>1109</v>
       </c>
       <c r="F591" s="1">
-        <v>46247</v>
+        <v>46258</v>
       </c>
       <c r="G591" s="1">
-        <v>46247</v>
+        <v>46258</v>
       </c>
     </row>
     <row r="592" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A592" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B592" t="s">
         <v>1121</v>
@@ -17482,107 +17476,61 @@
         <v>2</v>
       </c>
       <c r="D592" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="E592" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="F592" s="1">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="G592" s="1">
-        <v>46255</v>
+        <v>46265</v>
       </c>
     </row>
     <row r="593" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A593" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B593" t="s">
         <v>1122</v>
       </c>
       <c r="C593" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D593" t="s">
-        <v>1110</v>
+        <v>13</v>
       </c>
       <c r="E593" t="s">
-        <v>1111</v>
+        <v>14</v>
       </c>
       <c r="F593" s="1">
-        <v>46258</v>
+        <v>46281</v>
       </c>
       <c r="G593" s="1">
-        <v>46258</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="594" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A594" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B594" t="s">
         <v>1123</v>
       </c>
       <c r="C594" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D594" t="s">
-        <v>1110</v>
+        <v>1124</v>
       </c>
       <c r="E594" t="s">
-        <v>1111</v>
+        <v>1125</v>
       </c>
       <c r="F594" s="1">
-        <v>46262</v>
+        <v>46296</v>
       </c>
       <c r="G594" s="1">
-        <v>46265</v>
-      </c>
-    </row>
-    <row r="595" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A595" t="s">
-        <v>1108</v>
-      </c>
-      <c r="B595" t="s">
-        <v>1124</v>
-      </c>
-      <c r="C595" t="s">
-        <v>6</v>
-      </c>
-      <c r="D595" t="s">
-        <v>13</v>
-      </c>
-      <c r="E595" t="s">
-        <v>14</v>
-      </c>
-      <c r="F595" s="1">
-        <v>46281</v>
-      </c>
-      <c r="G595" s="1">
-        <v>46283</v>
-      </c>
-    </row>
-    <row r="596" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A596" t="s">
-        <v>1108</v>
-      </c>
-      <c r="B596" t="s">
-        <v>1125</v>
-      </c>
-      <c r="C596" t="s">
-        <v>80</v>
-      </c>
-      <c r="D596" t="s">
-        <v>1126</v>
-      </c>
-      <c r="E596" t="s">
-        <v>1127</v>
-      </c>
-      <c r="F596" s="1">
-        <v>46296</v>
-      </c>
-      <c r="G596" s="1">
         <v>46296</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 07/10/2026 06:15:01
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E881DEAA-F71C-4D68-9FEB-739812AF0C6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3FA92BC2-AC2D-449D-803C-1DD22BD3DBFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89B1FA2D-B3E7-4A06-8837-ED1EBFC83EED}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{4A7C9FCC-8ACC-4C71-8143-3C4F66FF6395}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2958" uniqueCount="1117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2978" uniqueCount="1127">
   <si>
     <t>0001</t>
   </si>
@@ -3047,6 +3047,36 @@
   </si>
   <si>
     <t xml:space="preserve">  217107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217109</t>
+  </si>
+  <si>
+    <t>LN02</t>
+  </si>
+  <si>
+    <t>LA NORIA REVESIMIENTOS S.A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217110</t>
+  </si>
+  <si>
+    <t>AB08</t>
+  </si>
+  <si>
+    <t>ABELSON S.A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217111</t>
+  </si>
+  <si>
+    <t>GI09</t>
+  </si>
+  <si>
+    <t>GRUPO INNOVARE SRL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217112</t>
   </si>
   <si>
     <t>0004</t>
@@ -3820,34 +3850,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6827804E-F2A3-4D11-A68D-6506E0605E1F}">
-  <dimension ref="A1:H591"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3805E581-45E9-4BDB-9E62-FC6A01FC27C0}">
+  <dimension ref="A1:H595"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>1109</v>
+        <v>1119</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1110</v>
+        <v>1120</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1111</v>
+        <v>1121</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>1112</v>
+        <v>1122</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>1113</v>
+        <v>1123</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>1114</v>
+        <v>1124</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>1115</v>
+        <v>1125</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>1116</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -15613,7 +15643,7 @@
         <v>1</v>
       </c>
       <c r="D454" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="E454" t="s">
         <v>77</v>
@@ -17268,62 +17298,62 @@
     </row>
     <row r="518" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A518" t="s">
+        <v>0</v>
+      </c>
+      <c r="B518" t="s">
         <v>1009</v>
       </c>
-      <c r="B518" t="s">
+      <c r="C518">
+        <v>1</v>
+      </c>
+      <c r="D518" t="s">
+        <v>80</v>
+      </c>
+      <c r="E518" t="s">
         <v>1010</v>
       </c>
-      <c r="C518">
-        <v>1</v>
-      </c>
-      <c r="D518" t="s">
-        <v>2</v>
-      </c>
-      <c r="E518" t="s">
-        <v>200</v>
-      </c>
       <c r="F518" t="s">
-        <v>201</v>
+        <v>1011</v>
       </c>
       <c r="G518" s="1">
-        <v>46148</v>
+        <v>46301</v>
       </c>
       <c r="H518" s="1">
-        <v>46149</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="519" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A519" t="s">
-        <v>1009</v>
+        <v>0</v>
       </c>
       <c r="B519" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="C519">
         <v>1</v>
       </c>
       <c r="D519" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="E519" t="s">
-        <v>112</v>
+        <v>1013</v>
       </c>
       <c r="F519" t="s">
-        <v>113</v>
+        <v>1014</v>
       </c>
       <c r="G519" s="1">
-        <v>46268</v>
+        <v>46301</v>
       </c>
       <c r="H519" s="1">
-        <v>46268</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="520" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A520" t="s">
-        <v>1009</v>
+        <v>0</v>
       </c>
       <c r="B520" t="s">
-        <v>1012</v>
+        <v>1015</v>
       </c>
       <c r="C520">
         <v>1</v>
@@ -17332,10 +17362,10 @@
         <v>80</v>
       </c>
       <c r="E520" t="s">
-        <v>741</v>
+        <v>1016</v>
       </c>
       <c r="F520" t="s">
-        <v>742</v>
+        <v>1017</v>
       </c>
       <c r="G520" s="1">
         <v>46301</v>
@@ -17346,10 +17376,10 @@
     </row>
     <row r="521" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A521" t="s">
-        <v>1009</v>
+        <v>0</v>
       </c>
       <c r="B521" t="s">
-        <v>1013</v>
+        <v>1018</v>
       </c>
       <c r="C521">
         <v>1</v>
@@ -17358,10 +17388,10 @@
         <v>80</v>
       </c>
       <c r="E521" t="s">
-        <v>1014</v>
+        <v>1016</v>
       </c>
       <c r="F521" t="s">
-        <v>1015</v>
+        <v>1017</v>
       </c>
       <c r="G521" s="1">
         <v>46301</v>
@@ -17372,140 +17402,140 @@
     </row>
     <row r="522" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A522" t="s">
-        <v>1009</v>
+        <v>1019</v>
       </c>
       <c r="B522" t="s">
-        <v>1016</v>
+        <v>1020</v>
       </c>
       <c r="C522">
         <v>1</v>
       </c>
       <c r="D522" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="E522" t="s">
-        <v>741</v>
+        <v>200</v>
       </c>
       <c r="F522" t="s">
-        <v>742</v>
+        <v>201</v>
       </c>
       <c r="G522" s="1">
-        <v>46301</v>
+        <v>46148</v>
       </c>
       <c r="H522" s="1">
-        <v>46301</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="523" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A523" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
       <c r="B523" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="C523">
         <v>1</v>
       </c>
       <c r="D523" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E523" t="s">
-        <v>41</v>
+        <v>112</v>
       </c>
       <c r="F523" t="s">
-        <v>42</v>
+        <v>113</v>
       </c>
       <c r="G523" s="1">
-        <v>46133</v>
+        <v>46268</v>
       </c>
       <c r="H523" s="1">
-        <v>46134</v>
+        <v>46268</v>
       </c>
     </row>
     <row r="524" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A524" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
       <c r="B524" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C524">
         <v>1</v>
       </c>
       <c r="D524" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="E524" t="s">
-        <v>41</v>
+        <v>741</v>
       </c>
       <c r="F524" t="s">
-        <v>42</v>
+        <v>742</v>
       </c>
       <c r="G524" s="1">
-        <v>46134</v>
+        <v>46301</v>
       </c>
       <c r="H524" s="1">
-        <v>46134</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="525" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A525" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
       <c r="B525" t="s">
-        <v>1020</v>
+        <v>1023</v>
       </c>
       <c r="C525">
         <v>1</v>
       </c>
       <c r="D525" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="E525" t="s">
-        <v>19</v>
+        <v>1024</v>
       </c>
       <c r="F525" t="s">
-        <v>20</v>
+        <v>1025</v>
       </c>
       <c r="G525" s="1">
-        <v>46156</v>
+        <v>46301</v>
       </c>
       <c r="H525" s="1">
-        <v>46156</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="526" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A526" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
       <c r="B526" t="s">
-        <v>1021</v>
+        <v>1026</v>
       </c>
       <c r="C526">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D526" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="E526" t="s">
-        <v>1022</v>
+        <v>741</v>
       </c>
       <c r="F526" t="s">
-        <v>1023</v>
+        <v>742</v>
       </c>
       <c r="G526" s="1">
-        <v>46209</v>
+        <v>46301</v>
       </c>
       <c r="H526" s="1">
-        <v>46218</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="527" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A527" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B527" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C527">
         <v>1</v>
@@ -17514,47 +17544,47 @@
         <v>6</v>
       </c>
       <c r="E527" t="s">
-        <v>1025</v>
+        <v>41</v>
       </c>
       <c r="F527" t="s">
-        <v>1026</v>
+        <v>42</v>
       </c>
       <c r="G527" s="1">
-        <v>46213</v>
+        <v>46133</v>
       </c>
       <c r="H527" s="1">
-        <v>46213</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="528" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A528" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B528" t="s">
-        <v>1027</v>
+        <v>1029</v>
       </c>
       <c r="C528">
         <v>1</v>
       </c>
       <c r="D528" t="s">
-        <v>96</v>
+        <v>6</v>
       </c>
       <c r="E528" t="s">
-        <v>1028</v>
+        <v>41</v>
       </c>
       <c r="F528" t="s">
-        <v>1029</v>
+        <v>42</v>
       </c>
       <c r="G528" s="1">
-        <v>46213</v>
+        <v>46134</v>
       </c>
       <c r="H528" s="1">
-        <v>46216</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="529" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A529" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B529" t="s">
         <v>1030</v>
@@ -17563,33 +17593,33 @@
         <v>1</v>
       </c>
       <c r="D529" t="s">
-        <v>96</v>
+        <v>6</v>
       </c>
       <c r="E529" t="s">
-        <v>1028</v>
+        <v>19</v>
       </c>
       <c r="F529" t="s">
-        <v>1029</v>
+        <v>20</v>
       </c>
       <c r="G529" s="1">
-        <v>46224</v>
+        <v>46156</v>
       </c>
       <c r="H529" s="1">
-        <v>46224</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="530" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A530" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B530" t="s">
         <v>1031</v>
       </c>
       <c r="C530">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D530" t="s">
-        <v>6</v>
+        <v>96</v>
       </c>
       <c r="E530" t="s">
         <v>1032</v>
@@ -17598,15 +17628,15 @@
         <v>1033</v>
       </c>
       <c r="G530" s="1">
-        <v>46253</v>
+        <v>46209</v>
       </c>
       <c r="H530" s="1">
-        <v>46253</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="531" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A531" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B531" t="s">
         <v>1034</v>
@@ -17615,157 +17645,157 @@
         <v>1</v>
       </c>
       <c r="D531" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E531" t="s">
-        <v>211</v>
+        <v>1035</v>
       </c>
       <c r="F531" t="s">
-        <v>212</v>
+        <v>1036</v>
       </c>
       <c r="G531" s="1">
-        <v>46273</v>
+        <v>46213</v>
       </c>
       <c r="H531" s="1">
-        <v>46274</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="532" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A532" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B532" t="s">
-        <v>1035</v>
+        <v>1037</v>
       </c>
       <c r="C532">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D532" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="E532" t="s">
-        <v>41</v>
+        <v>1038</v>
       </c>
       <c r="F532" t="s">
-        <v>42</v>
+        <v>1039</v>
       </c>
       <c r="G532" s="1">
-        <v>46289</v>
+        <v>46213</v>
       </c>
       <c r="H532" s="1">
-        <v>46296</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="533" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A533" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B533" t="s">
-        <v>1036</v>
+        <v>1040</v>
       </c>
       <c r="C533">
         <v>1</v>
       </c>
       <c r="D533" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="E533" t="s">
-        <v>1022</v>
+        <v>1038</v>
       </c>
       <c r="F533" t="s">
-        <v>1023</v>
+        <v>1039</v>
       </c>
       <c r="G533" s="1">
-        <v>46295</v>
+        <v>46224</v>
       </c>
       <c r="H533" s="1">
-        <v>46295</v>
+        <v>46224</v>
       </c>
     </row>
     <row r="534" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A534" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B534" t="s">
-        <v>1037</v>
+        <v>1041</v>
       </c>
       <c r="C534">
         <v>1</v>
       </c>
       <c r="D534" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="E534" t="s">
-        <v>1038</v>
+        <v>1042</v>
       </c>
       <c r="F534" t="s">
-        <v>1039</v>
+        <v>1043</v>
       </c>
       <c r="G534" s="1">
-        <v>46295</v>
+        <v>46253</v>
       </c>
       <c r="H534" s="1">
-        <v>46301</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="535" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A535" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B535" t="s">
-        <v>1040</v>
+        <v>1044</v>
       </c>
       <c r="C535">
         <v>1</v>
       </c>
       <c r="D535" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="E535" t="s">
-        <v>1022</v>
+        <v>211</v>
       </c>
       <c r="F535" t="s">
-        <v>1023</v>
+        <v>212</v>
       </c>
       <c r="G535" s="1">
-        <v>46297</v>
+        <v>46273</v>
       </c>
       <c r="H535" s="1">
-        <v>46297</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="536" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A536" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B536" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
       <c r="C536">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D536" t="s">
         <v>80</v>
       </c>
       <c r="E536" t="s">
-        <v>710</v>
+        <v>41</v>
       </c>
       <c r="F536" t="s">
-        <v>711</v>
+        <v>42</v>
       </c>
       <c r="G536" s="1">
-        <v>46297</v>
+        <v>46289</v>
       </c>
       <c r="H536" s="1">
-        <v>46297</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="537" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A537" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B537" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
       <c r="C537">
         <v>1</v>
@@ -17774,24 +17804,24 @@
         <v>80</v>
       </c>
       <c r="E537" t="s">
-        <v>461</v>
+        <v>1032</v>
       </c>
       <c r="F537" t="s">
-        <v>462</v>
+        <v>1033</v>
       </c>
       <c r="G537" s="1">
-        <v>46297</v>
+        <v>46295</v>
       </c>
       <c r="H537" s="1">
-        <v>46300</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="538" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A538" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B538" t="s">
-        <v>1043</v>
+        <v>1047</v>
       </c>
       <c r="C538">
         <v>1</v>
@@ -17800,24 +17830,24 @@
         <v>80</v>
       </c>
       <c r="E538" t="s">
-        <v>744</v>
+        <v>1048</v>
       </c>
       <c r="F538" t="s">
-        <v>745</v>
+        <v>1049</v>
       </c>
       <c r="G538" s="1">
-        <v>46300</v>
+        <v>46295</v>
       </c>
       <c r="H538" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="539" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A539" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B539" t="s">
-        <v>1044</v>
+        <v>1050</v>
       </c>
       <c r="C539">
         <v>1</v>
@@ -17826,24 +17856,24 @@
         <v>80</v>
       </c>
       <c r="E539" t="s">
-        <v>1045</v>
+        <v>1032</v>
       </c>
       <c r="F539" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
       <c r="G539" s="1">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="H539" s="1">
-        <v>46300</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="540" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A540" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B540" t="s">
-        <v>1047</v>
+        <v>1051</v>
       </c>
       <c r="C540">
         <v>1</v>
@@ -17852,24 +17882,24 @@
         <v>80</v>
       </c>
       <c r="E540" t="s">
-        <v>1045</v>
+        <v>710</v>
       </c>
       <c r="F540" t="s">
-        <v>1046</v>
+        <v>711</v>
       </c>
       <c r="G540" s="1">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="H540" s="1">
-        <v>46300</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="541" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A541" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B541" t="s">
-        <v>1048</v>
+        <v>1052</v>
       </c>
       <c r="C541">
         <v>1</v>
@@ -17878,13 +17908,13 @@
         <v>80</v>
       </c>
       <c r="E541" t="s">
-        <v>1022</v>
+        <v>461</v>
       </c>
       <c r="F541" t="s">
-        <v>1023</v>
+        <v>462</v>
       </c>
       <c r="G541" s="1">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="H541" s="1">
         <v>46300</v>
@@ -17892,22 +17922,22 @@
     </row>
     <row r="542" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A542" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B542" t="s">
-        <v>1049</v>
+        <v>1053</v>
       </c>
       <c r="C542">
         <v>1</v>
       </c>
       <c r="D542" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="E542" t="s">
-        <v>221</v>
+        <v>744</v>
       </c>
       <c r="F542" t="s">
-        <v>222</v>
+        <v>745</v>
       </c>
       <c r="G542" s="1">
         <v>46300</v>
@@ -17918,10 +17948,10 @@
     </row>
     <row r="543" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A543" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B543" t="s">
-        <v>1050</v>
+        <v>1054</v>
       </c>
       <c r="C543">
         <v>1</v>
@@ -17930,10 +17960,10 @@
         <v>80</v>
       </c>
       <c r="E543" t="s">
-        <v>221</v>
+        <v>1055</v>
       </c>
       <c r="F543" t="s">
-        <v>222</v>
+        <v>1056</v>
       </c>
       <c r="G543" s="1">
         <v>46300</v>
@@ -17944,10 +17974,10 @@
     </row>
     <row r="544" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A544" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B544" t="s">
-        <v>1051</v>
+        <v>1057</v>
       </c>
       <c r="C544">
         <v>1</v>
@@ -17956,24 +17986,24 @@
         <v>80</v>
       </c>
       <c r="E544" t="s">
-        <v>1028</v>
+        <v>1055</v>
       </c>
       <c r="F544" t="s">
-        <v>1029</v>
+        <v>1056</v>
       </c>
       <c r="G544" s="1">
         <v>46300</v>
       </c>
       <c r="H544" s="1">
-        <v>46301</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="545" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A545" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B545" t="s">
-        <v>1052</v>
+        <v>1058</v>
       </c>
       <c r="C545">
         <v>1</v>
@@ -17982,10 +18012,10 @@
         <v>80</v>
       </c>
       <c r="E545" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="F545" t="s">
-        <v>1029</v>
+        <v>1033</v>
       </c>
       <c r="G545" s="1">
         <v>46300</v>
@@ -17996,22 +18026,22 @@
     </row>
     <row r="546" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A546" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B546" t="s">
-        <v>1053</v>
+        <v>1059</v>
       </c>
       <c r="C546">
         <v>1</v>
       </c>
       <c r="D546" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="E546" t="s">
-        <v>1028</v>
+        <v>221</v>
       </c>
       <c r="F546" t="s">
-        <v>1029</v>
+        <v>222</v>
       </c>
       <c r="G546" s="1">
         <v>46300</v>
@@ -18022,10 +18052,10 @@
     </row>
     <row r="547" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A547" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B547" t="s">
-        <v>1054</v>
+        <v>1060</v>
       </c>
       <c r="C547">
         <v>1</v>
@@ -18034,24 +18064,24 @@
         <v>80</v>
       </c>
       <c r="E547" t="s">
-        <v>744</v>
+        <v>221</v>
       </c>
       <c r="F547" t="s">
-        <v>745</v>
+        <v>222</v>
       </c>
       <c r="G547" s="1">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="H547" s="1">
-        <v>46301</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="548" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A548" t="s">
-        <v>1017</v>
+        <v>1027</v>
       </c>
       <c r="B548" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="C548">
         <v>1</v>
@@ -18060,13 +18090,13 @@
         <v>80</v>
       </c>
       <c r="E548" t="s">
-        <v>1045</v>
+        <v>1038</v>
       </c>
       <c r="F548" t="s">
-        <v>1046</v>
+        <v>1039</v>
       </c>
       <c r="G548" s="1">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="H548" s="1">
         <v>46301</v>
@@ -18074,146 +18104,146 @@
     </row>
     <row r="549" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A549" t="s">
-        <v>1056</v>
+        <v>1027</v>
       </c>
       <c r="B549" t="s">
-        <v>1057</v>
+        <v>1062</v>
       </c>
       <c r="C549">
         <v>1</v>
       </c>
       <c r="D549" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="E549" t="s">
-        <v>1058</v>
+        <v>1038</v>
       </c>
       <c r="F549" t="s">
-        <v>1059</v>
+        <v>1039</v>
       </c>
       <c r="G549" s="1">
-        <v>46063</v>
+        <v>46300</v>
       </c>
       <c r="H549" s="1">
-        <v>46064</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="550" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A550" t="s">
-        <v>1056</v>
+        <v>1027</v>
       </c>
       <c r="B550" t="s">
-        <v>1060</v>
+        <v>1063</v>
       </c>
       <c r="C550">
         <v>1</v>
       </c>
       <c r="D550" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="E550" t="s">
-        <v>57</v>
+        <v>1038</v>
       </c>
       <c r="F550" t="s">
-        <v>58</v>
+        <v>1039</v>
       </c>
       <c r="G550" s="1">
-        <v>46113</v>
+        <v>46300</v>
       </c>
       <c r="H550" s="1">
-        <v>46125</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="551" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A551" t="s">
-        <v>1056</v>
+        <v>1027</v>
       </c>
       <c r="B551" t="s">
-        <v>1061</v>
+        <v>1064</v>
       </c>
       <c r="C551">
         <v>1</v>
       </c>
       <c r="D551" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="E551" t="s">
-        <v>57</v>
+        <v>744</v>
       </c>
       <c r="F551" t="s">
-        <v>58</v>
+        <v>745</v>
       </c>
       <c r="G551" s="1">
-        <v>46125</v>
+        <v>46301</v>
       </c>
       <c r="H551" s="1">
-        <v>46125</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="552" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A552" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B552" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C552">
+        <v>1</v>
+      </c>
+      <c r="D552" t="s">
+        <v>80</v>
+      </c>
+      <c r="E552" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F552" t="s">
         <v>1056</v>
       </c>
-      <c r="B552" t="s">
-        <v>1062</v>
-      </c>
-      <c r="C552">
-        <v>1</v>
-      </c>
-      <c r="D552" t="s">
-        <v>2</v>
-      </c>
-      <c r="E552" t="s">
-        <v>57</v>
-      </c>
-      <c r="F552" t="s">
-        <v>58</v>
-      </c>
       <c r="G552" s="1">
-        <v>46126</v>
+        <v>46301</v>
       </c>
       <c r="H552" s="1">
-        <v>46126</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="553" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A553" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B553" t="s">
-        <v>1063</v>
+        <v>1067</v>
       </c>
       <c r="C553">
         <v>1</v>
       </c>
       <c r="D553" t="s">
-        <v>2</v>
+        <v>96</v>
       </c>
       <c r="E553" t="s">
-        <v>57</v>
+        <v>1068</v>
       </c>
       <c r="F553" t="s">
-        <v>58</v>
+        <v>1069</v>
       </c>
       <c r="G553" s="1">
-        <v>46126</v>
+        <v>46063</v>
       </c>
       <c r="H553" s="1">
-        <v>46126</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="554" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A554" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B554" t="s">
-        <v>1064</v>
+        <v>1070</v>
       </c>
       <c r="C554">
         <v>1</v>
       </c>
       <c r="D554" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E554" t="s">
         <v>57</v>
@@ -18222,24 +18252,24 @@
         <v>58</v>
       </c>
       <c r="G554" s="1">
-        <v>46128</v>
+        <v>46113</v>
       </c>
       <c r="H554" s="1">
-        <v>46128</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="555" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A555" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B555" t="s">
-        <v>1065</v>
+        <v>1071</v>
       </c>
       <c r="C555">
         <v>1</v>
       </c>
       <c r="D555" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E555" t="s">
         <v>57</v>
@@ -18248,18 +18278,18 @@
         <v>58</v>
       </c>
       <c r="G555" s="1">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="H555" s="1">
-        <v>46132</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="556" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A556" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B556" t="s">
-        <v>1066</v>
+        <v>1072</v>
       </c>
       <c r="C556">
         <v>1</v>
@@ -18274,18 +18304,18 @@
         <v>58</v>
       </c>
       <c r="G556" s="1">
-        <v>46161</v>
+        <v>46126</v>
       </c>
       <c r="H556" s="1">
-        <v>46161</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="557" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A557" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B557" t="s">
-        <v>1067</v>
+        <v>1073</v>
       </c>
       <c r="C557">
         <v>1</v>
@@ -18300,18 +18330,18 @@
         <v>58</v>
       </c>
       <c r="G557" s="1">
-        <v>46174</v>
+        <v>46126</v>
       </c>
       <c r="H557" s="1">
-        <v>46174</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="558" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A558" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B558" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="C558">
         <v>1</v>
@@ -18326,18 +18356,18 @@
         <v>58</v>
       </c>
       <c r="G558" s="1">
-        <v>46174</v>
+        <v>46128</v>
       </c>
       <c r="H558" s="1">
-        <v>46174</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="559" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A559" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B559" t="s">
-        <v>1069</v>
+        <v>1075</v>
       </c>
       <c r="C559">
         <v>1</v>
@@ -18352,24 +18382,24 @@
         <v>58</v>
       </c>
       <c r="G559" s="1">
-        <v>46195</v>
+        <v>46132</v>
       </c>
       <c r="H559" s="1">
-        <v>46252</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="560" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A560" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B560" t="s">
-        <v>1070</v>
+        <v>1076</v>
       </c>
       <c r="C560">
         <v>1</v>
       </c>
       <c r="D560" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E560" t="s">
         <v>57</v>
@@ -18378,18 +18408,18 @@
         <v>58</v>
       </c>
       <c r="G560" s="1">
-        <v>46210</v>
+        <v>46161</v>
       </c>
       <c r="H560" s="1">
-        <v>46210</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="561" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A561" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B561" t="s">
-        <v>1071</v>
+        <v>1077</v>
       </c>
       <c r="C561">
         <v>1</v>
@@ -18404,24 +18434,24 @@
         <v>58</v>
       </c>
       <c r="G561" s="1">
-        <v>46213</v>
+        <v>46174</v>
       </c>
       <c r="H561" s="1">
-        <v>46213</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="562" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A562" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B562" t="s">
-        <v>1072</v>
+        <v>1078</v>
       </c>
       <c r="C562">
         <v>1</v>
       </c>
       <c r="D562" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E562" t="s">
         <v>57</v>
@@ -18430,18 +18460,18 @@
         <v>58</v>
       </c>
       <c r="G562" s="1">
-        <v>46218</v>
+        <v>46174</v>
       </c>
       <c r="H562" s="1">
-        <v>46252</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="563" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A563" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B563" t="s">
-        <v>1073</v>
+        <v>1079</v>
       </c>
       <c r="C563">
         <v>1</v>
@@ -18450,30 +18480,30 @@
         <v>6</v>
       </c>
       <c r="E563" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="F563" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G563" s="1">
-        <v>46226</v>
+        <v>46195</v>
       </c>
       <c r="H563" s="1">
-        <v>46226</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="564" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A564" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B564" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="C564">
         <v>1</v>
       </c>
       <c r="D564" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="E564" t="s">
         <v>57</v>
@@ -18482,24 +18512,24 @@
         <v>58</v>
       </c>
       <c r="G564" s="1">
-        <v>46227</v>
+        <v>46210</v>
       </c>
       <c r="H564" s="1">
-        <v>46252</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="565" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A565" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B565" t="s">
-        <v>1075</v>
+        <v>1081</v>
       </c>
       <c r="C565">
         <v>1</v>
       </c>
       <c r="D565" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E565" t="s">
         <v>57</v>
@@ -18508,18 +18538,18 @@
         <v>58</v>
       </c>
       <c r="G565" s="1">
-        <v>46227</v>
+        <v>46213</v>
       </c>
       <c r="H565" s="1">
-        <v>46252</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="566" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A566" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B566" t="s">
-        <v>1076</v>
+        <v>1082</v>
       </c>
       <c r="C566">
         <v>1</v>
@@ -18534,18 +18564,18 @@
         <v>58</v>
       </c>
       <c r="G566" s="1">
-        <v>46227</v>
+        <v>46218</v>
       </c>
       <c r="H566" s="1">
-        <v>46228</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="567" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A567" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B567" t="s">
-        <v>1077</v>
+        <v>1083</v>
       </c>
       <c r="C567">
         <v>1</v>
@@ -18560,24 +18590,24 @@
         <v>78</v>
       </c>
       <c r="G567" s="1">
-        <v>46230</v>
+        <v>46226</v>
       </c>
       <c r="H567" s="1">
-        <v>46252</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="568" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A568" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B568" t="s">
-        <v>1078</v>
+        <v>1084</v>
       </c>
       <c r="C568">
         <v>1</v>
       </c>
       <c r="D568" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="E568" t="s">
         <v>57</v>
@@ -18586,18 +18616,18 @@
         <v>58</v>
       </c>
       <c r="G568" s="1">
-        <v>46231</v>
+        <v>46227</v>
       </c>
       <c r="H568" s="1">
-        <v>46231</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="569" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A569" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B569" t="s">
-        <v>1079</v>
+        <v>1085</v>
       </c>
       <c r="C569">
         <v>1</v>
@@ -18612,24 +18642,24 @@
         <v>58</v>
       </c>
       <c r="G569" s="1">
-        <v>46254</v>
+        <v>46227</v>
       </c>
       <c r="H569" s="1">
-        <v>46254</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="570" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A570" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B570" t="s">
-        <v>1080</v>
+        <v>1086</v>
       </c>
       <c r="C570">
         <v>1</v>
       </c>
       <c r="D570" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E570" t="s">
         <v>57</v>
@@ -18638,18 +18668,18 @@
         <v>58</v>
       </c>
       <c r="G570" s="1">
-        <v>46255</v>
+        <v>46227</v>
       </c>
       <c r="H570" s="1">
-        <v>46255</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="571" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A571" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B571" t="s">
-        <v>1081</v>
+        <v>1087</v>
       </c>
       <c r="C571">
         <v>1</v>
@@ -18658,24 +18688,24 @@
         <v>6</v>
       </c>
       <c r="E571" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="F571" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G571" s="1">
-        <v>46260</v>
+        <v>46230</v>
       </c>
       <c r="H571" s="1">
-        <v>46260</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="572" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A572" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B572" t="s">
-        <v>1082</v>
+        <v>1088</v>
       </c>
       <c r="C572">
         <v>1</v>
@@ -18690,18 +18720,18 @@
         <v>58</v>
       </c>
       <c r="G572" s="1">
-        <v>46289</v>
+        <v>46231</v>
       </c>
       <c r="H572" s="1">
-        <v>46289</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="573" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A573" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B573" t="s">
-        <v>1083</v>
+        <v>1089</v>
       </c>
       <c r="C573">
         <v>1</v>
@@ -18716,24 +18746,24 @@
         <v>58</v>
       </c>
       <c r="G573" s="1">
-        <v>46294</v>
+        <v>46254</v>
       </c>
       <c r="H573" s="1">
-        <v>46294</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="574" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A574" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B574" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="C574">
         <v>1</v>
       </c>
       <c r="D574" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="E574" t="s">
         <v>57</v>
@@ -18742,24 +18772,24 @@
         <v>58</v>
       </c>
       <c r="G574" s="1">
-        <v>46301</v>
+        <v>46255</v>
       </c>
       <c r="H574" s="1">
-        <v>46301</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="575" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A575" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B575" t="s">
-        <v>1085</v>
+        <v>1091</v>
       </c>
       <c r="C575">
         <v>1</v>
       </c>
       <c r="D575" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="E575" t="s">
         <v>57</v>
@@ -18768,24 +18798,24 @@
         <v>58</v>
       </c>
       <c r="G575" s="1">
-        <v>46301</v>
+        <v>46260</v>
       </c>
       <c r="H575" s="1">
-        <v>46301</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="576" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A576" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B576" t="s">
-        <v>1086</v>
+        <v>1092</v>
       </c>
       <c r="C576">
         <v>1</v>
       </c>
       <c r="D576" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="E576" t="s">
         <v>57</v>
@@ -18794,24 +18824,24 @@
         <v>58</v>
       </c>
       <c r="G576" s="1">
-        <v>46301</v>
+        <v>46289</v>
       </c>
       <c r="H576" s="1">
-        <v>46301</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="577" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A577" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B577" t="s">
-        <v>1087</v>
+        <v>1093</v>
       </c>
       <c r="C577">
         <v>1</v>
       </c>
       <c r="D577" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="E577" t="s">
         <v>57</v>
@@ -18820,18 +18850,18 @@
         <v>58</v>
       </c>
       <c r="G577" s="1">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="H577" s="1">
-        <v>46301</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="578" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A578" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B578" t="s">
-        <v>1088</v>
+        <v>1094</v>
       </c>
       <c r="C578">
         <v>1</v>
@@ -18854,10 +18884,10 @@
     </row>
     <row r="579" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A579" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B579" t="s">
-        <v>1089</v>
+        <v>1095</v>
       </c>
       <c r="C579">
         <v>1</v>
@@ -18880,10 +18910,10 @@
     </row>
     <row r="580" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A580" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B580" t="s">
-        <v>1090</v>
+        <v>1096</v>
       </c>
       <c r="C580">
         <v>1</v>
@@ -18906,10 +18936,10 @@
     </row>
     <row r="581" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A581" t="s">
-        <v>1056</v>
+        <v>1066</v>
       </c>
       <c r="B581" t="s">
-        <v>1091</v>
+        <v>1097</v>
       </c>
       <c r="C581">
         <v>1</v>
@@ -18932,114 +18962,114 @@
     </row>
     <row r="582" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A582" t="s">
-        <v>1092</v>
+        <v>1066</v>
       </c>
       <c r="B582" t="s">
-        <v>1093</v>
+        <v>1098</v>
       </c>
       <c r="C582">
         <v>1</v>
       </c>
       <c r="D582" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="E582" t="s">
-        <v>1094</v>
+        <v>57</v>
       </c>
       <c r="F582" t="s">
-        <v>1095</v>
+        <v>58</v>
       </c>
       <c r="G582" s="1">
-        <v>46157</v>
+        <v>46301</v>
       </c>
       <c r="H582" s="1">
-        <v>46157</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="583" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A583" t="s">
-        <v>1092</v>
+        <v>1066</v>
       </c>
       <c r="B583" t="s">
-        <v>1096</v>
+        <v>1099</v>
       </c>
       <c r="C583">
         <v>1</v>
       </c>
       <c r="D583" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="E583" t="s">
-        <v>1097</v>
+        <v>57</v>
       </c>
       <c r="F583" t="s">
-        <v>1098</v>
+        <v>58</v>
       </c>
       <c r="G583" s="1">
-        <v>46168</v>
+        <v>46301</v>
       </c>
       <c r="H583" s="1">
-        <v>46170</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="584" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A584" t="s">
-        <v>1092</v>
+        <v>1066</v>
       </c>
       <c r="B584" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="C584">
         <v>1</v>
       </c>
       <c r="D584" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="E584" t="s">
-        <v>1094</v>
+        <v>57</v>
       </c>
       <c r="F584" t="s">
-        <v>1095</v>
+        <v>58</v>
       </c>
       <c r="G584" s="1">
-        <v>46218</v>
+        <v>46301</v>
       </c>
       <c r="H584" s="1">
-        <v>46218</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="585" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A585" t="s">
-        <v>1092</v>
+        <v>1066</v>
       </c>
       <c r="B585" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="C585">
         <v>1</v>
       </c>
       <c r="D585" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="E585" t="s">
-        <v>1094</v>
+        <v>57</v>
       </c>
       <c r="F585" t="s">
-        <v>1095</v>
+        <v>58</v>
       </c>
       <c r="G585" s="1">
-        <v>46244</v>
+        <v>46301</v>
       </c>
       <c r="H585" s="1">
-        <v>46244</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="586" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A586" t="s">
-        <v>1092</v>
+        <v>1102</v>
       </c>
       <c r="B586" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
       <c r="C586">
         <v>1</v>
@@ -19048,24 +19078,24 @@
         <v>2</v>
       </c>
       <c r="E586" t="s">
-        <v>1094</v>
+        <v>1104</v>
       </c>
       <c r="F586" t="s">
-        <v>1095</v>
+        <v>1105</v>
       </c>
       <c r="G586" s="1">
-        <v>46247</v>
+        <v>46157</v>
       </c>
       <c r="H586" s="1">
-        <v>46247</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="587" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A587" t="s">
-        <v>1092</v>
+        <v>1102</v>
       </c>
       <c r="B587" t="s">
-        <v>1102</v>
+        <v>1106</v>
       </c>
       <c r="C587">
         <v>1</v>
@@ -19074,24 +19104,24 @@
         <v>2</v>
       </c>
       <c r="E587" t="s">
-        <v>1103</v>
+        <v>1107</v>
       </c>
       <c r="F587" t="s">
-        <v>1104</v>
+        <v>1108</v>
       </c>
       <c r="G587" s="1">
-        <v>46247</v>
+        <v>46168</v>
       </c>
       <c r="H587" s="1">
-        <v>46247</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="588" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A588" t="s">
-        <v>1092</v>
+        <v>1102</v>
       </c>
       <c r="B588" t="s">
-        <v>1105</v>
+        <v>1109</v>
       </c>
       <c r="C588">
         <v>1</v>
@@ -19100,24 +19130,24 @@
         <v>2</v>
       </c>
       <c r="E588" t="s">
-        <v>1094</v>
+        <v>1104</v>
       </c>
       <c r="F588" t="s">
-        <v>1095</v>
+        <v>1105</v>
       </c>
       <c r="G588" s="1">
-        <v>46255</v>
+        <v>46218</v>
       </c>
       <c r="H588" s="1">
-        <v>46255</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="589" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A589" t="s">
-        <v>1092</v>
+        <v>1102</v>
       </c>
       <c r="B589" t="s">
-        <v>1106</v>
+        <v>1110</v>
       </c>
       <c r="C589">
         <v>1</v>
@@ -19126,24 +19156,24 @@
         <v>2</v>
       </c>
       <c r="E589" t="s">
-        <v>1094</v>
+        <v>1104</v>
       </c>
       <c r="F589" t="s">
-        <v>1095</v>
+        <v>1105</v>
       </c>
       <c r="G589" s="1">
-        <v>46258</v>
+        <v>46244</v>
       </c>
       <c r="H589" s="1">
-        <v>46258</v>
+        <v>46244</v>
       </c>
     </row>
     <row r="590" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A590" t="s">
-        <v>1092</v>
+        <v>1102</v>
       </c>
       <c r="B590" t="s">
-        <v>1107</v>
+        <v>1111</v>
       </c>
       <c r="C590">
         <v>1</v>
@@ -19152,41 +19182,145 @@
         <v>2</v>
       </c>
       <c r="E590" t="s">
-        <v>1094</v>
+        <v>1104</v>
       </c>
       <c r="F590" t="s">
-        <v>1095</v>
+        <v>1105</v>
       </c>
       <c r="G590" s="1">
-        <v>46262</v>
+        <v>46247</v>
       </c>
       <c r="H590" s="1">
-        <v>46265</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="591" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A591" t="s">
-        <v>1092</v>
+        <v>1102</v>
       </c>
       <c r="B591" t="s">
-        <v>1108</v>
+        <v>1112</v>
       </c>
       <c r="C591">
         <v>1</v>
       </c>
       <c r="D591" t="s">
+        <v>2</v>
+      </c>
+      <c r="E591" t="s">
+        <v>1113</v>
+      </c>
+      <c r="F591" t="s">
+        <v>1114</v>
+      </c>
+      <c r="G591" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H591" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="592" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A592" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B592" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C592">
+        <v>1</v>
+      </c>
+      <c r="D592" t="s">
+        <v>2</v>
+      </c>
+      <c r="E592" t="s">
+        <v>1104</v>
+      </c>
+      <c r="F592" t="s">
+        <v>1105</v>
+      </c>
+      <c r="G592" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H592" s="1">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="593" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A593" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B593" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C593">
+        <v>1</v>
+      </c>
+      <c r="D593" t="s">
+        <v>2</v>
+      </c>
+      <c r="E593" t="s">
+        <v>1104</v>
+      </c>
+      <c r="F593" t="s">
+        <v>1105</v>
+      </c>
+      <c r="G593" s="1">
+        <v>46258</v>
+      </c>
+      <c r="H593" s="1">
+        <v>46258</v>
+      </c>
+    </row>
+    <row r="594" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A594" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B594" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C594">
+        <v>1</v>
+      </c>
+      <c r="D594" t="s">
+        <v>2</v>
+      </c>
+      <c r="E594" t="s">
+        <v>1104</v>
+      </c>
+      <c r="F594" t="s">
+        <v>1105</v>
+      </c>
+      <c r="G594" s="1">
+        <v>46262</v>
+      </c>
+      <c r="H594" s="1">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="595" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A595" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B595" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C595">
+        <v>1</v>
+      </c>
+      <c r="D595" t="s">
         <v>6</v>
       </c>
-      <c r="E591" t="s">
+      <c r="E595" t="s">
         <v>13</v>
       </c>
-      <c r="F591" t="s">
+      <c r="F595" t="s">
         <v>14</v>
       </c>
-      <c r="G591" s="1">
+      <c r="G595" s="1">
         <v>46281</v>
       </c>
-      <c r="H591" s="1">
+      <c r="H595" s="1">
         <v>46283</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 08/10/2026 05:57:01
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EAC9404-7A63-42B9-80ED-EA612F3D6A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AE01ED8-A4B1-4CC1-934F-86A74D524A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30930" yWindow="10005" windowWidth="15000" windowHeight="6195" xr2:uid="{C727072A-0D58-4435-95C8-6D57BFAA23E7}"/>
+    <workbookView xWindow="30930" yWindow="10005" windowWidth="15000" windowHeight="6195" xr2:uid="{CF312FA0-55D7-4249-8BA7-8CABA3C451E8}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2408" uniqueCount="943">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2493" uniqueCount="968">
   <si>
     <t>0001</t>
   </si>
@@ -2458,6 +2458,15 @@
     <t xml:space="preserve">  217150</t>
   </si>
   <si>
+    <t xml:space="preserve">  217151</t>
+  </si>
+  <si>
+    <t>SY05</t>
+  </si>
+  <si>
+    <t>SANITARIOS YRIGOYEN CABRERA S. R. L.</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217152</t>
   </si>
   <si>
@@ -2503,6 +2512,9 @@
     <t xml:space="preserve">  217161</t>
   </si>
   <si>
+    <t xml:space="preserve">  217162</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217163</t>
   </si>
   <si>
@@ -2530,6 +2542,15 @@
     <t xml:space="preserve">  217167</t>
   </si>
   <si>
+    <t xml:space="preserve">  217168</t>
+  </si>
+  <si>
+    <t>CM57</t>
+  </si>
+  <si>
+    <t>CELESIA MARIANO T-SANITARIOS LARRALDE 1724</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217169</t>
   </si>
   <si>
@@ -2540,6 +2561,60 @@
   </si>
   <si>
     <t xml:space="preserve">  217172</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217173</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217174</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217175</t>
+  </si>
+  <si>
+    <t>RP08</t>
+  </si>
+  <si>
+    <t>RUSSO PABLO D. -CASA SAN JUAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217176</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217177</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217178</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217179</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217180</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217181</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217182</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217183</t>
+  </si>
+  <si>
+    <t>VL05</t>
+  </si>
+  <si>
+    <t>VENTURA LEANDRO ARIEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217184</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217185</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217186</t>
   </si>
   <si>
     <t>0004</t>
@@ -3298,34 +3373,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F67BFF4B-4A03-4C70-B5CD-F4D4F6CABD57}">
-  <dimension ref="A1:H481"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0DB821C-4677-411C-A378-21B5CB267C5F}">
+  <dimension ref="A1:H498"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>935</v>
+        <v>960</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>936</v>
+        <v>961</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>937</v>
+        <v>962</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>938</v>
+        <v>963</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>939</v>
+        <v>964</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>940</v>
+        <v>965</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>941</v>
+        <v>966</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>942</v>
+        <v>967</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -13612,10 +13687,10 @@
         <v>154</v>
       </c>
       <c r="E397" t="s">
-        <v>761</v>
+        <v>819</v>
       </c>
       <c r="F397" t="s">
-        <v>762</v>
+        <v>820</v>
       </c>
       <c r="G397" s="1">
         <v>46302</v>
@@ -13629,7 +13704,7 @@
         <v>0</v>
       </c>
       <c r="B398" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
       <c r="C398">
         <v>1</v>
@@ -13638,10 +13713,10 @@
         <v>154</v>
       </c>
       <c r="E398" t="s">
-        <v>808</v>
+        <v>761</v>
       </c>
       <c r="F398" t="s">
-        <v>809</v>
+        <v>762</v>
       </c>
       <c r="G398" s="1">
         <v>46302</v>
@@ -13655,7 +13730,7 @@
         <v>0</v>
       </c>
       <c r="B399" t="s">
-        <v>820</v>
+        <v>822</v>
       </c>
       <c r="C399">
         <v>1</v>
@@ -13664,10 +13739,10 @@
         <v>154</v>
       </c>
       <c r="E399" t="s">
-        <v>821</v>
+        <v>808</v>
       </c>
       <c r="F399" t="s">
-        <v>822</v>
+        <v>809</v>
       </c>
       <c r="G399" s="1">
         <v>46302</v>
@@ -13690,10 +13765,10 @@
         <v>154</v>
       </c>
       <c r="E400" t="s">
-        <v>139</v>
+        <v>824</v>
       </c>
       <c r="F400" t="s">
-        <v>140</v>
+        <v>825</v>
       </c>
       <c r="G400" s="1">
         <v>46302</v>
@@ -13707,7 +13782,7 @@
         <v>0</v>
       </c>
       <c r="B401" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="C401">
         <v>1</v>
@@ -13733,7 +13808,7 @@
         <v>0</v>
       </c>
       <c r="B402" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="C402">
         <v>1</v>
@@ -13742,10 +13817,10 @@
         <v>154</v>
       </c>
       <c r="E402" t="s">
-        <v>48</v>
+        <v>139</v>
       </c>
       <c r="F402" t="s">
-        <v>49</v>
+        <v>140</v>
       </c>
       <c r="G402" s="1">
         <v>46302</v>
@@ -13759,7 +13834,7 @@
         <v>0</v>
       </c>
       <c r="B403" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="C403">
         <v>1</v>
@@ -13768,10 +13843,10 @@
         <v>154</v>
       </c>
       <c r="E403" t="s">
-        <v>139</v>
+        <v>48</v>
       </c>
       <c r="F403" t="s">
-        <v>140</v>
+        <v>49</v>
       </c>
       <c r="G403" s="1">
         <v>46302</v>
@@ -13785,7 +13860,7 @@
         <v>0</v>
       </c>
       <c r="B404" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="C404">
         <v>1</v>
@@ -13811,7 +13886,7 @@
         <v>0</v>
       </c>
       <c r="B405" t="s">
-        <v>828</v>
+        <v>830</v>
       </c>
       <c r="C405">
         <v>1</v>
@@ -13820,10 +13895,10 @@
         <v>154</v>
       </c>
       <c r="E405" t="s">
-        <v>829</v>
+        <v>748</v>
       </c>
       <c r="F405" t="s">
-        <v>830</v>
+        <v>749</v>
       </c>
       <c r="G405" s="1">
         <v>46302</v>
@@ -13846,10 +13921,10 @@
         <v>154</v>
       </c>
       <c r="E406" t="s">
-        <v>832</v>
+        <v>139</v>
       </c>
       <c r="F406" t="s">
-        <v>833</v>
+        <v>140</v>
       </c>
       <c r="G406" s="1">
         <v>46302</v>
@@ -13863,19 +13938,19 @@
         <v>0</v>
       </c>
       <c r="B407" t="s">
+        <v>832</v>
+      </c>
+      <c r="C407">
+        <v>1</v>
+      </c>
+      <c r="D407" t="s">
+        <v>154</v>
+      </c>
+      <c r="E407" t="s">
+        <v>833</v>
+      </c>
+      <c r="F407" t="s">
         <v>834</v>
-      </c>
-      <c r="C407">
-        <v>1</v>
-      </c>
-      <c r="D407" t="s">
-        <v>154</v>
-      </c>
-      <c r="E407" t="s">
-        <v>37</v>
-      </c>
-      <c r="F407" t="s">
-        <v>38</v>
       </c>
       <c r="G407" s="1">
         <v>46302</v>
@@ -13898,10 +13973,10 @@
         <v>154</v>
       </c>
       <c r="E408" t="s">
-        <v>37</v>
+        <v>836</v>
       </c>
       <c r="F408" t="s">
-        <v>38</v>
+        <v>837</v>
       </c>
       <c r="G408" s="1">
         <v>46302</v>
@@ -13915,7 +13990,7 @@
         <v>0</v>
       </c>
       <c r="B409" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="C409">
         <v>1</v>
@@ -13941,7 +14016,7 @@
         <v>0</v>
       </c>
       <c r="B410" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
       <c r="C410">
         <v>1</v>
@@ -13950,10 +14025,10 @@
         <v>154</v>
       </c>
       <c r="E410" t="s">
-        <v>264</v>
+        <v>37</v>
       </c>
       <c r="F410" t="s">
-        <v>265</v>
+        <v>38</v>
       </c>
       <c r="G410" s="1">
         <v>46302</v>
@@ -13967,7 +14042,7 @@
         <v>0</v>
       </c>
       <c r="B411" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="C411">
         <v>1</v>
@@ -13976,10 +14051,10 @@
         <v>154</v>
       </c>
       <c r="E411" t="s">
-        <v>692</v>
+        <v>841</v>
       </c>
       <c r="F411" t="s">
-        <v>693</v>
+        <v>842</v>
       </c>
       <c r="G411" s="1">
         <v>46302</v>
@@ -13993,7 +14068,7 @@
         <v>0</v>
       </c>
       <c r="B412" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
       <c r="C412">
         <v>1</v>
@@ -14016,62 +14091,62 @@
     </row>
     <row r="413" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A413" t="s">
-        <v>840</v>
+        <v>0</v>
       </c>
       <c r="B413" t="s">
-        <v>841</v>
+        <v>844</v>
       </c>
       <c r="C413">
         <v>1</v>
       </c>
       <c r="D413" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E413" t="s">
-        <v>200</v>
+        <v>264</v>
       </c>
       <c r="F413" t="s">
-        <v>201</v>
+        <v>265</v>
       </c>
       <c r="G413" s="1">
-        <v>46148</v>
+        <v>46302</v>
       </c>
       <c r="H413" s="1">
-        <v>46149</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="414" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A414" t="s">
-        <v>840</v>
+        <v>0</v>
       </c>
       <c r="B414" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="C414">
         <v>1</v>
       </c>
       <c r="D414" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E414" t="s">
-        <v>111</v>
+        <v>692</v>
       </c>
       <c r="F414" t="s">
-        <v>112</v>
+        <v>693</v>
       </c>
       <c r="G414" s="1">
-        <v>46268</v>
+        <v>46302</v>
       </c>
       <c r="H414" s="1">
-        <v>46268</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="415" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A415" t="s">
-        <v>840</v>
+        <v>0</v>
       </c>
       <c r="B415" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
       <c r="C415">
         <v>1</v>
@@ -14080,24 +14155,24 @@
         <v>154</v>
       </c>
       <c r="E415" t="s">
-        <v>844</v>
+        <v>37</v>
       </c>
       <c r="F415" t="s">
-        <v>845</v>
+        <v>38</v>
       </c>
       <c r="G415" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="H415" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="416" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A416" t="s">
-        <v>840</v>
+        <v>0</v>
       </c>
       <c r="B416" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C416">
         <v>1</v>
@@ -14106,10 +14181,10 @@
         <v>154</v>
       </c>
       <c r="E416" t="s">
-        <v>692</v>
+        <v>758</v>
       </c>
       <c r="F416" t="s">
-        <v>693</v>
+        <v>759</v>
       </c>
       <c r="G416" s="1">
         <v>46302</v>
@@ -14120,10 +14195,10 @@
     </row>
     <row r="417" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A417" t="s">
-        <v>840</v>
+        <v>0</v>
       </c>
       <c r="B417" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="C417">
         <v>1</v>
@@ -14132,10 +14207,10 @@
         <v>154</v>
       </c>
       <c r="E417" t="s">
-        <v>848</v>
+        <v>37</v>
       </c>
       <c r="F417" t="s">
-        <v>849</v>
+        <v>38</v>
       </c>
       <c r="G417" s="1">
         <v>46302</v>
@@ -14146,33 +14221,33 @@
     </row>
     <row r="418" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A418" t="s">
+        <v>0</v>
+      </c>
+      <c r="B418" t="s">
+        <v>849</v>
+      </c>
+      <c r="C418">
+        <v>1</v>
+      </c>
+      <c r="D418" t="s">
+        <v>154</v>
+      </c>
+      <c r="E418" t="s">
         <v>850</v>
       </c>
-      <c r="B418" t="s">
+      <c r="F418" t="s">
         <v>851</v>
       </c>
-      <c r="C418">
-        <v>1</v>
-      </c>
-      <c r="D418" t="s">
-        <v>6</v>
-      </c>
-      <c r="E418" t="s">
-        <v>41</v>
-      </c>
-      <c r="F418" t="s">
-        <v>42</v>
-      </c>
       <c r="G418" s="1">
-        <v>46133</v>
+        <v>46302</v>
       </c>
       <c r="H418" s="1">
-        <v>46134</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="419" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A419" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B419" t="s">
         <v>852</v>
@@ -14181,24 +14256,24 @@
         <v>1</v>
       </c>
       <c r="D419" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E419" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F419" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G419" s="1">
-        <v>46134</v>
+        <v>46302</v>
       </c>
       <c r="H419" s="1">
-        <v>46134</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="420" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A420" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B420" t="s">
         <v>853</v>
@@ -14207,183 +14282,183 @@
         <v>1</v>
       </c>
       <c r="D420" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E420" t="s">
-        <v>19</v>
+        <v>850</v>
       </c>
       <c r="F420" t="s">
-        <v>20</v>
+        <v>851</v>
       </c>
       <c r="G420" s="1">
-        <v>46156</v>
+        <v>46302</v>
       </c>
       <c r="H420" s="1">
-        <v>46156</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="421" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A421" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B421" t="s">
         <v>854</v>
       </c>
       <c r="C421">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D421" t="s">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="E421" t="s">
-        <v>855</v>
+        <v>614</v>
       </c>
       <c r="F421" t="s">
-        <v>856</v>
+        <v>615</v>
       </c>
       <c r="G421" s="1">
-        <v>46209</v>
+        <v>46302</v>
       </c>
       <c r="H421" s="1">
-        <v>46218</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="422" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A422" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B422" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="C422">
         <v>1</v>
       </c>
       <c r="D422" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E422" t="s">
-        <v>858</v>
+        <v>37</v>
       </c>
       <c r="F422" t="s">
-        <v>859</v>
+        <v>38</v>
       </c>
       <c r="G422" s="1">
-        <v>46213</v>
+        <v>46302</v>
       </c>
       <c r="H422" s="1">
-        <v>46213</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="423" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A423" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B423" t="s">
-        <v>860</v>
+        <v>856</v>
       </c>
       <c r="C423">
         <v>1</v>
       </c>
       <c r="D423" t="s">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="E423" t="s">
-        <v>861</v>
+        <v>37</v>
       </c>
       <c r="F423" t="s">
-        <v>862</v>
+        <v>38</v>
       </c>
       <c r="G423" s="1">
-        <v>46213</v>
+        <v>46302</v>
       </c>
       <c r="H423" s="1">
-        <v>46216</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="424" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A424" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B424" t="s">
-        <v>863</v>
+        <v>857</v>
       </c>
       <c r="C424">
         <v>1</v>
       </c>
       <c r="D424" t="s">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="E424" t="s">
-        <v>861</v>
+        <v>37</v>
       </c>
       <c r="F424" t="s">
-        <v>862</v>
+        <v>38</v>
       </c>
       <c r="G424" s="1">
-        <v>46224</v>
+        <v>46302</v>
       </c>
       <c r="H424" s="1">
-        <v>46224</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="425" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A425" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B425" t="s">
-        <v>864</v>
+        <v>858</v>
       </c>
       <c r="C425">
         <v>1</v>
       </c>
       <c r="D425" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E425" t="s">
-        <v>865</v>
+        <v>37</v>
       </c>
       <c r="F425" t="s">
-        <v>866</v>
+        <v>38</v>
       </c>
       <c r="G425" s="1">
-        <v>46253</v>
+        <v>46302</v>
       </c>
       <c r="H425" s="1">
-        <v>46253</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="426" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A426" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B426" t="s">
-        <v>867</v>
+        <v>859</v>
       </c>
       <c r="C426">
         <v>1</v>
       </c>
       <c r="D426" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E426" t="s">
-        <v>211</v>
+        <v>860</v>
       </c>
       <c r="F426" t="s">
-        <v>212</v>
+        <v>861</v>
       </c>
       <c r="G426" s="1">
-        <v>46273</v>
+        <v>46302</v>
       </c>
       <c r="H426" s="1">
-        <v>46274</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="427" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A427" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B427" t="s">
-        <v>868</v>
+        <v>862</v>
       </c>
       <c r="C427">
         <v>1</v>
@@ -14392,24 +14467,24 @@
         <v>154</v>
       </c>
       <c r="E427" t="s">
-        <v>510</v>
+        <v>860</v>
       </c>
       <c r="F427" t="s">
-        <v>511</v>
+        <v>861</v>
       </c>
       <c r="G427" s="1">
-        <v>46297</v>
+        <v>46302</v>
       </c>
       <c r="H427" s="1">
-        <v>46297</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="428" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A428" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B428" t="s">
-        <v>869</v>
+        <v>863</v>
       </c>
       <c r="C428">
         <v>1</v>
@@ -14418,24 +14493,24 @@
         <v>154</v>
       </c>
       <c r="E428" t="s">
-        <v>870</v>
+        <v>628</v>
       </c>
       <c r="F428" t="s">
-        <v>871</v>
+        <v>629</v>
       </c>
       <c r="G428" s="1">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="H428" s="1">
-        <v>46300</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="429" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A429" t="s">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="B429" t="s">
-        <v>872</v>
+        <v>864</v>
       </c>
       <c r="C429">
         <v>1</v>
@@ -14444,24 +14519,24 @@
         <v>154</v>
       </c>
       <c r="E429" t="s">
-        <v>870</v>
+        <v>841</v>
       </c>
       <c r="F429" t="s">
-        <v>871</v>
+        <v>842</v>
       </c>
       <c r="G429" s="1">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="H429" s="1">
-        <v>46300</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="430" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A430" t="s">
-        <v>850</v>
+        <v>865</v>
       </c>
       <c r="B430" t="s">
-        <v>873</v>
+        <v>866</v>
       </c>
       <c r="C430">
         <v>1</v>
@@ -14470,50 +14545,50 @@
         <v>2</v>
       </c>
       <c r="E430" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="F430" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="G430" s="1">
-        <v>46300</v>
+        <v>46148</v>
       </c>
       <c r="H430" s="1">
-        <v>46300</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="431" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A431" t="s">
-        <v>850</v>
+        <v>865</v>
       </c>
       <c r="B431" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="C431">
         <v>1</v>
       </c>
       <c r="D431" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E431" t="s">
-        <v>221</v>
+        <v>111</v>
       </c>
       <c r="F431" t="s">
-        <v>222</v>
+        <v>112</v>
       </c>
       <c r="G431" s="1">
-        <v>46300</v>
+        <v>46268</v>
       </c>
       <c r="H431" s="1">
-        <v>46300</v>
+        <v>46268</v>
       </c>
     </row>
     <row r="432" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A432" t="s">
-        <v>850</v>
+        <v>865</v>
       </c>
       <c r="B432" t="s">
-        <v>875</v>
+        <v>868</v>
       </c>
       <c r="C432">
         <v>1</v>
@@ -14522,13 +14597,13 @@
         <v>154</v>
       </c>
       <c r="E432" t="s">
-        <v>861</v>
+        <v>869</v>
       </c>
       <c r="F432" t="s">
-        <v>862</v>
+        <v>870</v>
       </c>
       <c r="G432" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H432" s="1">
         <v>46301</v>
@@ -14536,10 +14611,10 @@
     </row>
     <row r="433" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A433" t="s">
-        <v>850</v>
+        <v>865</v>
       </c>
       <c r="B433" t="s">
-        <v>876</v>
+        <v>871</v>
       </c>
       <c r="C433">
         <v>1</v>
@@ -14548,24 +14623,24 @@
         <v>154</v>
       </c>
       <c r="E433" t="s">
-        <v>861</v>
+        <v>692</v>
       </c>
       <c r="F433" t="s">
-        <v>862</v>
+        <v>693</v>
       </c>
       <c r="G433" s="1">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="H433" s="1">
-        <v>46300</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="434" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A434" t="s">
-        <v>850</v>
+        <v>865</v>
       </c>
       <c r="B434" t="s">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="C434">
         <v>1</v>
@@ -14574,125 +14649,125 @@
         <v>154</v>
       </c>
       <c r="E434" t="s">
-        <v>861</v>
+        <v>873</v>
       </c>
       <c r="F434" t="s">
-        <v>862</v>
+        <v>874</v>
       </c>
       <c r="G434" s="1">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="H434" s="1">
-        <v>46300</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="435" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A435" t="s">
-        <v>850</v>
+        <v>875</v>
       </c>
       <c r="B435" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="C435">
         <v>1</v>
       </c>
       <c r="D435" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E435" t="s">
-        <v>870</v>
+        <v>41</v>
       </c>
       <c r="F435" t="s">
-        <v>871</v>
+        <v>42</v>
       </c>
       <c r="G435" s="1">
-        <v>46301</v>
+        <v>46133</v>
       </c>
       <c r="H435" s="1">
-        <v>46301</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="436" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A436" t="s">
-        <v>850</v>
+        <v>875</v>
       </c>
       <c r="B436" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="C436">
         <v>1</v>
       </c>
       <c r="D436" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E436" t="s">
-        <v>474</v>
+        <v>41</v>
       </c>
       <c r="F436" t="s">
-        <v>475</v>
+        <v>42</v>
       </c>
       <c r="G436" s="1">
-        <v>46302</v>
+        <v>46134</v>
       </c>
       <c r="H436" s="1">
-        <v>46302</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="437" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A437" t="s">
-        <v>850</v>
+        <v>875</v>
       </c>
       <c r="B437" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="C437">
         <v>1</v>
       </c>
       <c r="D437" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E437" t="s">
-        <v>264</v>
+        <v>19</v>
       </c>
       <c r="F437" t="s">
-        <v>265</v>
+        <v>20</v>
       </c>
       <c r="G437" s="1">
-        <v>46302</v>
+        <v>46156</v>
       </c>
       <c r="H437" s="1">
-        <v>46302</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="438" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A438" t="s">
-        <v>850</v>
+        <v>875</v>
       </c>
       <c r="B438" t="s">
+        <v>879</v>
+      </c>
+      <c r="C438">
+        <v>2</v>
+      </c>
+      <c r="D438" t="s">
+        <v>95</v>
+      </c>
+      <c r="E438" t="s">
+        <v>880</v>
+      </c>
+      <c r="F438" t="s">
         <v>881</v>
       </c>
-      <c r="C438">
-        <v>1</v>
-      </c>
-      <c r="D438" t="s">
-        <v>154</v>
-      </c>
-      <c r="E438" t="s">
-        <v>855</v>
-      </c>
-      <c r="F438" t="s">
-        <v>856</v>
-      </c>
       <c r="G438" s="1">
-        <v>46302</v>
+        <v>46209</v>
       </c>
       <c r="H438" s="1">
-        <v>46302</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="439" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A439" t="s">
-        <v>850</v>
+        <v>875</v>
       </c>
       <c r="B439" t="s">
         <v>882</v>
@@ -14701,27 +14776,27 @@
         <v>1</v>
       </c>
       <c r="D439" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E439" t="s">
-        <v>264</v>
+        <v>883</v>
       </c>
       <c r="F439" t="s">
-        <v>265</v>
+        <v>884</v>
       </c>
       <c r="G439" s="1">
-        <v>46302</v>
+        <v>46213</v>
       </c>
       <c r="H439" s="1">
-        <v>46302</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="440" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A440" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B440" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="C440">
         <v>1</v>
@@ -14730,76 +14805,76 @@
         <v>95</v>
       </c>
       <c r="E440" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="F440" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="G440" s="1">
-        <v>46063</v>
+        <v>46213</v>
       </c>
       <c r="H440" s="1">
-        <v>46064</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="441" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A441" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B441" t="s">
+        <v>888</v>
+      </c>
+      <c r="C441">
+        <v>1</v>
+      </c>
+      <c r="D441" t="s">
+        <v>95</v>
+      </c>
+      <c r="E441" t="s">
+        <v>886</v>
+      </c>
+      <c r="F441" t="s">
         <v>887</v>
       </c>
-      <c r="C441">
-        <v>1</v>
-      </c>
-      <c r="D441" t="s">
-        <v>6</v>
-      </c>
-      <c r="E441" t="s">
-        <v>57</v>
-      </c>
-      <c r="F441" t="s">
-        <v>58</v>
-      </c>
       <c r="G441" s="1">
-        <v>46113</v>
+        <v>46224</v>
       </c>
       <c r="H441" s="1">
-        <v>46125</v>
+        <v>46224</v>
       </c>
     </row>
     <row r="442" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A442" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B442" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="C442">
         <v>1</v>
       </c>
       <c r="D442" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E442" t="s">
-        <v>57</v>
+        <v>890</v>
       </c>
       <c r="F442" t="s">
-        <v>58</v>
+        <v>891</v>
       </c>
       <c r="G442" s="1">
-        <v>46125</v>
+        <v>46253</v>
       </c>
       <c r="H442" s="1">
-        <v>46125</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="443" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A443" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B443" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="C443">
         <v>1</v>
@@ -14808,102 +14883,102 @@
         <v>2</v>
       </c>
       <c r="E443" t="s">
-        <v>57</v>
+        <v>211</v>
       </c>
       <c r="F443" t="s">
-        <v>58</v>
+        <v>212</v>
       </c>
       <c r="G443" s="1">
-        <v>46126</v>
+        <v>46273</v>
       </c>
       <c r="H443" s="1">
-        <v>46126</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="444" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A444" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B444" t="s">
-        <v>890</v>
+        <v>893</v>
       </c>
       <c r="C444">
         <v>1</v>
       </c>
       <c r="D444" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E444" t="s">
-        <v>57</v>
+        <v>510</v>
       </c>
       <c r="F444" t="s">
-        <v>58</v>
+        <v>511</v>
       </c>
       <c r="G444" s="1">
-        <v>46126</v>
+        <v>46297</v>
       </c>
       <c r="H444" s="1">
-        <v>46126</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="445" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A445" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B445" t="s">
-        <v>891</v>
+        <v>894</v>
       </c>
       <c r="C445">
         <v>1</v>
       </c>
       <c r="D445" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E445" t="s">
-        <v>57</v>
+        <v>895</v>
       </c>
       <c r="F445" t="s">
-        <v>58</v>
+        <v>896</v>
       </c>
       <c r="G445" s="1">
-        <v>46128</v>
+        <v>46300</v>
       </c>
       <c r="H445" s="1">
-        <v>46128</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="446" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A446" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B446" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="C446">
         <v>1</v>
       </c>
       <c r="D446" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E446" t="s">
-        <v>57</v>
+        <v>895</v>
       </c>
       <c r="F446" t="s">
-        <v>58</v>
+        <v>896</v>
       </c>
       <c r="G446" s="1">
-        <v>46132</v>
+        <v>46300</v>
       </c>
       <c r="H446" s="1">
-        <v>46132</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="447" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A447" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B447" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="C447">
         <v>1</v>
@@ -14912,206 +14987,206 @@
         <v>2</v>
       </c>
       <c r="E447" t="s">
-        <v>57</v>
+        <v>221</v>
       </c>
       <c r="F447" t="s">
-        <v>58</v>
+        <v>222</v>
       </c>
       <c r="G447" s="1">
-        <v>46161</v>
+        <v>46300</v>
       </c>
       <c r="H447" s="1">
-        <v>46161</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="448" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A448" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B448" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
       <c r="C448">
         <v>1</v>
       </c>
       <c r="D448" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E448" t="s">
-        <v>57</v>
+        <v>221</v>
       </c>
       <c r="F448" t="s">
-        <v>58</v>
+        <v>222</v>
       </c>
       <c r="G448" s="1">
-        <v>46174</v>
+        <v>46300</v>
       </c>
       <c r="H448" s="1">
-        <v>46174</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="449" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A449" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B449" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="C449">
         <v>1</v>
       </c>
       <c r="D449" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E449" t="s">
-        <v>57</v>
+        <v>886</v>
       </c>
       <c r="F449" t="s">
-        <v>58</v>
+        <v>887</v>
       </c>
       <c r="G449" s="1">
-        <v>46174</v>
+        <v>46300</v>
       </c>
       <c r="H449" s="1">
-        <v>46174</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="450" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A450" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B450" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="C450">
         <v>1</v>
       </c>
       <c r="D450" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E450" t="s">
-        <v>57</v>
+        <v>886</v>
       </c>
       <c r="F450" t="s">
-        <v>58</v>
+        <v>887</v>
       </c>
       <c r="G450" s="1">
-        <v>46195</v>
+        <v>46300</v>
       </c>
       <c r="H450" s="1">
-        <v>46252</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="451" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A451" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B451" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="C451">
         <v>1</v>
       </c>
       <c r="D451" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E451" t="s">
-        <v>57</v>
+        <v>886</v>
       </c>
       <c r="F451" t="s">
-        <v>58</v>
+        <v>887</v>
       </c>
       <c r="G451" s="1">
-        <v>46210</v>
+        <v>46300</v>
       </c>
       <c r="H451" s="1">
-        <v>46210</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="452" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A452" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B452" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="C452">
         <v>1</v>
       </c>
       <c r="D452" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E452" t="s">
-        <v>57</v>
+        <v>895</v>
       </c>
       <c r="F452" t="s">
-        <v>58</v>
+        <v>896</v>
       </c>
       <c r="G452" s="1">
-        <v>46213</v>
+        <v>46301</v>
       </c>
       <c r="H452" s="1">
-        <v>46213</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="453" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A453" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B453" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="C453">
         <v>1</v>
       </c>
       <c r="D453" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E453" t="s">
-        <v>57</v>
+        <v>474</v>
       </c>
       <c r="F453" t="s">
-        <v>58</v>
+        <v>475</v>
       </c>
       <c r="G453" s="1">
-        <v>46218</v>
+        <v>46302</v>
       </c>
       <c r="H453" s="1">
-        <v>46252</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="454" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A454" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B454" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="C454">
         <v>1</v>
       </c>
       <c r="D454" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E454" t="s">
-        <v>77</v>
+        <v>264</v>
       </c>
       <c r="F454" t="s">
-        <v>78</v>
+        <v>265</v>
       </c>
       <c r="G454" s="1">
-        <v>46226</v>
+        <v>46302</v>
       </c>
       <c r="H454" s="1">
-        <v>46226</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="455" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A455" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B455" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
       <c r="C455">
         <v>1</v>
@@ -15120,76 +15195,76 @@
         <v>154</v>
       </c>
       <c r="E455" t="s">
-        <v>57</v>
+        <v>880</v>
       </c>
       <c r="F455" t="s">
-        <v>58</v>
+        <v>881</v>
       </c>
       <c r="G455" s="1">
-        <v>46227</v>
+        <v>46302</v>
       </c>
       <c r="H455" s="1">
-        <v>46252</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="456" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A456" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B456" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="C456">
         <v>1</v>
       </c>
       <c r="D456" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E456" t="s">
-        <v>57</v>
+        <v>264</v>
       </c>
       <c r="F456" t="s">
-        <v>58</v>
+        <v>265</v>
       </c>
       <c r="G456" s="1">
-        <v>46227</v>
+        <v>46302</v>
       </c>
       <c r="H456" s="1">
-        <v>46252</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="457" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A457" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B457" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
       <c r="C457">
         <v>1</v>
       </c>
       <c r="D457" t="s">
-        <v>6</v>
+        <v>95</v>
       </c>
       <c r="E457" t="s">
-        <v>57</v>
+        <v>910</v>
       </c>
       <c r="F457" t="s">
-        <v>58</v>
+        <v>911</v>
       </c>
       <c r="G457" s="1">
-        <v>46227</v>
+        <v>46063</v>
       </c>
       <c r="H457" s="1">
-        <v>46228</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="458" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A458" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B458" t="s">
-        <v>904</v>
+        <v>912</v>
       </c>
       <c r="C458">
         <v>1</v>
@@ -15198,30 +15273,30 @@
         <v>6</v>
       </c>
       <c r="E458" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="F458" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G458" s="1">
-        <v>46230</v>
+        <v>46113</v>
       </c>
       <c r="H458" s="1">
-        <v>46252</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="459" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A459" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B459" t="s">
-        <v>905</v>
+        <v>913</v>
       </c>
       <c r="C459">
         <v>1</v>
       </c>
       <c r="D459" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E459" t="s">
         <v>57</v>
@@ -15230,24 +15305,24 @@
         <v>58</v>
       </c>
       <c r="G459" s="1">
-        <v>46231</v>
+        <v>46125</v>
       </c>
       <c r="H459" s="1">
-        <v>46231</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="460" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A460" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B460" t="s">
-        <v>906</v>
+        <v>914</v>
       </c>
       <c r="C460">
         <v>1</v>
       </c>
       <c r="D460" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E460" t="s">
         <v>57</v>
@@ -15256,18 +15331,18 @@
         <v>58</v>
       </c>
       <c r="G460" s="1">
-        <v>46254</v>
+        <v>46126</v>
       </c>
       <c r="H460" s="1">
-        <v>46254</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="461" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A461" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B461" t="s">
-        <v>907</v>
+        <v>915</v>
       </c>
       <c r="C461">
         <v>1</v>
@@ -15282,24 +15357,24 @@
         <v>58</v>
       </c>
       <c r="G461" s="1">
-        <v>46255</v>
+        <v>46126</v>
       </c>
       <c r="H461" s="1">
-        <v>46255</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="462" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A462" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B462" t="s">
-        <v>908</v>
+        <v>916</v>
       </c>
       <c r="C462">
         <v>1</v>
       </c>
       <c r="D462" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E462" t="s">
         <v>57</v>
@@ -15308,18 +15383,18 @@
         <v>58</v>
       </c>
       <c r="G462" s="1">
-        <v>46260</v>
+        <v>46128</v>
       </c>
       <c r="H462" s="1">
-        <v>46260</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="463" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A463" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B463" t="s">
-        <v>909</v>
+        <v>917</v>
       </c>
       <c r="C463">
         <v>1</v>
@@ -15334,24 +15409,24 @@
         <v>58</v>
       </c>
       <c r="G463" s="1">
-        <v>46289</v>
+        <v>46132</v>
       </c>
       <c r="H463" s="1">
-        <v>46289</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="464" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A464" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B464" t="s">
-        <v>910</v>
+        <v>918</v>
       </c>
       <c r="C464">
         <v>1</v>
       </c>
       <c r="D464" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E464" t="s">
         <v>57</v>
@@ -15360,24 +15435,24 @@
         <v>58</v>
       </c>
       <c r="G464" s="1">
-        <v>46294</v>
+        <v>46161</v>
       </c>
       <c r="H464" s="1">
-        <v>46294</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="465" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A465" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B465" t="s">
-        <v>911</v>
+        <v>919</v>
       </c>
       <c r="C465">
         <v>1</v>
       </c>
       <c r="D465" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E465" t="s">
         <v>57</v>
@@ -15386,50 +15461,50 @@
         <v>58</v>
       </c>
       <c r="G465" s="1">
-        <v>46302</v>
+        <v>46174</v>
       </c>
       <c r="H465" s="1">
-        <v>46302</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="466" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A466" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B466" t="s">
-        <v>912</v>
+        <v>920</v>
       </c>
       <c r="C466">
         <v>1</v>
       </c>
       <c r="D466" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E466" t="s">
-        <v>605</v>
+        <v>57</v>
       </c>
       <c r="F466" t="s">
-        <v>606</v>
+        <v>58</v>
       </c>
       <c r="G466" s="1">
-        <v>46302</v>
+        <v>46174</v>
       </c>
       <c r="H466" s="1">
-        <v>46302</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="467" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A467" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B467" t="s">
-        <v>913</v>
+        <v>921</v>
       </c>
       <c r="C467">
         <v>1</v>
       </c>
       <c r="D467" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E467" t="s">
         <v>57</v>
@@ -15438,24 +15513,24 @@
         <v>58</v>
       </c>
       <c r="G467" s="1">
-        <v>46302</v>
+        <v>46195</v>
       </c>
       <c r="H467" s="1">
-        <v>46302</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="468" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A468" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B468" t="s">
-        <v>914</v>
+        <v>922</v>
       </c>
       <c r="C468">
         <v>1</v>
       </c>
       <c r="D468" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E468" t="s">
         <v>57</v>
@@ -15464,24 +15539,24 @@
         <v>58</v>
       </c>
       <c r="G468" s="1">
-        <v>46302</v>
+        <v>46210</v>
       </c>
       <c r="H468" s="1">
-        <v>46302</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="469" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A469" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B469" t="s">
-        <v>915</v>
+        <v>923</v>
       </c>
       <c r="C469">
         <v>1</v>
       </c>
       <c r="D469" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E469" t="s">
         <v>57</v>
@@ -15490,24 +15565,24 @@
         <v>58</v>
       </c>
       <c r="G469" s="1">
-        <v>46302</v>
+        <v>46213</v>
       </c>
       <c r="H469" s="1">
-        <v>46302</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="470" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A470" t="s">
-        <v>883</v>
+        <v>908</v>
       </c>
       <c r="B470" t="s">
-        <v>916</v>
+        <v>924</v>
       </c>
       <c r="C470">
         <v>1</v>
       </c>
       <c r="D470" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E470" t="s">
         <v>57</v>
@@ -15516,200 +15591,200 @@
         <v>58</v>
       </c>
       <c r="G470" s="1">
-        <v>46302</v>
+        <v>46218</v>
       </c>
       <c r="H470" s="1">
-        <v>46302</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="471" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A471" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B471" t="s">
-        <v>918</v>
+        <v>925</v>
       </c>
       <c r="C471">
         <v>1</v>
       </c>
       <c r="D471" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E471" t="s">
-        <v>919</v>
+        <v>77</v>
       </c>
       <c r="F471" t="s">
-        <v>920</v>
+        <v>78</v>
       </c>
       <c r="G471" s="1">
-        <v>46157</v>
+        <v>46226</v>
       </c>
       <c r="H471" s="1">
-        <v>46157</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="472" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A472" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B472" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="C472">
         <v>1</v>
       </c>
       <c r="D472" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E472" t="s">
-        <v>922</v>
+        <v>57</v>
       </c>
       <c r="F472" t="s">
-        <v>923</v>
+        <v>58</v>
       </c>
       <c r="G472" s="1">
-        <v>46168</v>
+        <v>46227</v>
       </c>
       <c r="H472" s="1">
-        <v>46170</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="473" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A473" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B473" t="s">
-        <v>924</v>
+        <v>927</v>
       </c>
       <c r="C473">
         <v>1</v>
       </c>
       <c r="D473" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E473" t="s">
-        <v>919</v>
+        <v>57</v>
       </c>
       <c r="F473" t="s">
-        <v>920</v>
+        <v>58</v>
       </c>
       <c r="G473" s="1">
-        <v>46218</v>
+        <v>46227</v>
       </c>
       <c r="H473" s="1">
-        <v>46218</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="474" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A474" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B474" t="s">
-        <v>925</v>
+        <v>928</v>
       </c>
       <c r="C474">
         <v>1</v>
       </c>
       <c r="D474" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E474" t="s">
-        <v>919</v>
+        <v>57</v>
       </c>
       <c r="F474" t="s">
-        <v>920</v>
+        <v>58</v>
       </c>
       <c r="G474" s="1">
-        <v>46244</v>
+        <v>46227</v>
       </c>
       <c r="H474" s="1">
-        <v>46244</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="475" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A475" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B475" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="C475">
         <v>1</v>
       </c>
       <c r="D475" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E475" t="s">
-        <v>919</v>
+        <v>77</v>
       </c>
       <c r="F475" t="s">
-        <v>920</v>
+        <v>78</v>
       </c>
       <c r="G475" s="1">
-        <v>46247</v>
+        <v>46230</v>
       </c>
       <c r="H475" s="1">
-        <v>46247</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="476" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A476" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B476" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C476">
         <v>1</v>
       </c>
       <c r="D476" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E476" t="s">
-        <v>928</v>
+        <v>57</v>
       </c>
       <c r="F476" t="s">
-        <v>929</v>
+        <v>58</v>
       </c>
       <c r="G476" s="1">
-        <v>46247</v>
+        <v>46231</v>
       </c>
       <c r="H476" s="1">
-        <v>46247</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="477" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A477" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B477" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="C477">
         <v>1</v>
       </c>
       <c r="D477" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E477" t="s">
-        <v>919</v>
+        <v>57</v>
       </c>
       <c r="F477" t="s">
-        <v>920</v>
+        <v>58</v>
       </c>
       <c r="G477" s="1">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="H477" s="1">
-        <v>46255</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="478" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A478" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B478" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="C478">
         <v>1</v>
@@ -15718,50 +15793,50 @@
         <v>2</v>
       </c>
       <c r="E478" t="s">
-        <v>919</v>
+        <v>57</v>
       </c>
       <c r="F478" t="s">
-        <v>920</v>
+        <v>58</v>
       </c>
       <c r="G478" s="1">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="H478" s="1">
-        <v>46258</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="479" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A479" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B479" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="C479">
         <v>1</v>
       </c>
       <c r="D479" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E479" t="s">
-        <v>919</v>
+        <v>57</v>
       </c>
       <c r="F479" t="s">
-        <v>920</v>
+        <v>58</v>
       </c>
       <c r="G479" s="1">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="H479" s="1">
-        <v>46265</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="480" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A480" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B480" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="C480">
         <v>1</v>
@@ -15770,41 +15845,483 @@
         <v>6</v>
       </c>
       <c r="E480" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="F480" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="G480" s="1">
-        <v>46281</v>
+        <v>46289</v>
       </c>
       <c r="H480" s="1">
-        <v>46283</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="481" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A481" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="B481" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="C481">
         <v>1</v>
       </c>
       <c r="D481" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E481" t="s">
-        <v>861</v>
+        <v>57</v>
       </c>
       <c r="F481" t="s">
-        <v>862</v>
+        <v>58</v>
       </c>
       <c r="G481" s="1">
-        <v>46302</v>
+        <v>46294</v>
       </c>
       <c r="H481" s="1">
+        <v>46294</v>
+      </c>
+    </row>
+    <row r="482" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A482" t="s">
+        <v>908</v>
+      </c>
+      <c r="B482" t="s">
+        <v>936</v>
+      </c>
+      <c r="C482">
+        <v>1</v>
+      </c>
+      <c r="D482" t="s">
+        <v>154</v>
+      </c>
+      <c r="E482" t="s">
+        <v>57</v>
+      </c>
+      <c r="F482" t="s">
+        <v>58</v>
+      </c>
+      <c r="G482" s="1">
+        <v>46302</v>
+      </c>
+      <c r="H482" s="1">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="483" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A483" t="s">
+        <v>908</v>
+      </c>
+      <c r="B483" t="s">
+        <v>937</v>
+      </c>
+      <c r="C483">
+        <v>1</v>
+      </c>
+      <c r="D483" t="s">
+        <v>154</v>
+      </c>
+      <c r="E483" t="s">
+        <v>605</v>
+      </c>
+      <c r="F483" t="s">
+        <v>606</v>
+      </c>
+      <c r="G483" s="1">
+        <v>46302</v>
+      </c>
+      <c r="H483" s="1">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="484" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A484" t="s">
+        <v>908</v>
+      </c>
+      <c r="B484" t="s">
+        <v>938</v>
+      </c>
+      <c r="C484">
+        <v>1</v>
+      </c>
+      <c r="D484" t="s">
+        <v>154</v>
+      </c>
+      <c r="E484" t="s">
+        <v>57</v>
+      </c>
+      <c r="F484" t="s">
+        <v>58</v>
+      </c>
+      <c r="G484" s="1">
+        <v>46302</v>
+      </c>
+      <c r="H484" s="1">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="485" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A485" t="s">
+        <v>908</v>
+      </c>
+      <c r="B485" t="s">
+        <v>939</v>
+      </c>
+      <c r="C485">
+        <v>1</v>
+      </c>
+      <c r="D485" t="s">
+        <v>154</v>
+      </c>
+      <c r="E485" t="s">
+        <v>57</v>
+      </c>
+      <c r="F485" t="s">
+        <v>58</v>
+      </c>
+      <c r="G485" s="1">
+        <v>46302</v>
+      </c>
+      <c r="H485" s="1">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="486" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A486" t="s">
+        <v>908</v>
+      </c>
+      <c r="B486" t="s">
+        <v>940</v>
+      </c>
+      <c r="C486">
+        <v>1</v>
+      </c>
+      <c r="D486" t="s">
+        <v>154</v>
+      </c>
+      <c r="E486" t="s">
+        <v>57</v>
+      </c>
+      <c r="F486" t="s">
+        <v>58</v>
+      </c>
+      <c r="G486" s="1">
+        <v>46302</v>
+      </c>
+      <c r="H486" s="1">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="487" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A487" t="s">
+        <v>908</v>
+      </c>
+      <c r="B487" t="s">
+        <v>941</v>
+      </c>
+      <c r="C487">
+        <v>1</v>
+      </c>
+      <c r="D487" t="s">
+        <v>154</v>
+      </c>
+      <c r="E487" t="s">
+        <v>57</v>
+      </c>
+      <c r="F487" t="s">
+        <v>58</v>
+      </c>
+      <c r="G487" s="1">
+        <v>46302</v>
+      </c>
+      <c r="H487" s="1">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="488" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A488" t="s">
+        <v>942</v>
+      </c>
+      <c r="B488" t="s">
+        <v>943</v>
+      </c>
+      <c r="C488">
+        <v>1</v>
+      </c>
+      <c r="D488" t="s">
+        <v>2</v>
+      </c>
+      <c r="E488" t="s">
+        <v>944</v>
+      </c>
+      <c r="F488" t="s">
+        <v>945</v>
+      </c>
+      <c r="G488" s="1">
+        <v>46157</v>
+      </c>
+      <c r="H488" s="1">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="489" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A489" t="s">
+        <v>942</v>
+      </c>
+      <c r="B489" t="s">
+        <v>946</v>
+      </c>
+      <c r="C489">
+        <v>1</v>
+      </c>
+      <c r="D489" t="s">
+        <v>2</v>
+      </c>
+      <c r="E489" t="s">
+        <v>947</v>
+      </c>
+      <c r="F489" t="s">
+        <v>948</v>
+      </c>
+      <c r="G489" s="1">
+        <v>46168</v>
+      </c>
+      <c r="H489" s="1">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="490" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A490" t="s">
+        <v>942</v>
+      </c>
+      <c r="B490" t="s">
+        <v>949</v>
+      </c>
+      <c r="C490">
+        <v>1</v>
+      </c>
+      <c r="D490" t="s">
+        <v>2</v>
+      </c>
+      <c r="E490" t="s">
+        <v>944</v>
+      </c>
+      <c r="F490" t="s">
+        <v>945</v>
+      </c>
+      <c r="G490" s="1">
+        <v>46218</v>
+      </c>
+      <c r="H490" s="1">
+        <v>46218</v>
+      </c>
+    </row>
+    <row r="491" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A491" t="s">
+        <v>942</v>
+      </c>
+      <c r="B491" t="s">
+        <v>950</v>
+      </c>
+      <c r="C491">
+        <v>1</v>
+      </c>
+      <c r="D491" t="s">
+        <v>2</v>
+      </c>
+      <c r="E491" t="s">
+        <v>944</v>
+      </c>
+      <c r="F491" t="s">
+        <v>945</v>
+      </c>
+      <c r="G491" s="1">
+        <v>46244</v>
+      </c>
+      <c r="H491" s="1">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="492" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A492" t="s">
+        <v>942</v>
+      </c>
+      <c r="B492" t="s">
+        <v>951</v>
+      </c>
+      <c r="C492">
+        <v>1</v>
+      </c>
+      <c r="D492" t="s">
+        <v>2</v>
+      </c>
+      <c r="E492" t="s">
+        <v>944</v>
+      </c>
+      <c r="F492" t="s">
+        <v>945</v>
+      </c>
+      <c r="G492" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H492" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="493" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A493" t="s">
+        <v>942</v>
+      </c>
+      <c r="B493" t="s">
+        <v>952</v>
+      </c>
+      <c r="C493">
+        <v>1</v>
+      </c>
+      <c r="D493" t="s">
+        <v>2</v>
+      </c>
+      <c r="E493" t="s">
+        <v>953</v>
+      </c>
+      <c r="F493" t="s">
+        <v>954</v>
+      </c>
+      <c r="G493" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H493" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="494" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A494" t="s">
+        <v>942</v>
+      </c>
+      <c r="B494" t="s">
+        <v>955</v>
+      </c>
+      <c r="C494">
+        <v>1</v>
+      </c>
+      <c r="D494" t="s">
+        <v>2</v>
+      </c>
+      <c r="E494" t="s">
+        <v>944</v>
+      </c>
+      <c r="F494" t="s">
+        <v>945</v>
+      </c>
+      <c r="G494" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H494" s="1">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="495" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A495" t="s">
+        <v>942</v>
+      </c>
+      <c r="B495" t="s">
+        <v>956</v>
+      </c>
+      <c r="C495">
+        <v>1</v>
+      </c>
+      <c r="D495" t="s">
+        <v>2</v>
+      </c>
+      <c r="E495" t="s">
+        <v>944</v>
+      </c>
+      <c r="F495" t="s">
+        <v>945</v>
+      </c>
+      <c r="G495" s="1">
+        <v>46258</v>
+      </c>
+      <c r="H495" s="1">
+        <v>46258</v>
+      </c>
+    </row>
+    <row r="496" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A496" t="s">
+        <v>942</v>
+      </c>
+      <c r="B496" t="s">
+        <v>957</v>
+      </c>
+      <c r="C496">
+        <v>1</v>
+      </c>
+      <c r="D496" t="s">
+        <v>2</v>
+      </c>
+      <c r="E496" t="s">
+        <v>944</v>
+      </c>
+      <c r="F496" t="s">
+        <v>945</v>
+      </c>
+      <c r="G496" s="1">
+        <v>46262</v>
+      </c>
+      <c r="H496" s="1">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="497" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A497" t="s">
+        <v>942</v>
+      </c>
+      <c r="B497" t="s">
+        <v>958</v>
+      </c>
+      <c r="C497">
+        <v>1</v>
+      </c>
+      <c r="D497" t="s">
+        <v>6</v>
+      </c>
+      <c r="E497" t="s">
+        <v>13</v>
+      </c>
+      <c r="F497" t="s">
+        <v>14</v>
+      </c>
+      <c r="G497" s="1">
+        <v>46281</v>
+      </c>
+      <c r="H497" s="1">
+        <v>46283</v>
+      </c>
+    </row>
+    <row r="498" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A498" t="s">
+        <v>942</v>
+      </c>
+      <c r="B498" t="s">
+        <v>959</v>
+      </c>
+      <c r="C498">
+        <v>1</v>
+      </c>
+      <c r="D498" t="s">
+        <v>154</v>
+      </c>
+      <c r="E498" t="s">
+        <v>886</v>
+      </c>
+      <c r="F498" t="s">
+        <v>887</v>
+      </c>
+      <c r="G498" s="1">
+        <v>46302</v>
+      </c>
+      <c r="H498" s="1">
         <v>46302</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 08/10/2026 08:51:50
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AE01ED8-A4B1-4CC1-934F-86A74D524A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{610201F1-A254-4686-970A-966208E3BAD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30930" yWindow="10005" windowWidth="15000" windowHeight="6195" xr2:uid="{CF312FA0-55D7-4249-8BA7-8CABA3C451E8}"/>
+    <workbookView xWindow="30930" yWindow="10005" windowWidth="15000" windowHeight="6195" xr2:uid="{F95E397D-4038-4488-B2AD-99D02EA2A302}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2493" uniqueCount="968">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2508" uniqueCount="977">
   <si>
     <t>0001</t>
   </si>
@@ -2617,6 +2617,54 @@
     <t xml:space="preserve">  217186</t>
   </si>
   <si>
+    <t xml:space="preserve">  217187</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217188</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217189</t>
+  </si>
+  <si>
+    <t>SC38</t>
+  </si>
+  <si>
+    <t>SANITARIOS CORTESE SRL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217190</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217192</t>
+  </si>
+  <si>
+    <t>DA28</t>
+  </si>
+  <si>
+    <t>DAPESOL S.A. -MATERIALES ACON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217193</t>
+  </si>
+  <si>
+    <t>RR12</t>
+  </si>
+  <si>
+    <t>RIOS MARIA JOSE Y RIOS MARIA FERNANDA S.H.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217195</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217196</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217197</t>
+  </si>
+  <si>
     <t>0004</t>
   </si>
   <si>
@@ -2725,12 +2773,6 @@
     <t xml:space="preserve">    3006</t>
   </si>
   <si>
-    <t xml:space="preserve">    3007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    3008</t>
-  </si>
-  <si>
     <t xml:space="preserve">    3010</t>
   </si>
   <si>
@@ -2830,22 +2872,7 @@
     <t xml:space="preserve">    2644</t>
   </si>
   <si>
-    <t xml:space="preserve">    2740</t>
-  </si>
-  <si>
     <t xml:space="preserve">    2741</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2742</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2745</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2746</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2748</t>
   </si>
   <si>
     <t>9999</t>
@@ -3373,34 +3400,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0DB821C-4677-411C-A378-21B5CB267C5F}">
-  <dimension ref="A1:H498"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FAE6636-3677-47F9-89D2-E2156C95ADD9}">
+  <dimension ref="A1:H501"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>960</v>
+        <v>969</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>961</v>
+        <v>970</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>962</v>
+        <v>971</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>963</v>
+        <v>972</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>964</v>
+        <v>973</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>965</v>
+        <v>974</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>966</v>
+        <v>975</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>967</v>
+        <v>976</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -6430,7 +6457,7 @@
         <v>2</v>
       </c>
       <c r="D118" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E118" t="s">
         <v>290</v>
@@ -7990,7 +8017,7 @@
         <v>1</v>
       </c>
       <c r="D178" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E178" t="s">
         <v>48</v>
@@ -8016,7 +8043,7 @@
         <v>1</v>
       </c>
       <c r="D179" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E179" t="s">
         <v>16</v>
@@ -8042,7 +8069,7 @@
         <v>1</v>
       </c>
       <c r="D180" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E180" t="s">
         <v>182</v>
@@ -8250,7 +8277,7 @@
         <v>1</v>
       </c>
       <c r="D188" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E188" t="s">
         <v>420</v>
@@ -8302,7 +8329,7 @@
         <v>1</v>
       </c>
       <c r="D190" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E190" t="s">
         <v>417</v>
@@ -8484,7 +8511,7 @@
         <v>1</v>
       </c>
       <c r="D197" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E197" t="s">
         <v>48</v>
@@ -8562,7 +8589,7 @@
         <v>1</v>
       </c>
       <c r="D200" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E200" t="s">
         <v>16</v>
@@ -8588,7 +8615,7 @@
         <v>1</v>
       </c>
       <c r="D201" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E201" t="s">
         <v>290</v>
@@ -8614,7 +8641,7 @@
         <v>1</v>
       </c>
       <c r="D202" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E202" t="s">
         <v>182</v>
@@ -8692,7 +8719,7 @@
         <v>1</v>
       </c>
       <c r="D205" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E205" t="s">
         <v>172</v>
@@ -10928,7 +10955,7 @@
         <v>1</v>
       </c>
       <c r="D291" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E291" t="s">
         <v>620</v>
@@ -10980,7 +11007,7 @@
         <v>1</v>
       </c>
       <c r="D293" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E293" t="s">
         <v>624</v>
@@ -11084,7 +11111,7 @@
         <v>1</v>
       </c>
       <c r="D297" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E297" t="s">
         <v>635</v>
@@ -11110,7 +11137,7 @@
         <v>1</v>
       </c>
       <c r="D298" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E298" t="s">
         <v>638</v>
@@ -11188,7 +11215,7 @@
         <v>1</v>
       </c>
       <c r="D301" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E301" t="s">
         <v>642</v>
@@ -11214,7 +11241,7 @@
         <v>1</v>
       </c>
       <c r="D302" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E302" t="s">
         <v>642</v>
@@ -11786,7 +11813,7 @@
         <v>1</v>
       </c>
       <c r="D324" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E324" t="s">
         <v>16</v>
@@ -11812,7 +11839,7 @@
         <v>1</v>
       </c>
       <c r="D325" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E325" t="s">
         <v>16</v>
@@ -12514,7 +12541,7 @@
         <v>1</v>
       </c>
       <c r="D352" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E352" t="s">
         <v>642</v>
@@ -12540,7 +12567,7 @@
         <v>1</v>
       </c>
       <c r="D353" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E353" t="s">
         <v>635</v>
@@ -12800,7 +12827,7 @@
         <v>1</v>
       </c>
       <c r="D363" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E363" t="s">
         <v>761</v>
@@ -12826,7 +12853,7 @@
         <v>1</v>
       </c>
       <c r="D364" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E364" t="s">
         <v>764</v>
@@ -13060,7 +13087,7 @@
         <v>1</v>
       </c>
       <c r="D373" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E373" t="s">
         <v>172</v>
@@ -13632,7 +13659,7 @@
         <v>1</v>
       </c>
       <c r="D395" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E395" t="s">
         <v>813</v>
@@ -14533,88 +14560,88 @@
     </row>
     <row r="430" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A430" t="s">
+        <v>0</v>
+      </c>
+      <c r="B430" t="s">
         <v>865</v>
       </c>
-      <c r="B430" t="s">
-        <v>866</v>
-      </c>
       <c r="C430">
         <v>1</v>
       </c>
       <c r="D430" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E430" t="s">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="F430" t="s">
-        <v>201</v>
+        <v>81</v>
       </c>
       <c r="G430" s="1">
-        <v>46148</v>
+        <v>46302</v>
       </c>
       <c r="H430" s="1">
-        <v>46149</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="431" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A431" t="s">
-        <v>865</v>
+        <v>0</v>
       </c>
       <c r="B431" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="C431">
         <v>1</v>
       </c>
       <c r="D431" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E431" t="s">
-        <v>111</v>
+        <v>813</v>
       </c>
       <c r="F431" t="s">
-        <v>112</v>
+        <v>814</v>
       </c>
       <c r="G431" s="1">
-        <v>46268</v>
+        <v>46302</v>
       </c>
       <c r="H431" s="1">
-        <v>46268</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="432" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A432" t="s">
-        <v>865</v>
+        <v>0</v>
       </c>
       <c r="B432" t="s">
+        <v>867</v>
+      </c>
+      <c r="C432">
+        <v>1</v>
+      </c>
+      <c r="D432" t="s">
+        <v>154</v>
+      </c>
+      <c r="E432" t="s">
         <v>868</v>
       </c>
-      <c r="C432">
-        <v>1</v>
-      </c>
-      <c r="D432" t="s">
-        <v>154</v>
-      </c>
-      <c r="E432" t="s">
+      <c r="F432" t="s">
         <v>869</v>
       </c>
-      <c r="F432" t="s">
-        <v>870</v>
-      </c>
       <c r="G432" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="H432" s="1">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="433" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A433" t="s">
-        <v>865</v>
+        <v>0</v>
       </c>
       <c r="B433" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="C433">
         <v>1</v>
@@ -14623,73 +14650,73 @@
         <v>154</v>
       </c>
       <c r="E433" t="s">
-        <v>692</v>
+        <v>868</v>
       </c>
       <c r="F433" t="s">
-        <v>693</v>
+        <v>869</v>
       </c>
       <c r="G433" s="1">
         <v>46302</v>
       </c>
       <c r="H433" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="434" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A434" t="s">
-        <v>865</v>
+        <v>0</v>
       </c>
       <c r="B434" t="s">
+        <v>871</v>
+      </c>
+      <c r="C434">
+        <v>1</v>
+      </c>
+      <c r="D434" t="s">
+        <v>154</v>
+      </c>
+      <c r="E434" t="s">
         <v>872</v>
       </c>
-      <c r="C434">
-        <v>1</v>
-      </c>
-      <c r="D434" t="s">
-        <v>154</v>
-      </c>
-      <c r="E434" t="s">
+      <c r="F434" t="s">
         <v>873</v>
-      </c>
-      <c r="F434" t="s">
-        <v>874</v>
       </c>
       <c r="G434" s="1">
         <v>46302</v>
       </c>
       <c r="H434" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="435" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A435" t="s">
+        <v>0</v>
+      </c>
+      <c r="B435" t="s">
+        <v>874</v>
+      </c>
+      <c r="C435">
+        <v>1</v>
+      </c>
+      <c r="D435" t="s">
+        <v>154</v>
+      </c>
+      <c r="E435" t="s">
         <v>875</v>
       </c>
-      <c r="B435" t="s">
+      <c r="F435" t="s">
         <v>876</v>
       </c>
-      <c r="C435">
-        <v>1</v>
-      </c>
-      <c r="D435" t="s">
-        <v>6</v>
-      </c>
-      <c r="E435" t="s">
-        <v>41</v>
-      </c>
-      <c r="F435" t="s">
-        <v>42</v>
-      </c>
       <c r="G435" s="1">
-        <v>46133</v>
+        <v>46302</v>
       </c>
       <c r="H435" s="1">
-        <v>46134</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="436" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A436" t="s">
-        <v>875</v>
+        <v>0</v>
       </c>
       <c r="B436" t="s">
         <v>877</v>
@@ -14698,24 +14725,24 @@
         <v>1</v>
       </c>
       <c r="D436" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E436" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F436" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G436" s="1">
-        <v>46134</v>
+        <v>46303</v>
       </c>
       <c r="H436" s="1">
-        <v>46134</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="437" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A437" t="s">
-        <v>875</v>
+        <v>0</v>
       </c>
       <c r="B437" t="s">
         <v>878</v>
@@ -14724,183 +14751,183 @@
         <v>1</v>
       </c>
       <c r="D437" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E437" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F437" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="G437" s="1">
-        <v>46156</v>
+        <v>46303</v>
       </c>
       <c r="H437" s="1">
-        <v>46156</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="438" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A438" t="s">
-        <v>875</v>
+        <v>0</v>
       </c>
       <c r="B438" t="s">
         <v>879</v>
       </c>
       <c r="C438">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D438" t="s">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="E438" t="s">
-        <v>880</v>
+        <v>37</v>
       </c>
       <c r="F438" t="s">
-        <v>881</v>
+        <v>38</v>
       </c>
       <c r="G438" s="1">
-        <v>46209</v>
+        <v>46303</v>
       </c>
       <c r="H438" s="1">
-        <v>46218</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="439" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A439" t="s">
-        <v>875</v>
+        <v>0</v>
       </c>
       <c r="B439" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="C439">
         <v>1</v>
       </c>
       <c r="D439" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E439" t="s">
-        <v>883</v>
+        <v>37</v>
       </c>
       <c r="F439" t="s">
-        <v>884</v>
+        <v>38</v>
       </c>
       <c r="G439" s="1">
-        <v>46213</v>
+        <v>46303</v>
       </c>
       <c r="H439" s="1">
-        <v>46213</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="440" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A440" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="B440" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="C440">
         <v>1</v>
       </c>
       <c r="D440" t="s">
-        <v>95</v>
+        <v>2</v>
       </c>
       <c r="E440" t="s">
-        <v>886</v>
+        <v>200</v>
       </c>
       <c r="F440" t="s">
-        <v>887</v>
+        <v>201</v>
       </c>
       <c r="G440" s="1">
-        <v>46213</v>
+        <v>46148</v>
       </c>
       <c r="H440" s="1">
-        <v>46216</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="441" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A441" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="B441" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="C441">
         <v>1</v>
       </c>
       <c r="D441" t="s">
-        <v>95</v>
+        <v>2</v>
       </c>
       <c r="E441" t="s">
-        <v>886</v>
+        <v>111</v>
       </c>
       <c r="F441" t="s">
-        <v>887</v>
+        <v>112</v>
       </c>
       <c r="G441" s="1">
-        <v>46224</v>
+        <v>46268</v>
       </c>
       <c r="H441" s="1">
-        <v>46224</v>
+        <v>46268</v>
       </c>
     </row>
     <row r="442" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A442" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="B442" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="C442">
         <v>1</v>
       </c>
       <c r="D442" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E442" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="F442" t="s">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="G442" s="1">
-        <v>46253</v>
+        <v>46301</v>
       </c>
       <c r="H442" s="1">
-        <v>46253</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="443" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A443" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="B443" t="s">
-        <v>892</v>
+        <v>887</v>
       </c>
       <c r="C443">
         <v>1</v>
       </c>
       <c r="D443" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E443" t="s">
-        <v>211</v>
+        <v>692</v>
       </c>
       <c r="F443" t="s">
-        <v>212</v>
+        <v>693</v>
       </c>
       <c r="G443" s="1">
-        <v>46273</v>
+        <v>46302</v>
       </c>
       <c r="H443" s="1">
-        <v>46274</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="444" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A444" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="B444" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="C444">
         <v>1</v>
@@ -14909,151 +14936,151 @@
         <v>154</v>
       </c>
       <c r="E444" t="s">
-        <v>510</v>
+        <v>889</v>
       </c>
       <c r="F444" t="s">
-        <v>511</v>
+        <v>890</v>
       </c>
       <c r="G444" s="1">
-        <v>46297</v>
+        <v>46302</v>
       </c>
       <c r="H444" s="1">
-        <v>46297</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="445" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A445" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B445" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="C445">
         <v>1</v>
       </c>
       <c r="D445" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E445" t="s">
-        <v>895</v>
+        <v>41</v>
       </c>
       <c r="F445" t="s">
-        <v>896</v>
+        <v>42</v>
       </c>
       <c r="G445" s="1">
-        <v>46300</v>
+        <v>46133</v>
       </c>
       <c r="H445" s="1">
-        <v>46300</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="446" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A446" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B446" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="C446">
         <v>1</v>
       </c>
       <c r="D446" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E446" t="s">
-        <v>895</v>
+        <v>41</v>
       </c>
       <c r="F446" t="s">
-        <v>896</v>
+        <v>42</v>
       </c>
       <c r="G446" s="1">
-        <v>46300</v>
+        <v>46134</v>
       </c>
       <c r="H446" s="1">
-        <v>46300</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="447" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A447" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B447" t="s">
-        <v>898</v>
+        <v>894</v>
       </c>
       <c r="C447">
         <v>1</v>
       </c>
       <c r="D447" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E447" t="s">
-        <v>221</v>
+        <v>19</v>
       </c>
       <c r="F447" t="s">
-        <v>222</v>
+        <v>20</v>
       </c>
       <c r="G447" s="1">
-        <v>46300</v>
+        <v>46156</v>
       </c>
       <c r="H447" s="1">
-        <v>46300</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="448" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A448" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B448" t="s">
-        <v>899</v>
+        <v>895</v>
       </c>
       <c r="C448">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D448" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E448" t="s">
-        <v>221</v>
+        <v>896</v>
       </c>
       <c r="F448" t="s">
-        <v>222</v>
+        <v>897</v>
       </c>
       <c r="G448" s="1">
-        <v>46300</v>
+        <v>46209</v>
       </c>
       <c r="H448" s="1">
-        <v>46300</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="449" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A449" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B449" t="s">
+        <v>898</v>
+      </c>
+      <c r="C449">
+        <v>1</v>
+      </c>
+      <c r="D449" t="s">
+        <v>6</v>
+      </c>
+      <c r="E449" t="s">
+        <v>899</v>
+      </c>
+      <c r="F449" t="s">
         <v>900</v>
       </c>
-      <c r="C449">
-        <v>1</v>
-      </c>
-      <c r="D449" t="s">
-        <v>154</v>
-      </c>
-      <c r="E449" t="s">
-        <v>886</v>
-      </c>
-      <c r="F449" t="s">
-        <v>887</v>
-      </c>
       <c r="G449" s="1">
-        <v>46300</v>
+        <v>46213</v>
       </c>
       <c r="H449" s="1">
-        <v>46301</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="450" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A450" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B450" t="s">
         <v>901</v>
@@ -15062,105 +15089,105 @@
         <v>1</v>
       </c>
       <c r="D450" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E450" t="s">
-        <v>886</v>
+        <v>902</v>
       </c>
       <c r="F450" t="s">
-        <v>887</v>
+        <v>903</v>
       </c>
       <c r="G450" s="1">
-        <v>46300</v>
+        <v>46213</v>
       </c>
       <c r="H450" s="1">
-        <v>46300</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="451" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A451" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B451" t="s">
+        <v>904</v>
+      </c>
+      <c r="C451">
+        <v>1</v>
+      </c>
+      <c r="D451" t="s">
+        <v>95</v>
+      </c>
+      <c r="E451" t="s">
         <v>902</v>
       </c>
-      <c r="C451">
-        <v>1</v>
-      </c>
-      <c r="D451" t="s">
-        <v>154</v>
-      </c>
-      <c r="E451" t="s">
-        <v>886</v>
-      </c>
       <c r="F451" t="s">
-        <v>887</v>
+        <v>903</v>
       </c>
       <c r="G451" s="1">
-        <v>46300</v>
+        <v>46224</v>
       </c>
       <c r="H451" s="1">
-        <v>46300</v>
+        <v>46224</v>
       </c>
     </row>
     <row r="452" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A452" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B452" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="C452">
         <v>1</v>
       </c>
       <c r="D452" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E452" t="s">
-        <v>895</v>
+        <v>906</v>
       </c>
       <c r="F452" t="s">
-        <v>896</v>
+        <v>907</v>
       </c>
       <c r="G452" s="1">
-        <v>46301</v>
+        <v>46253</v>
       </c>
       <c r="H452" s="1">
-        <v>46301</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="453" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A453" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B453" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
       <c r="C453">
         <v>1</v>
       </c>
       <c r="D453" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E453" t="s">
-        <v>474</v>
+        <v>211</v>
       </c>
       <c r="F453" t="s">
-        <v>475</v>
+        <v>212</v>
       </c>
       <c r="G453" s="1">
-        <v>46302</v>
+        <v>46273</v>
       </c>
       <c r="H453" s="1">
-        <v>46302</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="454" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A454" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B454" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="C454">
         <v>1</v>
@@ -15169,24 +15196,24 @@
         <v>154</v>
       </c>
       <c r="E454" t="s">
-        <v>264</v>
+        <v>510</v>
       </c>
       <c r="F454" t="s">
-        <v>265</v>
+        <v>511</v>
       </c>
       <c r="G454" s="1">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="H454" s="1">
-        <v>46302</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="455" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A455" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B455" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="C455">
         <v>1</v>
@@ -15195,24 +15222,24 @@
         <v>154</v>
       </c>
       <c r="E455" t="s">
-        <v>880</v>
+        <v>911</v>
       </c>
       <c r="F455" t="s">
-        <v>881</v>
+        <v>912</v>
       </c>
       <c r="G455" s="1">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="H455" s="1">
-        <v>46302</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="456" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A456" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="B456" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="C456">
         <v>1</v>
@@ -15221,76 +15248,76 @@
         <v>154</v>
       </c>
       <c r="E456" t="s">
-        <v>264</v>
+        <v>911</v>
       </c>
       <c r="F456" t="s">
-        <v>265</v>
+        <v>912</v>
       </c>
       <c r="G456" s="1">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="H456" s="1">
-        <v>46302</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="457" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A457" t="s">
-        <v>908</v>
+        <v>891</v>
       </c>
       <c r="B457" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="C457">
         <v>1</v>
       </c>
       <c r="D457" t="s">
-        <v>95</v>
+        <v>2</v>
       </c>
       <c r="E457" t="s">
-        <v>910</v>
+        <v>221</v>
       </c>
       <c r="F457" t="s">
-        <v>911</v>
+        <v>222</v>
       </c>
       <c r="G457" s="1">
-        <v>46063</v>
+        <v>46300</v>
       </c>
       <c r="H457" s="1">
-        <v>46064</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="458" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A458" t="s">
-        <v>908</v>
+        <v>891</v>
       </c>
       <c r="B458" t="s">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="C458">
         <v>1</v>
       </c>
       <c r="D458" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E458" t="s">
-        <v>57</v>
+        <v>221</v>
       </c>
       <c r="F458" t="s">
-        <v>58</v>
+        <v>222</v>
       </c>
       <c r="G458" s="1">
-        <v>46113</v>
+        <v>46300</v>
       </c>
       <c r="H458" s="1">
-        <v>46125</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="459" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A459" t="s">
-        <v>908</v>
+        <v>891</v>
       </c>
       <c r="B459" t="s">
-        <v>913</v>
+        <v>916</v>
       </c>
       <c r="C459">
         <v>1</v>
@@ -15299,186 +15326,186 @@
         <v>2</v>
       </c>
       <c r="E459" t="s">
-        <v>57</v>
+        <v>902</v>
       </c>
       <c r="F459" t="s">
-        <v>58</v>
+        <v>903</v>
       </c>
       <c r="G459" s="1">
-        <v>46125</v>
+        <v>46300</v>
       </c>
       <c r="H459" s="1">
-        <v>46125</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="460" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A460" t="s">
-        <v>908</v>
+        <v>891</v>
       </c>
       <c r="B460" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="C460">
         <v>1</v>
       </c>
       <c r="D460" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E460" t="s">
-        <v>57</v>
+        <v>911</v>
       </c>
       <c r="F460" t="s">
-        <v>58</v>
+        <v>912</v>
       </c>
       <c r="G460" s="1">
-        <v>46126</v>
+        <v>46301</v>
       </c>
       <c r="H460" s="1">
-        <v>46126</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="461" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A461" t="s">
-        <v>908</v>
+        <v>891</v>
       </c>
       <c r="B461" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="C461">
         <v>1</v>
       </c>
       <c r="D461" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E461" t="s">
-        <v>57</v>
+        <v>474</v>
       </c>
       <c r="F461" t="s">
-        <v>58</v>
+        <v>475</v>
       </c>
       <c r="G461" s="1">
-        <v>46126</v>
+        <v>46302</v>
       </c>
       <c r="H461" s="1">
-        <v>46126</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="462" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A462" t="s">
-        <v>908</v>
+        <v>891</v>
       </c>
       <c r="B462" t="s">
-        <v>916</v>
+        <v>919</v>
       </c>
       <c r="C462">
         <v>1</v>
       </c>
       <c r="D462" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E462" t="s">
-        <v>57</v>
+        <v>264</v>
       </c>
       <c r="F462" t="s">
-        <v>58</v>
+        <v>265</v>
       </c>
       <c r="G462" s="1">
-        <v>46128</v>
+        <v>46302</v>
       </c>
       <c r="H462" s="1">
-        <v>46128</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="463" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A463" t="s">
-        <v>908</v>
+        <v>891</v>
       </c>
       <c r="B463" t="s">
-        <v>917</v>
+        <v>920</v>
       </c>
       <c r="C463">
         <v>1</v>
       </c>
       <c r="D463" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E463" t="s">
-        <v>57</v>
+        <v>896</v>
       </c>
       <c r="F463" t="s">
-        <v>58</v>
+        <v>897</v>
       </c>
       <c r="G463" s="1">
-        <v>46132</v>
+        <v>46302</v>
       </c>
       <c r="H463" s="1">
-        <v>46132</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="464" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A464" t="s">
-        <v>908</v>
+        <v>891</v>
       </c>
       <c r="B464" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="C464">
         <v>1</v>
       </c>
       <c r="D464" t="s">
-        <v>2</v>
+        <v>154</v>
       </c>
       <c r="E464" t="s">
-        <v>57</v>
+        <v>264</v>
       </c>
       <c r="F464" t="s">
-        <v>58</v>
+        <v>265</v>
       </c>
       <c r="G464" s="1">
-        <v>46161</v>
+        <v>46302</v>
       </c>
       <c r="H464" s="1">
-        <v>46161</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="465" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A465" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B465" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="C465">
         <v>1</v>
       </c>
       <c r="D465" t="s">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="E465" t="s">
-        <v>57</v>
+        <v>924</v>
       </c>
       <c r="F465" t="s">
-        <v>58</v>
+        <v>925</v>
       </c>
       <c r="G465" s="1">
-        <v>46174</v>
+        <v>46063</v>
       </c>
       <c r="H465" s="1">
-        <v>46174</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="466" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A466" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B466" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
       <c r="C466">
         <v>1</v>
       </c>
       <c r="D466" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E466" t="s">
         <v>57</v>
@@ -15487,24 +15514,24 @@
         <v>58</v>
       </c>
       <c r="G466" s="1">
-        <v>46174</v>
+        <v>46113</v>
       </c>
       <c r="H466" s="1">
-        <v>46174</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="467" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A467" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B467" t="s">
-        <v>921</v>
+        <v>927</v>
       </c>
       <c r="C467">
         <v>1</v>
       </c>
       <c r="D467" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E467" t="s">
         <v>57</v>
@@ -15513,24 +15540,24 @@
         <v>58</v>
       </c>
       <c r="G467" s="1">
-        <v>46195</v>
+        <v>46125</v>
       </c>
       <c r="H467" s="1">
-        <v>46252</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="468" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A468" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B468" t="s">
-        <v>922</v>
+        <v>928</v>
       </c>
       <c r="C468">
         <v>1</v>
       </c>
       <c r="D468" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E468" t="s">
         <v>57</v>
@@ -15539,18 +15566,18 @@
         <v>58</v>
       </c>
       <c r="G468" s="1">
-        <v>46210</v>
+        <v>46126</v>
       </c>
       <c r="H468" s="1">
-        <v>46210</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="469" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A469" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B469" t="s">
-        <v>923</v>
+        <v>929</v>
       </c>
       <c r="C469">
         <v>1</v>
@@ -15565,24 +15592,24 @@
         <v>58</v>
       </c>
       <c r="G469" s="1">
-        <v>46213</v>
+        <v>46126</v>
       </c>
       <c r="H469" s="1">
-        <v>46213</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="470" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A470" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B470" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
       <c r="C470">
         <v>1</v>
       </c>
       <c r="D470" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E470" t="s">
         <v>57</v>
@@ -15591,18 +15618,18 @@
         <v>58</v>
       </c>
       <c r="G470" s="1">
-        <v>46218</v>
+        <v>46128</v>
       </c>
       <c r="H470" s="1">
-        <v>46252</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="471" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A471" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B471" t="s">
-        <v>925</v>
+        <v>931</v>
       </c>
       <c r="C471">
         <v>1</v>
@@ -15611,30 +15638,30 @@
         <v>6</v>
       </c>
       <c r="E471" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="F471" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G471" s="1">
-        <v>46226</v>
+        <v>46132</v>
       </c>
       <c r="H471" s="1">
-        <v>46226</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="472" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A472" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B472" t="s">
-        <v>926</v>
+        <v>932</v>
       </c>
       <c r="C472">
         <v>1</v>
       </c>
       <c r="D472" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E472" t="s">
         <v>57</v>
@@ -15643,24 +15670,24 @@
         <v>58</v>
       </c>
       <c r="G472" s="1">
-        <v>46227</v>
+        <v>46161</v>
       </c>
       <c r="H472" s="1">
-        <v>46252</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="473" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A473" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B473" t="s">
-        <v>927</v>
+        <v>933</v>
       </c>
       <c r="C473">
         <v>1</v>
       </c>
       <c r="D473" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E473" t="s">
         <v>57</v>
@@ -15669,24 +15696,24 @@
         <v>58</v>
       </c>
       <c r="G473" s="1">
-        <v>46227</v>
+        <v>46174</v>
       </c>
       <c r="H473" s="1">
-        <v>46252</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="474" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A474" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B474" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="C474">
         <v>1</v>
       </c>
       <c r="D474" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E474" t="s">
         <v>57</v>
@@ -15695,18 +15722,18 @@
         <v>58</v>
       </c>
       <c r="G474" s="1">
-        <v>46227</v>
+        <v>46174</v>
       </c>
       <c r="H474" s="1">
-        <v>46228</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="475" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A475" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B475" t="s">
-        <v>929</v>
+        <v>935</v>
       </c>
       <c r="C475">
         <v>1</v>
@@ -15715,13 +15742,13 @@
         <v>6</v>
       </c>
       <c r="E475" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="F475" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G475" s="1">
-        <v>46230</v>
+        <v>46195</v>
       </c>
       <c r="H475" s="1">
         <v>46252</v>
@@ -15729,10 +15756,10 @@
     </row>
     <row r="476" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A476" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B476" t="s">
-        <v>930</v>
+        <v>936</v>
       </c>
       <c r="C476">
         <v>1</v>
@@ -15747,24 +15774,24 @@
         <v>58</v>
       </c>
       <c r="G476" s="1">
-        <v>46231</v>
+        <v>46210</v>
       </c>
       <c r="H476" s="1">
-        <v>46231</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="477" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A477" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B477" t="s">
-        <v>931</v>
+        <v>937</v>
       </c>
       <c r="C477">
         <v>1</v>
       </c>
       <c r="D477" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E477" t="s">
         <v>57</v>
@@ -15773,24 +15800,24 @@
         <v>58</v>
       </c>
       <c r="G477" s="1">
-        <v>46254</v>
+        <v>46213</v>
       </c>
       <c r="H477" s="1">
-        <v>46254</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="478" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A478" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B478" t="s">
-        <v>932</v>
+        <v>938</v>
       </c>
       <c r="C478">
         <v>1</v>
       </c>
       <c r="D478" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E478" t="s">
         <v>57</v>
@@ -15799,18 +15826,18 @@
         <v>58</v>
       </c>
       <c r="G478" s="1">
-        <v>46255</v>
+        <v>46218</v>
       </c>
       <c r="H478" s="1">
-        <v>46255</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="479" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A479" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B479" t="s">
-        <v>933</v>
+        <v>939</v>
       </c>
       <c r="C479">
         <v>1</v>
@@ -15819,30 +15846,30 @@
         <v>6</v>
       </c>
       <c r="E479" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="F479" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G479" s="1">
-        <v>46260</v>
+        <v>46226</v>
       </c>
       <c r="H479" s="1">
-        <v>46260</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="480" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A480" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B480" t="s">
-        <v>934</v>
+        <v>940</v>
       </c>
       <c r="C480">
         <v>1</v>
       </c>
       <c r="D480" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="E480" t="s">
         <v>57</v>
@@ -15851,18 +15878,18 @@
         <v>58</v>
       </c>
       <c r="G480" s="1">
-        <v>46289</v>
+        <v>46227</v>
       </c>
       <c r="H480" s="1">
-        <v>46289</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="481" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A481" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B481" t="s">
-        <v>935</v>
+        <v>941</v>
       </c>
       <c r="C481">
         <v>1</v>
@@ -15877,24 +15904,24 @@
         <v>58</v>
       </c>
       <c r="G481" s="1">
-        <v>46294</v>
+        <v>46227</v>
       </c>
       <c r="H481" s="1">
-        <v>46294</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="482" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A482" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B482" t="s">
-        <v>936</v>
+        <v>942</v>
       </c>
       <c r="C482">
         <v>1</v>
       </c>
       <c r="D482" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E482" t="s">
         <v>57</v>
@@ -15903,50 +15930,50 @@
         <v>58</v>
       </c>
       <c r="G482" s="1">
-        <v>46302</v>
+        <v>46227</v>
       </c>
       <c r="H482" s="1">
-        <v>46302</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="483" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A483" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B483" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
       <c r="C483">
         <v>1</v>
       </c>
       <c r="D483" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E483" t="s">
-        <v>605</v>
+        <v>77</v>
       </c>
       <c r="F483" t="s">
-        <v>606</v>
+        <v>78</v>
       </c>
       <c r="G483" s="1">
-        <v>46302</v>
+        <v>46230</v>
       </c>
       <c r="H483" s="1">
-        <v>46302</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="484" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A484" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B484" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="C484">
         <v>1</v>
       </c>
       <c r="D484" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E484" t="s">
         <v>57</v>
@@ -15955,24 +15982,24 @@
         <v>58</v>
       </c>
       <c r="G484" s="1">
-        <v>46302</v>
+        <v>46231</v>
       </c>
       <c r="H484" s="1">
-        <v>46302</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="485" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A485" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B485" t="s">
-        <v>939</v>
+        <v>945</v>
       </c>
       <c r="C485">
         <v>1</v>
       </c>
       <c r="D485" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E485" t="s">
         <v>57</v>
@@ -15981,24 +16008,24 @@
         <v>58</v>
       </c>
       <c r="G485" s="1">
-        <v>46302</v>
+        <v>46254</v>
       </c>
       <c r="H485" s="1">
-        <v>46302</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="486" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A486" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B486" t="s">
-        <v>940</v>
+        <v>946</v>
       </c>
       <c r="C486">
         <v>1</v>
       </c>
       <c r="D486" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E486" t="s">
         <v>57</v>
@@ -16007,24 +16034,24 @@
         <v>58</v>
       </c>
       <c r="G486" s="1">
-        <v>46302</v>
+        <v>46255</v>
       </c>
       <c r="H486" s="1">
-        <v>46302</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="487" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A487" t="s">
-        <v>908</v>
+        <v>922</v>
       </c>
       <c r="B487" t="s">
-        <v>941</v>
+        <v>947</v>
       </c>
       <c r="C487">
         <v>1</v>
       </c>
       <c r="D487" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
       <c r="E487" t="s">
         <v>57</v>
@@ -16033,96 +16060,96 @@
         <v>58</v>
       </c>
       <c r="G487" s="1">
-        <v>46302</v>
+        <v>46260</v>
       </c>
       <c r="H487" s="1">
-        <v>46302</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="488" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A488" t="s">
-        <v>942</v>
+        <v>922</v>
       </c>
       <c r="B488" t="s">
-        <v>943</v>
+        <v>948</v>
       </c>
       <c r="C488">
         <v>1</v>
       </c>
       <c r="D488" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E488" t="s">
-        <v>944</v>
+        <v>57</v>
       </c>
       <c r="F488" t="s">
-        <v>945</v>
+        <v>58</v>
       </c>
       <c r="G488" s="1">
-        <v>46157</v>
+        <v>46289</v>
       </c>
       <c r="H488" s="1">
-        <v>46157</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="489" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A489" t="s">
-        <v>942</v>
+        <v>922</v>
       </c>
       <c r="B489" t="s">
-        <v>946</v>
+        <v>949</v>
       </c>
       <c r="C489">
         <v>1</v>
       </c>
       <c r="D489" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E489" t="s">
-        <v>947</v>
+        <v>57</v>
       </c>
       <c r="F489" t="s">
-        <v>948</v>
+        <v>58</v>
       </c>
       <c r="G489" s="1">
-        <v>46168</v>
+        <v>46294</v>
       </c>
       <c r="H489" s="1">
-        <v>46170</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="490" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A490" t="s">
-        <v>942</v>
+        <v>922</v>
       </c>
       <c r="B490" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="C490">
         <v>1</v>
       </c>
       <c r="D490" t="s">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="E490" t="s">
-        <v>944</v>
+        <v>605</v>
       </c>
       <c r="F490" t="s">
-        <v>945</v>
+        <v>606</v>
       </c>
       <c r="G490" s="1">
-        <v>46218</v>
+        <v>46302</v>
       </c>
       <c r="H490" s="1">
-        <v>46218</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="491" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A491" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="B491" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="C491">
         <v>1</v>
@@ -16131,24 +16158,24 @@
         <v>2</v>
       </c>
       <c r="E491" t="s">
-        <v>944</v>
+        <v>953</v>
       </c>
       <c r="F491" t="s">
-        <v>945</v>
+        <v>954</v>
       </c>
       <c r="G491" s="1">
-        <v>46244</v>
+        <v>46157</v>
       </c>
       <c r="H491" s="1">
-        <v>46244</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="492" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A492" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="B492" t="s">
-        <v>951</v>
+        <v>955</v>
       </c>
       <c r="C492">
         <v>1</v>
@@ -16157,24 +16184,24 @@
         <v>2</v>
       </c>
       <c r="E492" t="s">
-        <v>944</v>
+        <v>956</v>
       </c>
       <c r="F492" t="s">
-        <v>945</v>
+        <v>957</v>
       </c>
       <c r="G492" s="1">
-        <v>46247</v>
+        <v>46168</v>
       </c>
       <c r="H492" s="1">
-        <v>46247</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="493" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A493" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="B493" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="C493">
         <v>1</v>
@@ -16189,18 +16216,18 @@
         <v>954</v>
       </c>
       <c r="G493" s="1">
-        <v>46247</v>
+        <v>46218</v>
       </c>
       <c r="H493" s="1">
-        <v>46247</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="494" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A494" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="B494" t="s">
-        <v>955</v>
+        <v>959</v>
       </c>
       <c r="C494">
         <v>1</v>
@@ -16209,24 +16236,24 @@
         <v>2</v>
       </c>
       <c r="E494" t="s">
-        <v>944</v>
+        <v>953</v>
       </c>
       <c r="F494" t="s">
-        <v>945</v>
+        <v>954</v>
       </c>
       <c r="G494" s="1">
-        <v>46255</v>
+        <v>46244</v>
       </c>
       <c r="H494" s="1">
-        <v>46255</v>
+        <v>46244</v>
       </c>
     </row>
     <row r="495" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A495" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="B495" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
       <c r="C495">
         <v>1</v>
@@ -16235,24 +16262,24 @@
         <v>2</v>
       </c>
       <c r="E495" t="s">
-        <v>944</v>
+        <v>953</v>
       </c>
       <c r="F495" t="s">
-        <v>945</v>
+        <v>954</v>
       </c>
       <c r="G495" s="1">
-        <v>46258</v>
+        <v>46247</v>
       </c>
       <c r="H495" s="1">
-        <v>46258</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="496" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A496" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="B496" t="s">
-        <v>957</v>
+        <v>961</v>
       </c>
       <c r="C496">
         <v>1</v>
@@ -16261,67 +16288,145 @@
         <v>2</v>
       </c>
       <c r="E496" t="s">
-        <v>944</v>
+        <v>962</v>
       </c>
       <c r="F496" t="s">
-        <v>945</v>
+        <v>963</v>
       </c>
       <c r="G496" s="1">
-        <v>46262</v>
+        <v>46247</v>
       </c>
       <c r="H496" s="1">
-        <v>46265</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="497" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A497" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="B497" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="C497">
         <v>1</v>
       </c>
       <c r="D497" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E497" t="s">
-        <v>13</v>
+        <v>953</v>
       </c>
       <c r="F497" t="s">
-        <v>14</v>
+        <v>954</v>
       </c>
       <c r="G497" s="1">
-        <v>46281</v>
+        <v>46255</v>
       </c>
       <c r="H497" s="1">
-        <v>46283</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="498" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A498" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="B498" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="C498">
         <v>1</v>
       </c>
       <c r="D498" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="E498" t="s">
-        <v>886</v>
+        <v>953</v>
       </c>
       <c r="F498" t="s">
-        <v>887</v>
+        <v>954</v>
       </c>
       <c r="G498" s="1">
+        <v>46258</v>
+      </c>
+      <c r="H498" s="1">
+        <v>46258</v>
+      </c>
+    </row>
+    <row r="499" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A499" t="s">
+        <v>951</v>
+      </c>
+      <c r="B499" t="s">
+        <v>966</v>
+      </c>
+      <c r="C499">
+        <v>1</v>
+      </c>
+      <c r="D499" t="s">
+        <v>2</v>
+      </c>
+      <c r="E499" t="s">
+        <v>953</v>
+      </c>
+      <c r="F499" t="s">
+        <v>954</v>
+      </c>
+      <c r="G499" s="1">
+        <v>46262</v>
+      </c>
+      <c r="H499" s="1">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="500" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A500" t="s">
+        <v>951</v>
+      </c>
+      <c r="B500" t="s">
+        <v>967</v>
+      </c>
+      <c r="C500">
+        <v>1</v>
+      </c>
+      <c r="D500" t="s">
+        <v>6</v>
+      </c>
+      <c r="E500" t="s">
+        <v>13</v>
+      </c>
+      <c r="F500" t="s">
+        <v>14</v>
+      </c>
+      <c r="G500" s="1">
+        <v>46281</v>
+      </c>
+      <c r="H500" s="1">
+        <v>46283</v>
+      </c>
+    </row>
+    <row r="501" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A501" t="s">
+        <v>951</v>
+      </c>
+      <c r="B501" t="s">
+        <v>968</v>
+      </c>
+      <c r="C501">
+        <v>1</v>
+      </c>
+      <c r="D501" t="s">
+        <v>154</v>
+      </c>
+      <c r="E501" t="s">
+        <v>902</v>
+      </c>
+      <c r="F501" t="s">
+        <v>903</v>
+      </c>
+      <c r="G501" s="1">
         <v>46302</v>
       </c>
-      <c r="H498" s="1">
+      <c r="H501" s="1">
         <v>46302</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 13/10/2026 10:08:09
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B9876D3-807C-4034-A5EC-B42D9524EA09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA011AFE-DE55-43AF-AB39-5E0BC944D65B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{D2CB09EE-8AA8-4E23-BE9E-BB5DBEBD4743}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{683CEE99-5F64-4EA1-9111-00B5A2B7BAD5}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2083" uniqueCount="810">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2223" uniqueCount="860">
   <si>
     <t>0001</t>
   </si>
@@ -2167,6 +2167,162 @@
     <t xml:space="preserve">  217344</t>
   </si>
   <si>
+    <t xml:space="preserve">  217345</t>
+  </si>
+  <si>
+    <t>SC39</t>
+  </si>
+  <si>
+    <t>SURVALMEDA CONSTRUCCIONES S. A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217346</t>
+  </si>
+  <si>
+    <t>DB14</t>
+  </si>
+  <si>
+    <t>DIMA BAÑOS &amp; COCINAS S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217347</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217348</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217349</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217350</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217352</t>
+  </si>
+  <si>
+    <t>JA01</t>
+  </si>
+  <si>
+    <t>JOSE ANACLETO E HIJOS S.A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217353</t>
+  </si>
+  <si>
+    <t>SA40</t>
+  </si>
+  <si>
+    <t>SANICENTRO S.A. SANITARIOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217355</t>
+  </si>
+  <si>
+    <t>MJ21</t>
+  </si>
+  <si>
+    <t>MELCON JUAN CARLOS - SANITARIOS CAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217356</t>
+  </si>
+  <si>
+    <t>HI10</t>
+  </si>
+  <si>
+    <t>HIPERCAÑO S.A.S.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217357</t>
+  </si>
+  <si>
+    <t>DC18</t>
+  </si>
+  <si>
+    <t>DI CARLO SEBASTIAN F -DI CARLO SANIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217358</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217359</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217361</t>
+  </si>
+  <si>
+    <t>TR21</t>
+  </si>
+  <si>
+    <t>TROFA SA - MUNDO CAÑO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217362</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217363</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217364</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217366</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217367</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217368</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217369</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217370</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217371</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217373</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217374</t>
+  </si>
+  <si>
+    <t>TC11</t>
+  </si>
+  <si>
+    <t>TRIPOLI CARLOS L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217375</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>TRIPOLI ARNALDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217376</t>
+  </si>
+  <si>
+    <t>AA05</t>
+  </si>
+  <si>
+    <t>SANITARIOS ALVAREZ SOC. LEY 19550 CAP. I SECCION I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217377</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217379</t>
+  </si>
+  <si>
     <t>0004</t>
   </si>
   <si>
@@ -2281,6 +2437,9 @@
     <t xml:space="preserve">    3025</t>
   </si>
   <si>
+    <t xml:space="preserve">    3026</t>
+  </si>
+  <si>
     <t>4444</t>
   </si>
   <si>
@@ -2365,10 +2524,7 @@
     <t xml:space="preserve">    2644</t>
   </si>
   <si>
-    <t xml:space="preserve">    2760</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2781</t>
+    <t xml:space="preserve">    2783</t>
   </si>
   <si>
     <t>9999</t>
@@ -2420,12 +2576,6 @@
   </si>
   <si>
     <t xml:space="preserve">      98</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     119</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     120</t>
   </si>
   <si>
     <t>Puesto</t>
@@ -2899,34 +3049,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9675168B-BF31-4FEE-B71B-A5364C0BB2C9}">
-  <dimension ref="A1:H416"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{774CBD00-FDE7-40F4-898D-A22423531B4A}">
+  <dimension ref="A1:H444"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>802</v>
+        <v>852</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>803</v>
+        <v>853</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>804</v>
+        <v>854</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>805</v>
+        <v>855</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>806</v>
+        <v>856</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>807</v>
+        <v>857</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>808</v>
+        <v>858</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>809</v>
+        <v>859</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -6242,7 +6392,7 @@
         <v>1</v>
       </c>
       <c r="D129" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E129" t="s">
         <v>37</v>
@@ -7724,7 +7874,7 @@
         <v>1</v>
       </c>
       <c r="D186" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E186" t="s">
         <v>406</v>
@@ -7880,7 +8030,7 @@
         <v>1</v>
       </c>
       <c r="D192" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E192" t="s">
         <v>422</v>
@@ -9596,7 +9746,7 @@
         <v>1</v>
       </c>
       <c r="D258" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E258" t="s">
         <v>544</v>
@@ -9648,7 +9798,7 @@
         <v>1</v>
       </c>
       <c r="D260" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E260" t="s">
         <v>548</v>
@@ -10064,7 +10214,7 @@
         <v>1</v>
       </c>
       <c r="D276" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E276" t="s">
         <v>132</v>
@@ -10220,7 +10370,7 @@
         <v>1</v>
       </c>
       <c r="D282" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E282" t="s">
         <v>590</v>
@@ -10246,7 +10396,7 @@
         <v>1</v>
       </c>
       <c r="D283" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E283" t="s">
         <v>593</v>
@@ -10974,7 +11124,7 @@
         <v>1</v>
       </c>
       <c r="D311" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E311" t="s">
         <v>151</v>
@@ -11208,7 +11358,7 @@
         <v>1</v>
       </c>
       <c r="D320" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E320" t="s">
         <v>654</v>
@@ -11286,7 +11436,7 @@
         <v>1</v>
       </c>
       <c r="D323" t="s">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="E323" t="s">
         <v>654</v>
@@ -12031,62 +12181,62 @@
     </row>
     <row r="352" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
+        <v>0</v>
+      </c>
+      <c r="B352" t="s">
         <v>715</v>
       </c>
-      <c r="B352" t="s">
+      <c r="C352">
+        <v>1</v>
+      </c>
+      <c r="D352" t="s">
+        <v>170</v>
+      </c>
+      <c r="E352" t="s">
         <v>716</v>
       </c>
-      <c r="C352">
-        <v>1</v>
-      </c>
-      <c r="D352" t="s">
-        <v>2</v>
-      </c>
-      <c r="E352" t="s">
-        <v>200</v>
-      </c>
       <c r="F352" t="s">
-        <v>201</v>
+        <v>717</v>
       </c>
       <c r="G352" s="1">
-        <v>46148</v>
+        <v>46304</v>
       </c>
       <c r="H352" s="1">
-        <v>46149</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="353" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A353" t="s">
-        <v>715</v>
+        <v>0</v>
       </c>
       <c r="B353" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C353">
         <v>1</v>
       </c>
       <c r="D353" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E353" t="s">
-        <v>111</v>
+        <v>719</v>
       </c>
       <c r="F353" t="s">
-        <v>112</v>
+        <v>720</v>
       </c>
       <c r="G353" s="1">
-        <v>46268</v>
+        <v>46304</v>
       </c>
       <c r="H353" s="1">
-        <v>46268</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="354" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
-        <v>715</v>
+        <v>0</v>
       </c>
       <c r="B354" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="C354">
         <v>1</v>
@@ -12095,24 +12245,24 @@
         <v>170</v>
       </c>
       <c r="E354" t="s">
-        <v>393</v>
+        <v>719</v>
       </c>
       <c r="F354" t="s">
-        <v>394</v>
+        <v>720</v>
       </c>
       <c r="G354" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="H354" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="355" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A355" t="s">
-        <v>715</v>
+        <v>0</v>
       </c>
       <c r="B355" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="C355">
         <v>1</v>
@@ -12121,21 +12271,21 @@
         <v>170</v>
       </c>
       <c r="E355" t="s">
-        <v>720</v>
+        <v>590</v>
       </c>
       <c r="F355" t="s">
-        <v>721</v>
+        <v>591</v>
       </c>
       <c r="G355" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="H355" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="356" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A356" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B356" t="s">
         <v>723</v>
@@ -12144,24 +12294,24 @@
         <v>1</v>
       </c>
       <c r="D356" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E356" t="s">
-        <v>41</v>
+        <v>214</v>
       </c>
       <c r="F356" t="s">
-        <v>42</v>
+        <v>215</v>
       </c>
       <c r="G356" s="1">
-        <v>46133</v>
+        <v>46304</v>
       </c>
       <c r="H356" s="1">
-        <v>46134</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="357" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A357" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B357" t="s">
         <v>724</v>
@@ -12170,24 +12320,24 @@
         <v>1</v>
       </c>
       <c r="D357" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E357" t="s">
-        <v>41</v>
+        <v>214</v>
       </c>
       <c r="F357" t="s">
-        <v>42</v>
+        <v>215</v>
       </c>
       <c r="G357" s="1">
-        <v>46134</v>
+        <v>46304</v>
       </c>
       <c r="H357" s="1">
-        <v>46134</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="358" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B358" t="s">
         <v>725</v>
@@ -12196,287 +12346,287 @@
         <v>1</v>
       </c>
       <c r="D358" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E358" t="s">
-        <v>19</v>
+        <v>726</v>
       </c>
       <c r="F358" t="s">
-        <v>20</v>
+        <v>727</v>
       </c>
       <c r="G358" s="1">
-        <v>46156</v>
+        <v>46305</v>
       </c>
       <c r="H358" s="1">
-        <v>46156</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="359" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A359" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B359" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="C359">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D359" t="s">
-        <v>95</v>
+        <v>170</v>
       </c>
       <c r="E359" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="F359" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="G359" s="1">
-        <v>46209</v>
+        <v>46305</v>
       </c>
       <c r="H359" s="1">
-        <v>46218</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="360" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A360" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B360" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="C360">
         <v>1</v>
       </c>
       <c r="D360" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E360" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="F360" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="G360" s="1">
-        <v>46213</v>
+        <v>46305</v>
       </c>
       <c r="H360" s="1">
-        <v>46213</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="361" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A361" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B361" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="C361">
         <v>1</v>
       </c>
       <c r="D361" t="s">
-        <v>95</v>
+        <v>170</v>
       </c>
       <c r="E361" t="s">
-        <v>625</v>
+        <v>735</v>
       </c>
       <c r="F361" t="s">
-        <v>626</v>
+        <v>736</v>
       </c>
       <c r="G361" s="1">
-        <v>46213</v>
+        <v>46305</v>
       </c>
       <c r="H361" s="1">
-        <v>46216</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="362" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A362" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B362" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="C362">
         <v>1</v>
       </c>
       <c r="D362" t="s">
-        <v>95</v>
+        <v>170</v>
       </c>
       <c r="E362" t="s">
-        <v>625</v>
+        <v>738</v>
       </c>
       <c r="F362" t="s">
-        <v>626</v>
+        <v>739</v>
       </c>
       <c r="G362" s="1">
-        <v>46224</v>
+        <v>46305</v>
       </c>
       <c r="H362" s="1">
-        <v>46224</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="363" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A363" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B363" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="C363">
         <v>1</v>
       </c>
       <c r="D363" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E363" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="F363" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="G363" s="1">
-        <v>46253</v>
+        <v>46305</v>
       </c>
       <c r="H363" s="1">
-        <v>46253</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="364" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A364" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B364" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="C364">
         <v>1</v>
       </c>
       <c r="D364" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E364" t="s">
-        <v>211</v>
+        <v>719</v>
       </c>
       <c r="F364" t="s">
-        <v>212</v>
+        <v>720</v>
       </c>
       <c r="G364" s="1">
-        <v>46273</v>
+        <v>46307</v>
       </c>
       <c r="H364" s="1">
-        <v>46274</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="365" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A365" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B365" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="C365">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D365" t="s">
         <v>170</v>
       </c>
       <c r="E365" t="s">
-        <v>739</v>
+        <v>376</v>
       </c>
       <c r="F365" t="s">
-        <v>740</v>
+        <v>377</v>
       </c>
       <c r="G365" s="1">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="H365" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="366" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A366" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B366" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="C366">
         <v>1</v>
       </c>
       <c r="D366" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E366" t="s">
-        <v>221</v>
+        <v>744</v>
       </c>
       <c r="F366" t="s">
-        <v>222</v>
+        <v>745</v>
       </c>
       <c r="G366" s="1">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="H366" s="1">
-        <v>46300</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="367" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A367" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B367" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="C367">
         <v>1</v>
       </c>
       <c r="D367" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E367" t="s">
-        <v>625</v>
+        <v>744</v>
       </c>
       <c r="F367" t="s">
-        <v>626</v>
+        <v>745</v>
       </c>
       <c r="G367" s="1">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="H367" s="1">
-        <v>46301</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="368" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A368" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B368" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="C368">
         <v>1</v>
       </c>
       <c r="D368" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E368" t="s">
-        <v>347</v>
+        <v>596</v>
       </c>
       <c r="F368" t="s">
-        <v>348</v>
+        <v>597</v>
       </c>
       <c r="G368" s="1">
-        <v>46302</v>
+        <v>46307</v>
       </c>
       <c r="H368" s="1">
-        <v>46302</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="369" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A369" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B369" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="C369">
         <v>1</v>
@@ -12485,24 +12635,24 @@
         <v>170</v>
       </c>
       <c r="E369" t="s">
+        <v>726</v>
+      </c>
+      <c r="F369" t="s">
         <v>727</v>
       </c>
-      <c r="F369" t="s">
-        <v>728</v>
-      </c>
       <c r="G369" s="1">
-        <v>46302</v>
+        <v>46307</v>
       </c>
       <c r="H369" s="1">
-        <v>46302</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="370" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A370" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B370" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="C370">
         <v>1</v>
@@ -12511,50 +12661,50 @@
         <v>170</v>
       </c>
       <c r="E370" t="s">
-        <v>513</v>
+        <v>373</v>
       </c>
       <c r="F370" t="s">
-        <v>514</v>
+        <v>374</v>
       </c>
       <c r="G370" s="1">
-        <v>46303</v>
+        <v>46307</v>
       </c>
       <c r="H370" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="371" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A371" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B371" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="C371">
         <v>1</v>
       </c>
       <c r="D371" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E371" t="s">
-        <v>537</v>
+        <v>234</v>
       </c>
       <c r="F371" t="s">
-        <v>538</v>
+        <v>235</v>
       </c>
       <c r="G371" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="H371" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="372" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A372" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B372" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="C372">
         <v>1</v>
@@ -12563,24 +12713,24 @@
         <v>170</v>
       </c>
       <c r="E372" t="s">
-        <v>537</v>
+        <v>204</v>
       </c>
       <c r="F372" t="s">
-        <v>538</v>
+        <v>205</v>
       </c>
       <c r="G372" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="H372" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="373" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A373" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B373" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="C373">
         <v>1</v>
@@ -12589,24 +12739,24 @@
         <v>170</v>
       </c>
       <c r="E373" t="s">
-        <v>537</v>
+        <v>92</v>
       </c>
       <c r="F373" t="s">
-        <v>538</v>
+        <v>93</v>
       </c>
       <c r="G373" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="H373" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="374" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A374" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B374" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="C374">
         <v>1</v>
@@ -12615,24 +12765,24 @@
         <v>170</v>
       </c>
       <c r="E374" t="s">
-        <v>132</v>
+        <v>92</v>
       </c>
       <c r="F374" t="s">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="G374" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="H374" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="375" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A375" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B375" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="C375">
         <v>1</v>
@@ -12641,24 +12791,24 @@
         <v>170</v>
       </c>
       <c r="E375" t="s">
-        <v>625</v>
+        <v>16</v>
       </c>
       <c r="F375" t="s">
-        <v>626</v>
+        <v>17</v>
       </c>
       <c r="G375" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="H375" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="376" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A376" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B376" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="C376">
         <v>1</v>
@@ -12667,24 +12817,24 @@
         <v>170</v>
       </c>
       <c r="E376" t="s">
-        <v>727</v>
+        <v>487</v>
       </c>
       <c r="F376" t="s">
-        <v>728</v>
+        <v>488</v>
       </c>
       <c r="G376" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="H376" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="377" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A377" t="s">
-        <v>722</v>
+        <v>0</v>
       </c>
       <c r="B377" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="C377">
         <v>1</v>
@@ -12693,128 +12843,128 @@
         <v>170</v>
       </c>
       <c r="E377" t="s">
-        <v>657</v>
+        <v>757</v>
       </c>
       <c r="F377" t="s">
-        <v>658</v>
+        <v>758</v>
       </c>
       <c r="G377" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="H377" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="378" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A378" t="s">
-        <v>753</v>
+        <v>0</v>
       </c>
       <c r="B378" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="C378">
         <v>1</v>
       </c>
       <c r="D378" t="s">
-        <v>95</v>
+        <v>170</v>
       </c>
       <c r="E378" t="s">
-        <v>755</v>
+        <v>760</v>
       </c>
       <c r="F378" t="s">
-        <v>756</v>
+        <v>761</v>
       </c>
       <c r="G378" s="1">
-        <v>46063</v>
+        <v>46308</v>
       </c>
       <c r="H378" s="1">
-        <v>46064</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="379" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A379" t="s">
-        <v>753</v>
+        <v>0</v>
       </c>
       <c r="B379" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
       <c r="C379">
         <v>1</v>
       </c>
       <c r="D379" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E379" t="s">
-        <v>57</v>
+        <v>763</v>
       </c>
       <c r="F379" t="s">
-        <v>58</v>
+        <v>764</v>
       </c>
       <c r="G379" s="1">
-        <v>46113</v>
+        <v>46308</v>
       </c>
       <c r="H379" s="1">
-        <v>46125</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="380" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A380" t="s">
-        <v>753</v>
+        <v>0</v>
       </c>
       <c r="B380" t="s">
-        <v>758</v>
+        <v>765</v>
       </c>
       <c r="C380">
         <v>1</v>
       </c>
       <c r="D380" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E380" t="s">
-        <v>57</v>
+        <v>224</v>
       </c>
       <c r="F380" t="s">
-        <v>58</v>
+        <v>225</v>
       </c>
       <c r="G380" s="1">
-        <v>46125</v>
+        <v>46308</v>
       </c>
       <c r="H380" s="1">
-        <v>46125</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="381" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A381" t="s">
-        <v>753</v>
+        <v>0</v>
       </c>
       <c r="B381" t="s">
-        <v>759</v>
+        <v>766</v>
       </c>
       <c r="C381">
         <v>1</v>
       </c>
       <c r="D381" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E381" t="s">
-        <v>57</v>
+        <v>431</v>
       </c>
       <c r="F381" t="s">
-        <v>58</v>
+        <v>432</v>
       </c>
       <c r="G381" s="1">
-        <v>46126</v>
+        <v>46308</v>
       </c>
       <c r="H381" s="1">
-        <v>46126</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="382" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A382" t="s">
-        <v>753</v>
+        <v>767</v>
       </c>
       <c r="B382" t="s">
-        <v>760</v>
+        <v>768</v>
       </c>
       <c r="C382">
         <v>1</v>
@@ -12823,24 +12973,24 @@
         <v>2</v>
       </c>
       <c r="E382" t="s">
-        <v>57</v>
+        <v>200</v>
       </c>
       <c r="F382" t="s">
-        <v>58</v>
+        <v>201</v>
       </c>
       <c r="G382" s="1">
-        <v>46126</v>
+        <v>46148</v>
       </c>
       <c r="H382" s="1">
-        <v>46126</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="383" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A383" t="s">
-        <v>753</v>
+        <v>767</v>
       </c>
       <c r="B383" t="s">
-        <v>761</v>
+        <v>769</v>
       </c>
       <c r="C383">
         <v>1</v>
@@ -12849,128 +12999,128 @@
         <v>2</v>
       </c>
       <c r="E383" t="s">
-        <v>57</v>
+        <v>111</v>
       </c>
       <c r="F383" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="G383" s="1">
-        <v>46128</v>
+        <v>46268</v>
       </c>
       <c r="H383" s="1">
-        <v>46128</v>
+        <v>46268</v>
       </c>
     </row>
     <row r="384" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A384" t="s">
-        <v>753</v>
+        <v>767</v>
       </c>
       <c r="B384" t="s">
-        <v>762</v>
+        <v>770</v>
       </c>
       <c r="C384">
         <v>1</v>
       </c>
       <c r="D384" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E384" t="s">
-        <v>57</v>
+        <v>393</v>
       </c>
       <c r="F384" t="s">
-        <v>58</v>
+        <v>394</v>
       </c>
       <c r="G384" s="1">
-        <v>46132</v>
+        <v>46303</v>
       </c>
       <c r="H384" s="1">
-        <v>46132</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="385" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A385" t="s">
-        <v>753</v>
+        <v>767</v>
       </c>
       <c r="B385" t="s">
-        <v>763</v>
+        <v>771</v>
       </c>
       <c r="C385">
         <v>1</v>
       </c>
       <c r="D385" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E385" t="s">
-        <v>57</v>
+        <v>772</v>
       </c>
       <c r="F385" t="s">
-        <v>58</v>
+        <v>773</v>
       </c>
       <c r="G385" s="1">
-        <v>46161</v>
+        <v>46303</v>
       </c>
       <c r="H385" s="1">
-        <v>46161</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="386" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A386" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B386" t="s">
-        <v>764</v>
+        <v>775</v>
       </c>
       <c r="C386">
         <v>1</v>
       </c>
       <c r="D386" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E386" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="F386" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="G386" s="1">
-        <v>46174</v>
+        <v>46133</v>
       </c>
       <c r="H386" s="1">
-        <v>46174</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="387" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A387" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B387" t="s">
-        <v>765</v>
+        <v>776</v>
       </c>
       <c r="C387">
         <v>1</v>
       </c>
       <c r="D387" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E387" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="F387" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="G387" s="1">
-        <v>46174</v>
+        <v>46134</v>
       </c>
       <c r="H387" s="1">
-        <v>46174</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="388" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A388" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B388" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
       <c r="C388">
         <v>1</v>
@@ -12979,62 +13129,62 @@
         <v>6</v>
       </c>
       <c r="E388" t="s">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="F388" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="G388" s="1">
-        <v>46195</v>
+        <v>46156</v>
       </c>
       <c r="H388" s="1">
-        <v>46252</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="389" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A389" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B389" t="s">
-        <v>767</v>
+        <v>778</v>
       </c>
       <c r="C389">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D389" t="s">
-        <v>6</v>
+        <v>95</v>
       </c>
       <c r="E389" t="s">
-        <v>57</v>
+        <v>779</v>
       </c>
       <c r="F389" t="s">
-        <v>58</v>
+        <v>780</v>
       </c>
       <c r="G389" s="1">
-        <v>46210</v>
+        <v>46209</v>
       </c>
       <c r="H389" s="1">
-        <v>46210</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="390" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A390" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B390" t="s">
-        <v>768</v>
+        <v>781</v>
       </c>
       <c r="C390">
         <v>1</v>
       </c>
       <c r="D390" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E390" t="s">
-        <v>57</v>
+        <v>782</v>
       </c>
       <c r="F390" t="s">
-        <v>58</v>
+        <v>783</v>
       </c>
       <c r="G390" s="1">
         <v>46213</v>
@@ -13045,270 +13195,270 @@
     </row>
     <row r="391" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A391" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B391" t="s">
-        <v>769</v>
+        <v>784</v>
       </c>
       <c r="C391">
         <v>1</v>
       </c>
       <c r="D391" t="s">
-        <v>6</v>
+        <v>95</v>
       </c>
       <c r="E391" t="s">
-        <v>57</v>
+        <v>625</v>
       </c>
       <c r="F391" t="s">
-        <v>58</v>
+        <v>626</v>
       </c>
       <c r="G391" s="1">
-        <v>46218</v>
+        <v>46213</v>
       </c>
       <c r="H391" s="1">
-        <v>46252</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="392" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A392" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B392" t="s">
-        <v>770</v>
+        <v>785</v>
       </c>
       <c r="C392">
         <v>1</v>
       </c>
       <c r="D392" t="s">
-        <v>6</v>
+        <v>95</v>
       </c>
       <c r="E392" t="s">
-        <v>77</v>
+        <v>625</v>
       </c>
       <c r="F392" t="s">
-        <v>78</v>
+        <v>626</v>
       </c>
       <c r="G392" s="1">
-        <v>46226</v>
+        <v>46224</v>
       </c>
       <c r="H392" s="1">
-        <v>46226</v>
+        <v>46224</v>
       </c>
     </row>
     <row r="393" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A393" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B393" t="s">
-        <v>771</v>
+        <v>786</v>
       </c>
       <c r="C393">
         <v>1</v>
       </c>
       <c r="D393" t="s">
-        <v>170</v>
+        <v>6</v>
       </c>
       <c r="E393" t="s">
-        <v>57</v>
+        <v>787</v>
       </c>
       <c r="F393" t="s">
-        <v>58</v>
+        <v>788</v>
       </c>
       <c r="G393" s="1">
-        <v>46227</v>
+        <v>46253</v>
       </c>
       <c r="H393" s="1">
-        <v>46252</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="394" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A394" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B394" t="s">
-        <v>772</v>
+        <v>789</v>
       </c>
       <c r="C394">
         <v>1</v>
       </c>
       <c r="D394" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E394" t="s">
-        <v>57</v>
+        <v>211</v>
       </c>
       <c r="F394" t="s">
-        <v>58</v>
+        <v>212</v>
       </c>
       <c r="G394" s="1">
-        <v>46227</v>
+        <v>46273</v>
       </c>
       <c r="H394" s="1">
-        <v>46252</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="395" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A395" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B395" t="s">
-        <v>773</v>
+        <v>790</v>
       </c>
       <c r="C395">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D395" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E395" t="s">
-        <v>57</v>
+        <v>791</v>
       </c>
       <c r="F395" t="s">
-        <v>58</v>
+        <v>792</v>
       </c>
       <c r="G395" s="1">
-        <v>46227</v>
+        <v>46300</v>
       </c>
       <c r="H395" s="1">
-        <v>46228</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="396" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A396" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B396" t="s">
-        <v>774</v>
+        <v>793</v>
       </c>
       <c r="C396">
         <v>1</v>
       </c>
       <c r="D396" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E396" t="s">
-        <v>77</v>
+        <v>221</v>
       </c>
       <c r="F396" t="s">
-        <v>78</v>
+        <v>222</v>
       </c>
       <c r="G396" s="1">
-        <v>46230</v>
+        <v>46300</v>
       </c>
       <c r="H396" s="1">
-        <v>46252</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="397" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A397" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B397" t="s">
-        <v>775</v>
+        <v>794</v>
       </c>
       <c r="C397">
         <v>1</v>
       </c>
       <c r="D397" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E397" t="s">
-        <v>57</v>
+        <v>625</v>
       </c>
       <c r="F397" t="s">
-        <v>58</v>
+        <v>626</v>
       </c>
       <c r="G397" s="1">
-        <v>46231</v>
+        <v>46300</v>
       </c>
       <c r="H397" s="1">
-        <v>46231</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="398" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A398" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B398" t="s">
-        <v>776</v>
+        <v>795</v>
       </c>
       <c r="C398">
         <v>1</v>
       </c>
       <c r="D398" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E398" t="s">
-        <v>57</v>
+        <v>347</v>
       </c>
       <c r="F398" t="s">
-        <v>58</v>
+        <v>348</v>
       </c>
       <c r="G398" s="1">
-        <v>46254</v>
+        <v>46302</v>
       </c>
       <c r="H398" s="1">
-        <v>46254</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="399" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A399" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B399" t="s">
-        <v>777</v>
+        <v>796</v>
       </c>
       <c r="C399">
         <v>1</v>
       </c>
       <c r="D399" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E399" t="s">
-        <v>57</v>
+        <v>779</v>
       </c>
       <c r="F399" t="s">
-        <v>58</v>
+        <v>780</v>
       </c>
       <c r="G399" s="1">
-        <v>46255</v>
+        <v>46302</v>
       </c>
       <c r="H399" s="1">
-        <v>46255</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="400" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A400" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B400" t="s">
-        <v>778</v>
+        <v>797</v>
       </c>
       <c r="C400">
         <v>1</v>
       </c>
       <c r="D400" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E400" t="s">
-        <v>57</v>
+        <v>513</v>
       </c>
       <c r="F400" t="s">
-        <v>58</v>
+        <v>514</v>
       </c>
       <c r="G400" s="1">
-        <v>46260</v>
+        <v>46303</v>
       </c>
       <c r="H400" s="1">
-        <v>46260</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="401" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A401" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B401" t="s">
-        <v>779</v>
+        <v>798</v>
       </c>
       <c r="C401">
         <v>1</v>
@@ -13317,76 +13467,76 @@
         <v>6</v>
       </c>
       <c r="E401" t="s">
-        <v>57</v>
+        <v>537</v>
       </c>
       <c r="F401" t="s">
-        <v>58</v>
+        <v>538</v>
       </c>
       <c r="G401" s="1">
-        <v>46289</v>
+        <v>46303</v>
       </c>
       <c r="H401" s="1">
-        <v>46289</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="402" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A402" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B402" t="s">
-        <v>780</v>
+        <v>799</v>
       </c>
       <c r="C402">
         <v>1</v>
       </c>
       <c r="D402" t="s">
-        <v>6</v>
+        <v>170</v>
       </c>
       <c r="E402" t="s">
-        <v>57</v>
+        <v>537</v>
       </c>
       <c r="F402" t="s">
-        <v>58</v>
+        <v>538</v>
       </c>
       <c r="G402" s="1">
-        <v>46294</v>
+        <v>46303</v>
       </c>
       <c r="H402" s="1">
-        <v>46294</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="403" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A403" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B403" t="s">
-        <v>781</v>
+        <v>800</v>
       </c>
       <c r="C403">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D403" t="s">
-        <v>95</v>
+        <v>170</v>
       </c>
       <c r="E403" t="s">
-        <v>57</v>
+        <v>537</v>
       </c>
       <c r="F403" t="s">
-        <v>58</v>
+        <v>538</v>
       </c>
       <c r="G403" s="1">
         <v>46303</v>
       </c>
       <c r="H403" s="1">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="404" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A404" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="B404" t="s">
-        <v>782</v>
+        <v>801</v>
       </c>
       <c r="C404">
         <v>1</v>
@@ -13395,180 +13545,180 @@
         <v>170</v>
       </c>
       <c r="E404" t="s">
-        <v>57</v>
+        <v>132</v>
       </c>
       <c r="F404" t="s">
-        <v>58</v>
+        <v>133</v>
       </c>
       <c r="G404" s="1">
-        <v>46308</v>
+        <v>46303</v>
       </c>
       <c r="H404" s="1">
-        <v>46308</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="405" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A405" t="s">
-        <v>783</v>
+        <v>774</v>
       </c>
       <c r="B405" t="s">
-        <v>784</v>
+        <v>802</v>
       </c>
       <c r="C405">
         <v>1</v>
       </c>
       <c r="D405" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E405" t="s">
-        <v>785</v>
+        <v>625</v>
       </c>
       <c r="F405" t="s">
-        <v>786</v>
+        <v>626</v>
       </c>
       <c r="G405" s="1">
-        <v>46157</v>
+        <v>46304</v>
       </c>
       <c r="H405" s="1">
-        <v>46157</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="406" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A406" t="s">
-        <v>783</v>
+        <v>774</v>
       </c>
       <c r="B406" t="s">
-        <v>787</v>
+        <v>803</v>
       </c>
       <c r="C406">
         <v>1</v>
       </c>
       <c r="D406" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E406" t="s">
-        <v>788</v>
+        <v>779</v>
       </c>
       <c r="F406" t="s">
-        <v>789</v>
+        <v>780</v>
       </c>
       <c r="G406" s="1">
-        <v>46168</v>
+        <v>46304</v>
       </c>
       <c r="H406" s="1">
-        <v>46170</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="407" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A407" t="s">
-        <v>783</v>
+        <v>774</v>
       </c>
       <c r="B407" t="s">
-        <v>790</v>
+        <v>804</v>
       </c>
       <c r="C407">
         <v>1</v>
       </c>
       <c r="D407" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E407" t="s">
-        <v>785</v>
+        <v>657</v>
       </c>
       <c r="F407" t="s">
-        <v>786</v>
+        <v>658</v>
       </c>
       <c r="G407" s="1">
-        <v>46218</v>
+        <v>46304</v>
       </c>
       <c r="H407" s="1">
-        <v>46218</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="408" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A408" t="s">
-        <v>783</v>
+        <v>774</v>
       </c>
       <c r="B408" t="s">
-        <v>791</v>
+        <v>805</v>
       </c>
       <c r="C408">
         <v>1</v>
       </c>
       <c r="D408" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="E408" t="s">
-        <v>785</v>
+        <v>83</v>
       </c>
       <c r="F408" t="s">
-        <v>786</v>
+        <v>84</v>
       </c>
       <c r="G408" s="1">
-        <v>46244</v>
+        <v>46308</v>
       </c>
       <c r="H408" s="1">
-        <v>46244</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="409" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A409" t="s">
-        <v>783</v>
+        <v>806</v>
       </c>
       <c r="B409" t="s">
-        <v>792</v>
+        <v>807</v>
       </c>
       <c r="C409">
         <v>1</v>
       </c>
       <c r="D409" t="s">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="E409" t="s">
-        <v>785</v>
+        <v>808</v>
       </c>
       <c r="F409" t="s">
-        <v>786</v>
+        <v>809</v>
       </c>
       <c r="G409" s="1">
-        <v>46247</v>
+        <v>46063</v>
       </c>
       <c r="H409" s="1">
-        <v>46247</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="410" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A410" t="s">
-        <v>783</v>
+        <v>806</v>
       </c>
       <c r="B410" t="s">
-        <v>793</v>
+        <v>810</v>
       </c>
       <c r="C410">
         <v>1</v>
       </c>
       <c r="D410" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E410" t="s">
-        <v>794</v>
+        <v>57</v>
       </c>
       <c r="F410" t="s">
-        <v>795</v>
+        <v>58</v>
       </c>
       <c r="G410" s="1">
-        <v>46247</v>
+        <v>46113</v>
       </c>
       <c r="H410" s="1">
-        <v>46247</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="411" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A411" t="s">
-        <v>783</v>
+        <v>806</v>
       </c>
       <c r="B411" t="s">
-        <v>796</v>
+        <v>811</v>
       </c>
       <c r="C411">
         <v>1</v>
@@ -13577,24 +13727,24 @@
         <v>2</v>
       </c>
       <c r="E411" t="s">
-        <v>785</v>
+        <v>57</v>
       </c>
       <c r="F411" t="s">
-        <v>786</v>
+        <v>58</v>
       </c>
       <c r="G411" s="1">
-        <v>46255</v>
+        <v>46125</v>
       </c>
       <c r="H411" s="1">
-        <v>46255</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="412" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A412" t="s">
-        <v>783</v>
+        <v>806</v>
       </c>
       <c r="B412" t="s">
-        <v>797</v>
+        <v>812</v>
       </c>
       <c r="C412">
         <v>1</v>
@@ -13603,24 +13753,24 @@
         <v>2</v>
       </c>
       <c r="E412" t="s">
-        <v>785</v>
+        <v>57</v>
       </c>
       <c r="F412" t="s">
-        <v>786</v>
+        <v>58</v>
       </c>
       <c r="G412" s="1">
-        <v>46258</v>
+        <v>46126</v>
       </c>
       <c r="H412" s="1">
-        <v>46258</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="413" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A413" t="s">
-        <v>783</v>
+        <v>806</v>
       </c>
       <c r="B413" t="s">
-        <v>798</v>
+        <v>813</v>
       </c>
       <c r="C413">
         <v>1</v>
@@ -13629,56 +13779,56 @@
         <v>2</v>
       </c>
       <c r="E413" t="s">
-        <v>785</v>
+        <v>57</v>
       </c>
       <c r="F413" t="s">
-        <v>786</v>
+        <v>58</v>
       </c>
       <c r="G413" s="1">
-        <v>46262</v>
+        <v>46126</v>
       </c>
       <c r="H413" s="1">
-        <v>46265</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="414" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A414" t="s">
-        <v>783</v>
+        <v>806</v>
       </c>
       <c r="B414" t="s">
-        <v>799</v>
+        <v>814</v>
       </c>
       <c r="C414">
         <v>1</v>
       </c>
       <c r="D414" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E414" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="F414" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="G414" s="1">
-        <v>46281</v>
+        <v>46128</v>
       </c>
       <c r="H414" s="1">
-        <v>46283</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="415" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A415" t="s">
-        <v>783</v>
+        <v>806</v>
       </c>
       <c r="B415" t="s">
-        <v>800</v>
+        <v>815</v>
       </c>
       <c r="C415">
         <v>1</v>
       </c>
       <c r="D415" t="s">
-        <v>95</v>
+        <v>6</v>
       </c>
       <c r="E415" t="s">
         <v>57</v>
@@ -13687,24 +13837,24 @@
         <v>58</v>
       </c>
       <c r="G415" s="1">
-        <v>46304</v>
+        <v>46132</v>
       </c>
       <c r="H415" s="1">
-        <v>46304</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="416" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A416" t="s">
-        <v>783</v>
+        <v>806</v>
       </c>
       <c r="B416" t="s">
-        <v>801</v>
+        <v>816</v>
       </c>
       <c r="C416">
         <v>1</v>
       </c>
       <c r="D416" t="s">
-        <v>95</v>
+        <v>2</v>
       </c>
       <c r="E416" t="s">
         <v>57</v>
@@ -13713,10 +13863,738 @@
         <v>58</v>
       </c>
       <c r="G416" s="1">
-        <v>46304</v>
+        <v>46161</v>
       </c>
       <c r="H416" s="1">
-        <v>46304</v>
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="417" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A417" t="s">
+        <v>806</v>
+      </c>
+      <c r="B417" t="s">
+        <v>817</v>
+      </c>
+      <c r="C417">
+        <v>1</v>
+      </c>
+      <c r="D417" t="s">
+        <v>2</v>
+      </c>
+      <c r="E417" t="s">
+        <v>57</v>
+      </c>
+      <c r="F417" t="s">
+        <v>58</v>
+      </c>
+      <c r="G417" s="1">
+        <v>46174</v>
+      </c>
+      <c r="H417" s="1">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="418" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A418" t="s">
+        <v>806</v>
+      </c>
+      <c r="B418" t="s">
+        <v>818</v>
+      </c>
+      <c r="C418">
+        <v>1</v>
+      </c>
+      <c r="D418" t="s">
+        <v>2</v>
+      </c>
+      <c r="E418" t="s">
+        <v>57</v>
+      </c>
+      <c r="F418" t="s">
+        <v>58</v>
+      </c>
+      <c r="G418" s="1">
+        <v>46174</v>
+      </c>
+      <c r="H418" s="1">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="419" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A419" t="s">
+        <v>806</v>
+      </c>
+      <c r="B419" t="s">
+        <v>819</v>
+      </c>
+      <c r="C419">
+        <v>1</v>
+      </c>
+      <c r="D419" t="s">
+        <v>6</v>
+      </c>
+      <c r="E419" t="s">
+        <v>57</v>
+      </c>
+      <c r="F419" t="s">
+        <v>58</v>
+      </c>
+      <c r="G419" s="1">
+        <v>46195</v>
+      </c>
+      <c r="H419" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="420" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A420" t="s">
+        <v>806</v>
+      </c>
+      <c r="B420" t="s">
+        <v>820</v>
+      </c>
+      <c r="C420">
+        <v>1</v>
+      </c>
+      <c r="D420" t="s">
+        <v>6</v>
+      </c>
+      <c r="E420" t="s">
+        <v>57</v>
+      </c>
+      <c r="F420" t="s">
+        <v>58</v>
+      </c>
+      <c r="G420" s="1">
+        <v>46210</v>
+      </c>
+      <c r="H420" s="1">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="421" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A421" t="s">
+        <v>806</v>
+      </c>
+      <c r="B421" t="s">
+        <v>821</v>
+      </c>
+      <c r="C421">
+        <v>1</v>
+      </c>
+      <c r="D421" t="s">
+        <v>2</v>
+      </c>
+      <c r="E421" t="s">
+        <v>57</v>
+      </c>
+      <c r="F421" t="s">
+        <v>58</v>
+      </c>
+      <c r="G421" s="1">
+        <v>46213</v>
+      </c>
+      <c r="H421" s="1">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="422" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A422" t="s">
+        <v>806</v>
+      </c>
+      <c r="B422" t="s">
+        <v>822</v>
+      </c>
+      <c r="C422">
+        <v>1</v>
+      </c>
+      <c r="D422" t="s">
+        <v>6</v>
+      </c>
+      <c r="E422" t="s">
+        <v>57</v>
+      </c>
+      <c r="F422" t="s">
+        <v>58</v>
+      </c>
+      <c r="G422" s="1">
+        <v>46218</v>
+      </c>
+      <c r="H422" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="423" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A423" t="s">
+        <v>806</v>
+      </c>
+      <c r="B423" t="s">
+        <v>823</v>
+      </c>
+      <c r="C423">
+        <v>1</v>
+      </c>
+      <c r="D423" t="s">
+        <v>6</v>
+      </c>
+      <c r="E423" t="s">
+        <v>77</v>
+      </c>
+      <c r="F423" t="s">
+        <v>78</v>
+      </c>
+      <c r="G423" s="1">
+        <v>46226</v>
+      </c>
+      <c r="H423" s="1">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="424" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A424" t="s">
+        <v>806</v>
+      </c>
+      <c r="B424" t="s">
+        <v>824</v>
+      </c>
+      <c r="C424">
+        <v>1</v>
+      </c>
+      <c r="D424" t="s">
+        <v>170</v>
+      </c>
+      <c r="E424" t="s">
+        <v>57</v>
+      </c>
+      <c r="F424" t="s">
+        <v>58</v>
+      </c>
+      <c r="G424" s="1">
+        <v>46227</v>
+      </c>
+      <c r="H424" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="425" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A425" t="s">
+        <v>806</v>
+      </c>
+      <c r="B425" t="s">
+        <v>825</v>
+      </c>
+      <c r="C425">
+        <v>1</v>
+      </c>
+      <c r="D425" t="s">
+        <v>6</v>
+      </c>
+      <c r="E425" t="s">
+        <v>57</v>
+      </c>
+      <c r="F425" t="s">
+        <v>58</v>
+      </c>
+      <c r="G425" s="1">
+        <v>46227</v>
+      </c>
+      <c r="H425" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="426" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A426" t="s">
+        <v>806</v>
+      </c>
+      <c r="B426" t="s">
+        <v>826</v>
+      </c>
+      <c r="C426">
+        <v>1</v>
+      </c>
+      <c r="D426" t="s">
+        <v>6</v>
+      </c>
+      <c r="E426" t="s">
+        <v>57</v>
+      </c>
+      <c r="F426" t="s">
+        <v>58</v>
+      </c>
+      <c r="G426" s="1">
+        <v>46227</v>
+      </c>
+      <c r="H426" s="1">
+        <v>46228</v>
+      </c>
+    </row>
+    <row r="427" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A427" t="s">
+        <v>806</v>
+      </c>
+      <c r="B427" t="s">
+        <v>827</v>
+      </c>
+      <c r="C427">
+        <v>1</v>
+      </c>
+      <c r="D427" t="s">
+        <v>6</v>
+      </c>
+      <c r="E427" t="s">
+        <v>77</v>
+      </c>
+      <c r="F427" t="s">
+        <v>78</v>
+      </c>
+      <c r="G427" s="1">
+        <v>46230</v>
+      </c>
+      <c r="H427" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="428" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A428" t="s">
+        <v>806</v>
+      </c>
+      <c r="B428" t="s">
+        <v>828</v>
+      </c>
+      <c r="C428">
+        <v>1</v>
+      </c>
+      <c r="D428" t="s">
+        <v>6</v>
+      </c>
+      <c r="E428" t="s">
+        <v>57</v>
+      </c>
+      <c r="F428" t="s">
+        <v>58</v>
+      </c>
+      <c r="G428" s="1">
+        <v>46231</v>
+      </c>
+      <c r="H428" s="1">
+        <v>46231</v>
+      </c>
+    </row>
+    <row r="429" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A429" t="s">
+        <v>806</v>
+      </c>
+      <c r="B429" t="s">
+        <v>829</v>
+      </c>
+      <c r="C429">
+        <v>1</v>
+      </c>
+      <c r="D429" t="s">
+        <v>6</v>
+      </c>
+      <c r="E429" t="s">
+        <v>57</v>
+      </c>
+      <c r="F429" t="s">
+        <v>58</v>
+      </c>
+      <c r="G429" s="1">
+        <v>46254</v>
+      </c>
+      <c r="H429" s="1">
+        <v>46254</v>
+      </c>
+    </row>
+    <row r="430" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A430" t="s">
+        <v>806</v>
+      </c>
+      <c r="B430" t="s">
+        <v>830</v>
+      </c>
+      <c r="C430">
+        <v>1</v>
+      </c>
+      <c r="D430" t="s">
+        <v>2</v>
+      </c>
+      <c r="E430" t="s">
+        <v>57</v>
+      </c>
+      <c r="F430" t="s">
+        <v>58</v>
+      </c>
+      <c r="G430" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H430" s="1">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="431" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A431" t="s">
+        <v>806</v>
+      </c>
+      <c r="B431" t="s">
+        <v>831</v>
+      </c>
+      <c r="C431">
+        <v>1</v>
+      </c>
+      <c r="D431" t="s">
+        <v>6</v>
+      </c>
+      <c r="E431" t="s">
+        <v>57</v>
+      </c>
+      <c r="F431" t="s">
+        <v>58</v>
+      </c>
+      <c r="G431" s="1">
+        <v>46260</v>
+      </c>
+      <c r="H431" s="1">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="432" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A432" t="s">
+        <v>806</v>
+      </c>
+      <c r="B432" t="s">
+        <v>832</v>
+      </c>
+      <c r="C432">
+        <v>1</v>
+      </c>
+      <c r="D432" t="s">
+        <v>6</v>
+      </c>
+      <c r="E432" t="s">
+        <v>57</v>
+      </c>
+      <c r="F432" t="s">
+        <v>58</v>
+      </c>
+      <c r="G432" s="1">
+        <v>46289</v>
+      </c>
+      <c r="H432" s="1">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="433" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A433" t="s">
+        <v>806</v>
+      </c>
+      <c r="B433" t="s">
+        <v>833</v>
+      </c>
+      <c r="C433">
+        <v>1</v>
+      </c>
+      <c r="D433" t="s">
+        <v>6</v>
+      </c>
+      <c r="E433" t="s">
+        <v>57</v>
+      </c>
+      <c r="F433" t="s">
+        <v>58</v>
+      </c>
+      <c r="G433" s="1">
+        <v>46294</v>
+      </c>
+      <c r="H433" s="1">
+        <v>46294</v>
+      </c>
+    </row>
+    <row r="434" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A434" t="s">
+        <v>806</v>
+      </c>
+      <c r="B434" t="s">
+        <v>834</v>
+      </c>
+      <c r="C434">
+        <v>1</v>
+      </c>
+      <c r="D434" t="s">
+        <v>170</v>
+      </c>
+      <c r="E434" t="s">
+        <v>132</v>
+      </c>
+      <c r="F434" t="s">
+        <v>133</v>
+      </c>
+      <c r="G434" s="1">
+        <v>46308</v>
+      </c>
+      <c r="H434" s="1">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="435" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A435" t="s">
+        <v>835</v>
+      </c>
+      <c r="B435" t="s">
+        <v>836</v>
+      </c>
+      <c r="C435">
+        <v>1</v>
+      </c>
+      <c r="D435" t="s">
+        <v>2</v>
+      </c>
+      <c r="E435" t="s">
+        <v>837</v>
+      </c>
+      <c r="F435" t="s">
+        <v>838</v>
+      </c>
+      <c r="G435" s="1">
+        <v>46157</v>
+      </c>
+      <c r="H435" s="1">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="436" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A436" t="s">
+        <v>835</v>
+      </c>
+      <c r="B436" t="s">
+        <v>839</v>
+      </c>
+      <c r="C436">
+        <v>1</v>
+      </c>
+      <c r="D436" t="s">
+        <v>2</v>
+      </c>
+      <c r="E436" t="s">
+        <v>840</v>
+      </c>
+      <c r="F436" t="s">
+        <v>841</v>
+      </c>
+      <c r="G436" s="1">
+        <v>46168</v>
+      </c>
+      <c r="H436" s="1">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="437" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A437" t="s">
+        <v>835</v>
+      </c>
+      <c r="B437" t="s">
+        <v>842</v>
+      </c>
+      <c r="C437">
+        <v>1</v>
+      </c>
+      <c r="D437" t="s">
+        <v>2</v>
+      </c>
+      <c r="E437" t="s">
+        <v>837</v>
+      </c>
+      <c r="F437" t="s">
+        <v>838</v>
+      </c>
+      <c r="G437" s="1">
+        <v>46218</v>
+      </c>
+      <c r="H437" s="1">
+        <v>46218</v>
+      </c>
+    </row>
+    <row r="438" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A438" t="s">
+        <v>835</v>
+      </c>
+      <c r="B438" t="s">
+        <v>843</v>
+      </c>
+      <c r="C438">
+        <v>1</v>
+      </c>
+      <c r="D438" t="s">
+        <v>2</v>
+      </c>
+      <c r="E438" t="s">
+        <v>837</v>
+      </c>
+      <c r="F438" t="s">
+        <v>838</v>
+      </c>
+      <c r="G438" s="1">
+        <v>46244</v>
+      </c>
+      <c r="H438" s="1">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="439" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A439" t="s">
+        <v>835</v>
+      </c>
+      <c r="B439" t="s">
+        <v>844</v>
+      </c>
+      <c r="C439">
+        <v>1</v>
+      </c>
+      <c r="D439" t="s">
+        <v>2</v>
+      </c>
+      <c r="E439" t="s">
+        <v>837</v>
+      </c>
+      <c r="F439" t="s">
+        <v>838</v>
+      </c>
+      <c r="G439" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H439" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="440" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A440" t="s">
+        <v>835</v>
+      </c>
+      <c r="B440" t="s">
+        <v>845</v>
+      </c>
+      <c r="C440">
+        <v>1</v>
+      </c>
+      <c r="D440" t="s">
+        <v>2</v>
+      </c>
+      <c r="E440" t="s">
+        <v>846</v>
+      </c>
+      <c r="F440" t="s">
+        <v>847</v>
+      </c>
+      <c r="G440" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H440" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="441" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A441" t="s">
+        <v>835</v>
+      </c>
+      <c r="B441" t="s">
+        <v>848</v>
+      </c>
+      <c r="C441">
+        <v>1</v>
+      </c>
+      <c r="D441" t="s">
+        <v>2</v>
+      </c>
+      <c r="E441" t="s">
+        <v>837</v>
+      </c>
+      <c r="F441" t="s">
+        <v>838</v>
+      </c>
+      <c r="G441" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H441" s="1">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="442" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A442" t="s">
+        <v>835</v>
+      </c>
+      <c r="B442" t="s">
+        <v>849</v>
+      </c>
+      <c r="C442">
+        <v>1</v>
+      </c>
+      <c r="D442" t="s">
+        <v>2</v>
+      </c>
+      <c r="E442" t="s">
+        <v>837</v>
+      </c>
+      <c r="F442" t="s">
+        <v>838</v>
+      </c>
+      <c r="G442" s="1">
+        <v>46258</v>
+      </c>
+      <c r="H442" s="1">
+        <v>46258</v>
+      </c>
+    </row>
+    <row r="443" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A443" t="s">
+        <v>835</v>
+      </c>
+      <c r="B443" t="s">
+        <v>850</v>
+      </c>
+      <c r="C443">
+        <v>1</v>
+      </c>
+      <c r="D443" t="s">
+        <v>2</v>
+      </c>
+      <c r="E443" t="s">
+        <v>837</v>
+      </c>
+      <c r="F443" t="s">
+        <v>838</v>
+      </c>
+      <c r="G443" s="1">
+        <v>46262</v>
+      </c>
+      <c r="H443" s="1">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="444" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A444" t="s">
+        <v>835</v>
+      </c>
+      <c r="B444" t="s">
+        <v>851</v>
+      </c>
+      <c r="C444">
+        <v>1</v>
+      </c>
+      <c r="D444" t="s">
+        <v>6</v>
+      </c>
+      <c r="E444" t="s">
+        <v>13</v>
+      </c>
+      <c r="F444" t="s">
+        <v>14</v>
+      </c>
+      <c r="G444" s="1">
+        <v>46281</v>
+      </c>
+      <c r="H444" s="1">
+        <v>46283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 19/10/2026 06:03:47
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53CC9516-8E4E-465F-AA1C-259475813A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6C7AECD-426A-486B-9E6B-4EBF5C8A6EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{22288D16-38B9-40A5-878C-524199312A9F}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{137C0C18-F7D0-4EA6-8986-AB586058BE76}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2318" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2313" uniqueCount="874">
   <si>
     <t>0001</t>
   </si>
@@ -2480,9 +2480,6 @@
   </si>
   <si>
     <t xml:space="preserve">    3036</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    3037</t>
   </si>
   <si>
     <t>4444</t>
@@ -3094,34 +3091,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48AB220E-B375-4697-AECF-D3A2A53895DE}">
-  <dimension ref="A1:H463"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BD6D14C-BC21-4650-B206-D383288A53ED}">
+  <dimension ref="A1:H462"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>866</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>867</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>868</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>869</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>870</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>871</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>872</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>873</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>874</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -5735,7 +5732,7 @@
         <v>1</v>
       </c>
       <c r="D102" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E102" t="s">
         <v>245</v>
@@ -5891,7 +5888,7 @@
         <v>2</v>
       </c>
       <c r="D108" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E108" t="s">
         <v>257</v>
@@ -6827,7 +6824,7 @@
         <v>1</v>
       </c>
       <c r="D144" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E144" t="s">
         <v>319</v>
@@ -8049,7 +8046,7 @@
         <v>1</v>
       </c>
       <c r="D191" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E191" t="s">
         <v>319</v>
@@ -8101,7 +8098,7 @@
         <v>1</v>
       </c>
       <c r="D193" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E193" t="s">
         <v>396</v>
@@ -8153,7 +8150,7 @@
         <v>1</v>
       </c>
       <c r="D195" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E195" t="s">
         <v>402</v>
@@ -8439,7 +8436,7 @@
         <v>1</v>
       </c>
       <c r="D206" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E206" t="s">
         <v>402</v>
@@ -8647,7 +8644,7 @@
         <v>1</v>
       </c>
       <c r="D214" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E214" t="s">
         <v>95</v>
@@ -8673,7 +8670,7 @@
         <v>1</v>
       </c>
       <c r="D215" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E215" t="s">
         <v>172</v>
@@ -8855,7 +8852,7 @@
         <v>1</v>
       </c>
       <c r="D222" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E222" t="s">
         <v>453</v>
@@ -9297,7 +9294,7 @@
         <v>1</v>
       </c>
       <c r="D239" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E239" t="s">
         <v>86</v>
@@ -9401,7 +9398,7 @@
         <v>1</v>
       </c>
       <c r="D243" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E243" t="s">
         <v>492</v>
@@ -9661,7 +9658,7 @@
         <v>1</v>
       </c>
       <c r="D253" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E253" t="s">
         <v>172</v>
@@ -9713,7 +9710,7 @@
         <v>1</v>
       </c>
       <c r="D255" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E255" t="s">
         <v>453</v>
@@ -9791,7 +9788,7 @@
         <v>1</v>
       </c>
       <c r="D258" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E258" t="s">
         <v>519</v>
@@ -10285,7 +10282,7 @@
         <v>1</v>
       </c>
       <c r="D277" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E277" t="s">
         <v>453</v>
@@ -11039,7 +11036,7 @@
         <v>1</v>
       </c>
       <c r="D306" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E306" t="s">
         <v>609</v>
@@ -11481,7 +11478,7 @@
         <v>1</v>
       </c>
       <c r="D323" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E323" t="s">
         <v>638</v>
@@ -11559,7 +11556,7 @@
         <v>1</v>
       </c>
       <c r="D326" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E326" t="s">
         <v>645</v>
@@ -11585,7 +11582,7 @@
         <v>1</v>
       </c>
       <c r="D327" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E327" t="s">
         <v>648</v>
@@ -11793,7 +11790,7 @@
         <v>1</v>
       </c>
       <c r="D335" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E335" t="s">
         <v>662</v>
@@ -11845,7 +11842,7 @@
         <v>1</v>
       </c>
       <c r="D337" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E337" t="s">
         <v>662</v>
@@ -12261,7 +12258,7 @@
         <v>1</v>
       </c>
       <c r="D353" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E353" t="s">
         <v>692</v>
@@ -12807,7 +12804,7 @@
         <v>1</v>
       </c>
       <c r="D374" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E374" t="s">
         <v>304</v>
@@ -13873,7 +13870,7 @@
         <v>2</v>
       </c>
       <c r="D415" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E415" t="s">
         <v>805</v>
@@ -14176,59 +14173,59 @@
     </row>
     <row r="427" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A427" t="s">
-        <v>793</v>
+        <v>820</v>
       </c>
       <c r="B427" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="C427">
         <v>1</v>
       </c>
       <c r="D427" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E427" t="s">
-        <v>304</v>
+        <v>822</v>
       </c>
       <c r="F427" t="s">
-        <v>305</v>
+        <v>823</v>
       </c>
       <c r="G427" s="1">
-        <v>46311</v>
+        <v>46063</v>
       </c>
       <c r="H427" s="1">
-        <v>46311</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="428" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A428" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B428" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
       <c r="C428">
         <v>1</v>
       </c>
       <c r="D428" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E428" t="s">
-        <v>823</v>
+        <v>57</v>
       </c>
       <c r="F428" t="s">
-        <v>824</v>
+        <v>58</v>
       </c>
       <c r="G428" s="1">
-        <v>46063</v>
+        <v>46113</v>
       </c>
       <c r="H428" s="1">
-        <v>46064</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="429" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A429" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B429" t="s">
         <v>825</v>
@@ -14237,7 +14234,7 @@
         <v>1</v>
       </c>
       <c r="D429" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E429" t="s">
         <v>57</v>
@@ -14246,7 +14243,7 @@
         <v>58</v>
       </c>
       <c r="G429" s="1">
-        <v>46113</v>
+        <v>46125</v>
       </c>
       <c r="H429" s="1">
         <v>46125</v>
@@ -14254,7 +14251,7 @@
     </row>
     <row r="430" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A430" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B430" t="s">
         <v>826</v>
@@ -14272,15 +14269,15 @@
         <v>58</v>
       </c>
       <c r="G430" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="H430" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="431" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A431" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B431" t="s">
         <v>827</v>
@@ -14306,7 +14303,7 @@
     </row>
     <row r="432" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A432" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B432" t="s">
         <v>828</v>
@@ -14324,15 +14321,15 @@
         <v>58</v>
       </c>
       <c r="G432" s="1">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="H432" s="1">
-        <v>46126</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="433" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A433" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B433" t="s">
         <v>829</v>
@@ -14341,7 +14338,7 @@
         <v>1</v>
       </c>
       <c r="D433" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E433" t="s">
         <v>57</v>
@@ -14350,15 +14347,15 @@
         <v>58</v>
       </c>
       <c r="G433" s="1">
-        <v>46128</v>
+        <v>46132</v>
       </c>
       <c r="H433" s="1">
-        <v>46128</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="434" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A434" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B434" t="s">
         <v>830</v>
@@ -14367,7 +14364,7 @@
         <v>1</v>
       </c>
       <c r="D434" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E434" t="s">
         <v>57</v>
@@ -14376,15 +14373,15 @@
         <v>58</v>
       </c>
       <c r="G434" s="1">
-        <v>46132</v>
+        <v>46161</v>
       </c>
       <c r="H434" s="1">
-        <v>46132</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="435" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A435" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B435" t="s">
         <v>831</v>
@@ -14402,15 +14399,15 @@
         <v>58</v>
       </c>
       <c r="G435" s="1">
-        <v>46161</v>
+        <v>46174</v>
       </c>
       <c r="H435" s="1">
-        <v>46161</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="436" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A436" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B436" t="s">
         <v>832</v>
@@ -14436,7 +14433,7 @@
     </row>
     <row r="437" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A437" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B437" t="s">
         <v>833</v>
@@ -14445,7 +14442,7 @@
         <v>1</v>
       </c>
       <c r="D437" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E437" t="s">
         <v>57</v>
@@ -14454,15 +14451,15 @@
         <v>58</v>
       </c>
       <c r="G437" s="1">
-        <v>46174</v>
+        <v>46195</v>
       </c>
       <c r="H437" s="1">
-        <v>46174</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="438" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A438" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B438" t="s">
         <v>834</v>
@@ -14480,15 +14477,15 @@
         <v>58</v>
       </c>
       <c r="G438" s="1">
-        <v>46195</v>
+        <v>46210</v>
       </c>
       <c r="H438" s="1">
-        <v>46252</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="439" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A439" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B439" t="s">
         <v>835</v>
@@ -14497,7 +14494,7 @@
         <v>1</v>
       </c>
       <c r="D439" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E439" t="s">
         <v>57</v>
@@ -14506,15 +14503,15 @@
         <v>58</v>
       </c>
       <c r="G439" s="1">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="H439" s="1">
-        <v>46210</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="440" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A440" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B440" t="s">
         <v>836</v>
@@ -14523,7 +14520,7 @@
         <v>1</v>
       </c>
       <c r="D440" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E440" t="s">
         <v>57</v>
@@ -14532,15 +14529,15 @@
         <v>58</v>
       </c>
       <c r="G440" s="1">
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="H440" s="1">
-        <v>46213</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="441" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A441" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B441" t="s">
         <v>837</v>
@@ -14552,21 +14549,21 @@
         <v>6</v>
       </c>
       <c r="E441" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="F441" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G441" s="1">
-        <v>46218</v>
+        <v>46226</v>
       </c>
       <c r="H441" s="1">
-        <v>46252</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="442" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A442" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B442" t="s">
         <v>838</v>
@@ -14575,24 +14572,24 @@
         <v>1</v>
       </c>
       <c r="D442" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E442" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="F442" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G442" s="1">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="H442" s="1">
-        <v>46226</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="443" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A443" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B443" t="s">
         <v>839</v>
@@ -14601,7 +14598,7 @@
         <v>1</v>
       </c>
       <c r="D443" t="s">
-        <v>128</v>
+        <v>6</v>
       </c>
       <c r="E443" t="s">
         <v>57</v>
@@ -14618,7 +14615,7 @@
     </row>
     <row r="444" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A444" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B444" t="s">
         <v>840</v>
@@ -14639,12 +14636,12 @@
         <v>46227</v>
       </c>
       <c r="H444" s="1">
-        <v>46252</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="445" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A445" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B445" t="s">
         <v>841</v>
@@ -14656,21 +14653,21 @@
         <v>6</v>
       </c>
       <c r="E445" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="F445" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G445" s="1">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="H445" s="1">
-        <v>46228</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="446" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A446" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B446" t="s">
         <v>842</v>
@@ -14682,21 +14679,21 @@
         <v>6</v>
       </c>
       <c r="E446" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="F446" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G446" s="1">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="H446" s="1">
-        <v>46252</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="447" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A447" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B447" t="s">
         <v>843</v>
@@ -14714,15 +14711,15 @@
         <v>58</v>
       </c>
       <c r="G447" s="1">
-        <v>46231</v>
+        <v>46254</v>
       </c>
       <c r="H447" s="1">
-        <v>46231</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="448" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A448" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B448" t="s">
         <v>844</v>
@@ -14731,7 +14728,7 @@
         <v>1</v>
       </c>
       <c r="D448" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E448" t="s">
         <v>57</v>
@@ -14740,15 +14737,15 @@
         <v>58</v>
       </c>
       <c r="G448" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="H448" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="449" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A449" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B449" t="s">
         <v>845</v>
@@ -14757,7 +14754,7 @@
         <v>1</v>
       </c>
       <c r="D449" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E449" t="s">
         <v>57</v>
@@ -14766,15 +14763,15 @@
         <v>58</v>
       </c>
       <c r="G449" s="1">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H449" s="1">
-        <v>46255</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="450" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A450" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B450" t="s">
         <v>846</v>
@@ -14792,15 +14789,15 @@
         <v>58</v>
       </c>
       <c r="G450" s="1">
-        <v>46260</v>
+        <v>46289</v>
       </c>
       <c r="H450" s="1">
-        <v>46260</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="451" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A451" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B451" t="s">
         <v>847</v>
@@ -14818,15 +14815,15 @@
         <v>58</v>
       </c>
       <c r="G451" s="1">
-        <v>46289</v>
+        <v>46294</v>
       </c>
       <c r="H451" s="1">
-        <v>46289</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="452" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A452" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B452" t="s">
         <v>848</v>
@@ -14835,7 +14832,7 @@
         <v>1</v>
       </c>
       <c r="D452" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E452" t="s">
         <v>57</v>
@@ -14844,44 +14841,44 @@
         <v>58</v>
       </c>
       <c r="G452" s="1">
-        <v>46294</v>
+        <v>46311</v>
       </c>
       <c r="H452" s="1">
-        <v>46294</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="453" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A453" t="s">
-        <v>821</v>
+        <v>849</v>
       </c>
       <c r="B453" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="C453">
         <v>1</v>
       </c>
       <c r="D453" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E453" t="s">
-        <v>57</v>
+        <v>851</v>
       </c>
       <c r="F453" t="s">
-        <v>58</v>
+        <v>852</v>
       </c>
       <c r="G453" s="1">
-        <v>46311</v>
+        <v>46157</v>
       </c>
       <c r="H453" s="1">
-        <v>46311</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="454" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A454" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B454" t="s">
-        <v>851</v>
+        <v>853</v>
       </c>
       <c r="C454">
         <v>1</v>
@@ -14890,24 +14887,24 @@
         <v>2</v>
       </c>
       <c r="E454" t="s">
-        <v>852</v>
+        <v>854</v>
       </c>
       <c r="F454" t="s">
-        <v>853</v>
+        <v>855</v>
       </c>
       <c r="G454" s="1">
-        <v>46157</v>
+        <v>46168</v>
       </c>
       <c r="H454" s="1">
-        <v>46157</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="455" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A455" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B455" t="s">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="C455">
         <v>1</v>
@@ -14916,21 +14913,21 @@
         <v>2</v>
       </c>
       <c r="E455" t="s">
-        <v>855</v>
+        <v>851</v>
       </c>
       <c r="F455" t="s">
-        <v>856</v>
+        <v>852</v>
       </c>
       <c r="G455" s="1">
-        <v>46168</v>
+        <v>46218</v>
       </c>
       <c r="H455" s="1">
-        <v>46170</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="456" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A456" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B456" t="s">
         <v>857</v>
@@ -14942,21 +14939,21 @@
         <v>2</v>
       </c>
       <c r="E456" t="s">
+        <v>851</v>
+      </c>
+      <c r="F456" t="s">
         <v>852</v>
       </c>
-      <c r="F456" t="s">
-        <v>853</v>
-      </c>
       <c r="G456" s="1">
-        <v>46218</v>
+        <v>46244</v>
       </c>
       <c r="H456" s="1">
-        <v>46218</v>
+        <v>46244</v>
       </c>
     </row>
     <row r="457" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A457" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B457" t="s">
         <v>858</v>
@@ -14968,21 +14965,21 @@
         <v>2</v>
       </c>
       <c r="E457" t="s">
+        <v>851</v>
+      </c>
+      <c r="F457" t="s">
         <v>852</v>
       </c>
-      <c r="F457" t="s">
-        <v>853</v>
-      </c>
       <c r="G457" s="1">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="H457" s="1">
-        <v>46244</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="458" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A458" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B458" t="s">
         <v>859</v>
@@ -14994,10 +14991,10 @@
         <v>2</v>
       </c>
       <c r="E458" t="s">
-        <v>852</v>
+        <v>860</v>
       </c>
       <c r="F458" t="s">
-        <v>853</v>
+        <v>861</v>
       </c>
       <c r="G458" s="1">
         <v>46247</v>
@@ -15008,10 +15005,10 @@
     </row>
     <row r="459" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A459" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B459" t="s">
-        <v>860</v>
+        <v>862</v>
       </c>
       <c r="C459">
         <v>1</v>
@@ -15020,21 +15017,21 @@
         <v>2</v>
       </c>
       <c r="E459" t="s">
-        <v>861</v>
+        <v>851</v>
       </c>
       <c r="F459" t="s">
-        <v>862</v>
+        <v>852</v>
       </c>
       <c r="G459" s="1">
-        <v>46247</v>
+        <v>46255</v>
       </c>
       <c r="H459" s="1">
-        <v>46247</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="460" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A460" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B460" t="s">
         <v>863</v>
@@ -15046,21 +15043,21 @@
         <v>2</v>
       </c>
       <c r="E460" t="s">
+        <v>851</v>
+      </c>
+      <c r="F460" t="s">
         <v>852</v>
       </c>
-      <c r="F460" t="s">
-        <v>853</v>
-      </c>
       <c r="G460" s="1">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="H460" s="1">
-        <v>46255</v>
+        <v>46258</v>
       </c>
     </row>
     <row r="461" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A461" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B461" t="s">
         <v>864</v>
@@ -15072,21 +15069,21 @@
         <v>2</v>
       </c>
       <c r="E461" t="s">
+        <v>851</v>
+      </c>
+      <c r="F461" t="s">
         <v>852</v>
       </c>
-      <c r="F461" t="s">
-        <v>853</v>
-      </c>
       <c r="G461" s="1">
-        <v>46258</v>
+        <v>46262</v>
       </c>
       <c r="H461" s="1">
-        <v>46258</v>
+        <v>46265</v>
       </c>
     </row>
     <row r="462" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A462" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B462" t="s">
         <v>865</v>
@@ -15095,44 +15092,18 @@
         <v>1</v>
       </c>
       <c r="D462" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E462" t="s">
-        <v>852</v>
+        <v>13</v>
       </c>
       <c r="F462" t="s">
-        <v>853</v>
+        <v>14</v>
       </c>
       <c r="G462" s="1">
-        <v>46262</v>
+        <v>46281</v>
       </c>
       <c r="H462" s="1">
-        <v>46265</v>
-      </c>
-    </row>
-    <row r="463" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A463" t="s">
-        <v>850</v>
-      </c>
-      <c r="B463" t="s">
-        <v>866</v>
-      </c>
-      <c r="C463">
-        <v>1</v>
-      </c>
-      <c r="D463" t="s">
-        <v>6</v>
-      </c>
-      <c r="E463" t="s">
-        <v>13</v>
-      </c>
-      <c r="F463" t="s">
-        <v>14</v>
-      </c>
-      <c r="G463" s="1">
-        <v>46281</v>
-      </c>
-      <c r="H463" s="1">
         <v>46283</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 19/10/2026 13:46:53
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9534208-7359-444D-917F-546BA125C696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4DE8EA38-8553-47FE-AE1C-60ABE44AC086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{DFD691D7-9BE4-469A-B41B-2D3804B813B6}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{1E11C2D4-5331-47AE-BAF3-888CC7AE6D66}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2438" uniqueCount="916">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2563" uniqueCount="965">
   <si>
     <t>0001</t>
   </si>
@@ -2071,9 +2071,6 @@
     <t xml:space="preserve">  217682</t>
   </si>
   <si>
-    <t xml:space="preserve">  217683</t>
-  </si>
-  <si>
     <t xml:space="preserve">  217685</t>
   </si>
   <si>
@@ -2089,6 +2086,15 @@
     <t>ORQUEDA LUIS ALBERTO</t>
   </si>
   <si>
+    <t xml:space="preserve">  217688</t>
+  </si>
+  <si>
+    <t>CZ01</t>
+  </si>
+  <si>
+    <t>CASA ZEILA DE J.M.BERNALES</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217689</t>
   </si>
   <si>
@@ -2101,6 +2107,9 @@
     <t>MEDRANO CONSTRUCCIONES S.A.</t>
   </si>
   <si>
+    <t xml:space="preserve">  217691</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217693</t>
   </si>
   <si>
@@ -2158,6 +2167,15 @@
     <t xml:space="preserve">  217703</t>
   </si>
   <si>
+    <t xml:space="preserve">  217706</t>
+  </si>
+  <si>
+    <t>MM44</t>
+  </si>
+  <si>
+    <t>MOTTESI MATERIALES SA</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217707</t>
   </si>
   <si>
@@ -2170,6 +2188,24 @@
     <t xml:space="preserve">  217708</t>
   </si>
   <si>
+    <t xml:space="preserve">  217709</t>
+  </si>
+  <si>
+    <t>GI01</t>
+  </si>
+  <si>
+    <t>GILI Y CIA SRL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217710</t>
+  </si>
+  <si>
+    <t>GA31</t>
+  </si>
+  <si>
+    <t>GALBAHIA S.R.L.</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217711</t>
   </si>
   <si>
@@ -2194,6 +2230,9 @@
     <t>JOSE ANACLETO E HIJOS S.A.</t>
   </si>
   <si>
+    <t xml:space="preserve">  217716</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217717</t>
   </si>
   <si>
@@ -2332,6 +2371,15 @@
     <t>GAETO RUBEN ERNESTO</t>
   </si>
   <si>
+    <t xml:space="preserve">  217746</t>
+  </si>
+  <si>
+    <t>GG36</t>
+  </si>
+  <si>
+    <t>G36 SOCIEDAD SIMPLE</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217747</t>
   </si>
   <si>
@@ -2368,6 +2416,9 @@
     <t xml:space="preserve">  217752</t>
   </si>
   <si>
+    <t xml:space="preserve">  217753</t>
+  </si>
+  <si>
     <t xml:space="preserve">  217754</t>
   </si>
   <si>
@@ -2476,6 +2527,111 @@
     <t xml:space="preserve">  217773</t>
   </si>
   <si>
+    <t xml:space="preserve">  217775</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217776</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217777</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217778</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217779</t>
+  </si>
+  <si>
+    <t>EC11</t>
+  </si>
+  <si>
+    <t>ES-COR DESIGN S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217780</t>
+  </si>
+  <si>
+    <t>GE12</t>
+  </si>
+  <si>
+    <t>GERMANO S.R.L. -GERMANO MATERIALES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217781</t>
+  </si>
+  <si>
+    <t>BN01</t>
+  </si>
+  <si>
+    <t>BARBOSA NESTOR AGUSTIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217782</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217784</t>
+  </si>
+  <si>
+    <t>SS41</t>
+  </si>
+  <si>
+    <t>SANITARIOS SANJUAN S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217785</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217786</t>
+  </si>
+  <si>
+    <t>CE21</t>
+  </si>
+  <si>
+    <t>CERYSAN S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217787</t>
+  </si>
+  <si>
+    <t>MS27</t>
+  </si>
+  <si>
+    <t>MODULAR SOLUTIONS S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217788</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217789</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217790</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217791</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217792</t>
+  </si>
+  <si>
+    <t>SG13</t>
+  </si>
+  <si>
+    <t>SANITARIOS GAONA S.A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217793</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217794</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217795</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  217796</t>
+  </si>
+  <si>
     <t>0004</t>
   </si>
   <si>
@@ -2590,6 +2746,9 @@
     <t>VARIOS</t>
   </si>
   <si>
+    <t xml:space="preserve">    3041</t>
+  </si>
+  <si>
     <t>4444</t>
   </si>
   <si>
@@ -2681,18 +2840,6 @@
   </si>
   <si>
     <t xml:space="preserve">    2839</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2841</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2842</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2843</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2845</t>
   </si>
   <si>
     <t>9999</t>
@@ -3217,34 +3364,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E51FFFB9-157F-4F6B-A76B-A57C734685FA}">
-  <dimension ref="A1:H487"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01EF979-3FD2-49BF-85C2-90AF2D642C38}">
+  <dimension ref="A1:H512"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>908</v>
+        <v>957</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>909</v>
+        <v>958</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>910</v>
+        <v>959</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>911</v>
+        <v>960</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>912</v>
+        <v>961</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>913</v>
+        <v>962</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>914</v>
+        <v>963</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>915</v>
+        <v>964</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -5985,10 +6132,10 @@
         <v>255</v>
       </c>
       <c r="C107">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D107" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E107" t="s">
         <v>118</v>
@@ -6000,7 +6147,7 @@
         <v>46294</v>
       </c>
       <c r="H107" s="1">
-        <v>46294</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.2">
@@ -6794,7 +6941,7 @@
         <v>1</v>
       </c>
       <c r="D138" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E138" t="s">
         <v>37</v>
@@ -6846,7 +6993,7 @@
         <v>1</v>
       </c>
       <c r="D140" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E140" t="s">
         <v>37</v>
@@ -7002,7 +7149,7 @@
         <v>1</v>
       </c>
       <c r="D146" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E146" t="s">
         <v>37</v>
@@ -7444,7 +7591,7 @@
         <v>1</v>
       </c>
       <c r="D163" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E163" t="s">
         <v>37</v>
@@ -7470,7 +7617,7 @@
         <v>1</v>
       </c>
       <c r="D164" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E164" t="s">
         <v>37</v>
@@ -7652,7 +7799,7 @@
         <v>2</v>
       </c>
       <c r="D171" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E171" t="s">
         <v>364</v>
@@ -8198,7 +8345,7 @@
         <v>2</v>
       </c>
       <c r="D192" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E192" t="s">
         <v>393</v>
@@ -8250,7 +8397,7 @@
         <v>1</v>
       </c>
       <c r="D194" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E194" t="s">
         <v>332</v>
@@ -8328,7 +8475,7 @@
         <v>1</v>
       </c>
       <c r="D197" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E197" t="s">
         <v>273</v>
@@ -8458,7 +8605,7 @@
         <v>1</v>
       </c>
       <c r="D202" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E202" t="s">
         <v>332</v>
@@ -8640,7 +8787,7 @@
         <v>1</v>
       </c>
       <c r="D209" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E209" t="s">
         <v>385</v>
@@ -9238,7 +9385,7 @@
         <v>1</v>
       </c>
       <c r="D232" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E232" t="s">
         <v>468</v>
@@ -9264,7 +9411,7 @@
         <v>1</v>
       </c>
       <c r="D233" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E233" t="s">
         <v>471</v>
@@ -9342,7 +9489,7 @@
         <v>1</v>
       </c>
       <c r="D236" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E236" t="s">
         <v>478</v>
@@ -9394,7 +9541,7 @@
         <v>1</v>
       </c>
       <c r="D238" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E238" t="s">
         <v>332</v>
@@ -9888,7 +10035,7 @@
         <v>1</v>
       </c>
       <c r="D257" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E257" t="s">
         <v>519</v>
@@ -9914,7 +10061,7 @@
         <v>1</v>
       </c>
       <c r="D258" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E258" t="s">
         <v>332</v>
@@ -9966,7 +10113,7 @@
         <v>1</v>
       </c>
       <c r="D260" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E260" t="s">
         <v>152</v>
@@ -10772,7 +10919,7 @@
         <v>1</v>
       </c>
       <c r="D291" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E291" t="s">
         <v>519</v>
@@ -11422,7 +11569,7 @@
         <v>2</v>
       </c>
       <c r="D316" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E316" t="s">
         <v>624</v>
@@ -11448,7 +11595,7 @@
         <v>1</v>
       </c>
       <c r="D317" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E317" t="s">
         <v>385</v>
@@ -11500,7 +11647,7 @@
         <v>1</v>
       </c>
       <c r="D319" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E319" t="s">
         <v>604</v>
@@ -11838,7 +11985,7 @@
         <v>1</v>
       </c>
       <c r="D332" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E332" t="s">
         <v>650</v>
@@ -12046,7 +12193,7 @@
         <v>1</v>
       </c>
       <c r="D340" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E340" t="s">
         <v>664</v>
@@ -12072,7 +12219,7 @@
         <v>1</v>
       </c>
       <c r="D341" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E341" t="s">
         <v>664</v>
@@ -12150,7 +12297,7 @@
         <v>1</v>
       </c>
       <c r="D344" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E344" t="s">
         <v>664</v>
@@ -12332,7 +12479,7 @@
         <v>1</v>
       </c>
       <c r="D351" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E351" t="s">
         <v>364</v>
@@ -12358,13 +12505,13 @@
         <v>1</v>
       </c>
       <c r="D352" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E352" t="s">
-        <v>301</v>
+        <v>405</v>
       </c>
       <c r="F352" t="s">
-        <v>302</v>
+        <v>406</v>
       </c>
       <c r="G352" s="1">
         <v>46311</v>
@@ -12387,10 +12534,10 @@
         <v>128</v>
       </c>
       <c r="E353" t="s">
-        <v>405</v>
+        <v>390</v>
       </c>
       <c r="F353" t="s">
-        <v>406</v>
+        <v>391</v>
       </c>
       <c r="G353" s="1">
         <v>46311</v>
@@ -12413,10 +12560,10 @@
         <v>128</v>
       </c>
       <c r="E354" t="s">
-        <v>390</v>
+        <v>686</v>
       </c>
       <c r="F354" t="s">
-        <v>391</v>
+        <v>687</v>
       </c>
       <c r="G354" s="1">
         <v>46311</v>
@@ -12430,7 +12577,7 @@
         <v>0</v>
       </c>
       <c r="B355" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="C355">
         <v>1</v>
@@ -12439,16 +12586,16 @@
         <v>128</v>
       </c>
       <c r="E355" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="F355" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="G355" s="1">
         <v>46311</v>
       </c>
       <c r="H355" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="356" spans="1:8" x14ac:dyDescent="0.2">
@@ -12456,7 +12603,7 @@
         <v>0</v>
       </c>
       <c r="B356" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="C356">
         <v>1</v>
@@ -12465,10 +12612,10 @@
         <v>128</v>
       </c>
       <c r="E356" t="s">
+        <v>686</v>
+      </c>
+      <c r="F356" t="s">
         <v>687</v>
-      </c>
-      <c r="F356" t="s">
-        <v>688</v>
       </c>
       <c r="G356" s="1">
         <v>46311</v>
@@ -12482,7 +12629,7 @@
         <v>0</v>
       </c>
       <c r="B357" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="C357">
         <v>1</v>
@@ -12491,10 +12638,10 @@
         <v>128</v>
       </c>
       <c r="E357" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="F357" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="G357" s="1">
         <v>46311</v>
@@ -12508,7 +12655,7 @@
         <v>0</v>
       </c>
       <c r="B358" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="C358">
         <v>1</v>
@@ -12517,16 +12664,16 @@
         <v>128</v>
       </c>
       <c r="E358" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="F358" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="G358" s="1">
         <v>46311</v>
       </c>
       <c r="H358" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="359" spans="1:8" x14ac:dyDescent="0.2">
@@ -12540,13 +12687,13 @@
         <v>1</v>
       </c>
       <c r="D359" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E359" t="s">
-        <v>7</v>
+        <v>697</v>
       </c>
       <c r="F359" t="s">
-        <v>8</v>
+        <v>698</v>
       </c>
       <c r="G359" s="1">
         <v>46311</v>
@@ -12560,7 +12707,7 @@
         <v>0</v>
       </c>
       <c r="B360" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="C360">
         <v>1</v>
@@ -12569,10 +12716,10 @@
         <v>128</v>
       </c>
       <c r="E360" t="s">
-        <v>698</v>
+        <v>7</v>
       </c>
       <c r="F360" t="s">
-        <v>699</v>
+        <v>8</v>
       </c>
       <c r="G360" s="1">
         <v>46311</v>
@@ -12592,19 +12739,19 @@
         <v>1</v>
       </c>
       <c r="D361" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E361" t="s">
-        <v>95</v>
+        <v>701</v>
       </c>
       <c r="F361" t="s">
-        <v>96</v>
+        <v>702</v>
       </c>
       <c r="G361" s="1">
         <v>46311</v>
       </c>
       <c r="H361" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="362" spans="1:8" x14ac:dyDescent="0.2">
@@ -12612,7 +12759,7 @@
         <v>0</v>
       </c>
       <c r="B362" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="C362">
         <v>1</v>
@@ -12630,7 +12777,7 @@
         <v>46311</v>
       </c>
       <c r="H362" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="363" spans="1:8" x14ac:dyDescent="0.2">
@@ -12638,7 +12785,7 @@
         <v>0</v>
       </c>
       <c r="B363" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="C363">
         <v>1</v>
@@ -12647,10 +12794,10 @@
         <v>128</v>
       </c>
       <c r="E363" t="s">
-        <v>703</v>
+        <v>95</v>
       </c>
       <c r="F363" t="s">
-        <v>704</v>
+        <v>96</v>
       </c>
       <c r="G363" s="1">
         <v>46311</v>
@@ -12725,10 +12872,10 @@
         <v>128</v>
       </c>
       <c r="E366" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="F366" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="G366" s="1">
         <v>46311</v>
@@ -12742,19 +12889,19 @@
         <v>0</v>
       </c>
       <c r="B367" t="s">
+        <v>714</v>
+      </c>
+      <c r="C367">
+        <v>1</v>
+      </c>
+      <c r="D367" t="s">
+        <v>128</v>
+      </c>
+      <c r="E367" t="s">
         <v>712</v>
       </c>
-      <c r="C367">
-        <v>1</v>
-      </c>
-      <c r="D367" t="s">
-        <v>128</v>
-      </c>
-      <c r="E367" t="s">
+      <c r="F367" t="s">
         <v>713</v>
-      </c>
-      <c r="F367" t="s">
-        <v>714</v>
       </c>
       <c r="G367" s="1">
         <v>46311</v>
@@ -12777,16 +12924,16 @@
         <v>128</v>
       </c>
       <c r="E368" t="s">
-        <v>582</v>
+        <v>716</v>
       </c>
       <c r="F368" t="s">
-        <v>583</v>
+        <v>717</v>
       </c>
       <c r="G368" s="1">
         <v>46311</v>
       </c>
       <c r="H368" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="369" spans="1:8" x14ac:dyDescent="0.2">
@@ -12794,7 +12941,7 @@
         <v>0</v>
       </c>
       <c r="B369" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="C369">
         <v>1</v>
@@ -12803,10 +12950,10 @@
         <v>128</v>
       </c>
       <c r="E369" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="F369" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="G369" s="1">
         <v>46311</v>
@@ -12820,7 +12967,7 @@
         <v>0</v>
       </c>
       <c r="B370" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C370">
         <v>1</v>
@@ -12829,10 +12976,10 @@
         <v>128</v>
       </c>
       <c r="E370" t="s">
-        <v>553</v>
+        <v>582</v>
       </c>
       <c r="F370" t="s">
-        <v>554</v>
+        <v>583</v>
       </c>
       <c r="G370" s="1">
         <v>46311</v>
@@ -12846,7 +12993,7 @@
         <v>0</v>
       </c>
       <c r="B371" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C371">
         <v>1</v>
@@ -12855,16 +13002,16 @@
         <v>128</v>
       </c>
       <c r="E371" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="F371" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="G371" s="1">
         <v>46311</v>
       </c>
       <c r="H371" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="372" spans="1:8" x14ac:dyDescent="0.2">
@@ -12872,7 +13019,7 @@
         <v>0</v>
       </c>
       <c r="B372" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="C372">
         <v>1</v>
@@ -12881,16 +13028,16 @@
         <v>128</v>
       </c>
       <c r="E372" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="F372" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="G372" s="1">
         <v>46311</v>
       </c>
       <c r="H372" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="373" spans="1:8" x14ac:dyDescent="0.2">
@@ -12898,7 +13045,7 @@
         <v>0</v>
       </c>
       <c r="B373" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="C373">
         <v>1</v>
@@ -12907,16 +13054,16 @@
         <v>128</v>
       </c>
       <c r="E373" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="F373" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="G373" s="1">
         <v>46311</v>
       </c>
       <c r="H373" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="374" spans="1:8" x14ac:dyDescent="0.2">
@@ -12924,7 +13071,7 @@
         <v>0</v>
       </c>
       <c r="B374" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="C374">
         <v>1</v>
@@ -12933,10 +13080,10 @@
         <v>128</v>
       </c>
       <c r="E374" t="s">
-        <v>728</v>
+        <v>553</v>
       </c>
       <c r="F374" t="s">
-        <v>729</v>
+        <v>554</v>
       </c>
       <c r="G374" s="1">
         <v>46311</v>
@@ -12950,19 +13097,19 @@
         <v>0</v>
       </c>
       <c r="B375" t="s">
+        <v>732</v>
+      </c>
+      <c r="C375">
+        <v>1</v>
+      </c>
+      <c r="D375" t="s">
+        <v>128</v>
+      </c>
+      <c r="E375" t="s">
+        <v>729</v>
+      </c>
+      <c r="F375" t="s">
         <v>730</v>
-      </c>
-      <c r="C375">
-        <v>1</v>
-      </c>
-      <c r="D375" t="s">
-        <v>128</v>
-      </c>
-      <c r="E375" t="s">
-        <v>731</v>
-      </c>
-      <c r="F375" t="s">
-        <v>732</v>
       </c>
       <c r="G375" s="1">
         <v>46311</v>
@@ -12985,10 +13132,10 @@
         <v>128</v>
       </c>
       <c r="E376" t="s">
-        <v>345</v>
+        <v>734</v>
       </c>
       <c r="F376" t="s">
-        <v>346</v>
+        <v>735</v>
       </c>
       <c r="G376" s="1">
         <v>46311</v>
@@ -13002,7 +13149,7 @@
         <v>0</v>
       </c>
       <c r="B377" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="C377">
         <v>1</v>
@@ -13011,16 +13158,16 @@
         <v>128</v>
       </c>
       <c r="E377" t="s">
-        <v>722</v>
+        <v>64</v>
       </c>
       <c r="F377" t="s">
-        <v>723</v>
+        <v>65</v>
       </c>
       <c r="G377" s="1">
         <v>46311</v>
       </c>
       <c r="H377" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="378" spans="1:8" x14ac:dyDescent="0.2">
@@ -13028,7 +13175,7 @@
         <v>0</v>
       </c>
       <c r="B378" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="C378">
         <v>1</v>
@@ -13037,16 +13184,16 @@
         <v>128</v>
       </c>
       <c r="E378" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="F378" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="G378" s="1">
         <v>46311</v>
       </c>
       <c r="H378" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="379" spans="1:8" x14ac:dyDescent="0.2">
@@ -13054,7 +13201,7 @@
         <v>0</v>
       </c>
       <c r="B379" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="C379">
         <v>1</v>
@@ -13063,10 +13210,10 @@
         <v>128</v>
       </c>
       <c r="E379" t="s">
-        <v>219</v>
+        <v>741</v>
       </c>
       <c r="F379" t="s">
-        <v>220</v>
+        <v>742</v>
       </c>
       <c r="G379" s="1">
         <v>46311</v>
@@ -13080,7 +13227,7 @@
         <v>0</v>
       </c>
       <c r="B380" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="C380">
         <v>1</v>
@@ -13089,10 +13236,10 @@
         <v>128</v>
       </c>
       <c r="E380" t="s">
-        <v>16</v>
+        <v>744</v>
       </c>
       <c r="F380" t="s">
-        <v>17</v>
+        <v>745</v>
       </c>
       <c r="G380" s="1">
         <v>46311</v>
@@ -13106,7 +13253,7 @@
         <v>0</v>
       </c>
       <c r="B381" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="C381">
         <v>1</v>
@@ -13115,10 +13262,10 @@
         <v>128</v>
       </c>
       <c r="E381" t="s">
-        <v>16</v>
+        <v>345</v>
       </c>
       <c r="F381" t="s">
-        <v>17</v>
+        <v>346</v>
       </c>
       <c r="G381" s="1">
         <v>46311</v>
@@ -13132,7 +13279,7 @@
         <v>0</v>
       </c>
       <c r="B382" t="s">
-        <v>741</v>
+        <v>747</v>
       </c>
       <c r="C382">
         <v>1</v>
@@ -13141,10 +13288,10 @@
         <v>128</v>
       </c>
       <c r="E382" t="s">
-        <v>3</v>
+        <v>734</v>
       </c>
       <c r="F382" t="s">
-        <v>4</v>
+        <v>735</v>
       </c>
       <c r="G382" s="1">
         <v>46311</v>
@@ -13158,7 +13305,7 @@
         <v>0</v>
       </c>
       <c r="B383" t="s">
-        <v>742</v>
+        <v>748</v>
       </c>
       <c r="C383">
         <v>1</v>
@@ -13167,10 +13314,10 @@
         <v>128</v>
       </c>
       <c r="E383" t="s">
-        <v>728</v>
+        <v>749</v>
       </c>
       <c r="F383" t="s">
-        <v>729</v>
+        <v>750</v>
       </c>
       <c r="G383" s="1">
         <v>46311</v>
@@ -13184,7 +13331,7 @@
         <v>0</v>
       </c>
       <c r="B384" t="s">
-        <v>743</v>
+        <v>751</v>
       </c>
       <c r="C384">
         <v>1</v>
@@ -13193,16 +13340,16 @@
         <v>128</v>
       </c>
       <c r="E384" t="s">
-        <v>572</v>
+        <v>219</v>
       </c>
       <c r="F384" t="s">
-        <v>573</v>
+        <v>220</v>
       </c>
       <c r="G384" s="1">
         <v>46311</v>
       </c>
       <c r="H384" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="385" spans="1:8" x14ac:dyDescent="0.2">
@@ -13210,7 +13357,7 @@
         <v>0</v>
       </c>
       <c r="B385" t="s">
-        <v>744</v>
+        <v>752</v>
       </c>
       <c r="C385">
         <v>1</v>
@@ -13219,16 +13366,16 @@
         <v>128</v>
       </c>
       <c r="E385" t="s">
-        <v>745</v>
+        <v>16</v>
       </c>
       <c r="F385" t="s">
-        <v>746</v>
+        <v>17</v>
       </c>
       <c r="G385" s="1">
         <v>46311</v>
       </c>
       <c r="H385" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="386" spans="1:8" x14ac:dyDescent="0.2">
@@ -13236,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="B386" t="s">
-        <v>747</v>
+        <v>753</v>
       </c>
       <c r="C386">
         <v>1</v>
@@ -13245,16 +13392,16 @@
         <v>128</v>
       </c>
       <c r="E386" t="s">
-        <v>748</v>
+        <v>16</v>
       </c>
       <c r="F386" t="s">
-        <v>749</v>
+        <v>17</v>
       </c>
       <c r="G386" s="1">
         <v>46311</v>
       </c>
       <c r="H386" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="387" spans="1:8" x14ac:dyDescent="0.2">
@@ -13262,7 +13409,7 @@
         <v>0</v>
       </c>
       <c r="B387" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="C387">
         <v>1</v>
@@ -13271,16 +13418,16 @@
         <v>128</v>
       </c>
       <c r="E387" t="s">
-        <v>751</v>
+        <v>3</v>
       </c>
       <c r="F387" t="s">
-        <v>752</v>
+        <v>4</v>
       </c>
       <c r="G387" s="1">
         <v>46311</v>
       </c>
       <c r="H387" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="388" spans="1:8" x14ac:dyDescent="0.2">
@@ -13288,7 +13435,7 @@
         <v>0</v>
       </c>
       <c r="B388" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="C388">
         <v>1</v>
@@ -13297,16 +13444,16 @@
         <v>128</v>
       </c>
       <c r="E388" t="s">
-        <v>340</v>
+        <v>741</v>
       </c>
       <c r="F388" t="s">
-        <v>341</v>
+        <v>742</v>
       </c>
       <c r="G388" s="1">
         <v>46311</v>
       </c>
       <c r="H388" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="389" spans="1:8" x14ac:dyDescent="0.2">
@@ -13314,7 +13461,7 @@
         <v>0</v>
       </c>
       <c r="B389" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="C389">
         <v>1</v>
@@ -13323,13 +13470,13 @@
         <v>128</v>
       </c>
       <c r="E389" t="s">
-        <v>45</v>
+        <v>572</v>
       </c>
       <c r="F389" t="s">
-        <v>46</v>
+        <v>573</v>
       </c>
       <c r="G389" s="1">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="H389" s="1">
         <v>46314</v>
@@ -13340,7 +13487,7 @@
         <v>0</v>
       </c>
       <c r="B390" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="C390">
         <v>1</v>
@@ -13349,13 +13496,13 @@
         <v>128</v>
       </c>
       <c r="E390" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="F390" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="G390" s="1">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="H390" s="1">
         <v>46314</v>
@@ -13366,7 +13513,7 @@
         <v>0</v>
       </c>
       <c r="B391" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C391">
         <v>1</v>
@@ -13375,13 +13522,13 @@
         <v>128</v>
       </c>
       <c r="E391" t="s">
-        <v>496</v>
+        <v>761</v>
       </c>
       <c r="F391" t="s">
-        <v>497</v>
+        <v>762</v>
       </c>
       <c r="G391" s="1">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="H391" s="1">
         <v>46314</v>
@@ -13392,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="B392" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="C392">
         <v>1</v>
@@ -13401,13 +13548,13 @@
         <v>128</v>
       </c>
       <c r="E392" t="s">
-        <v>282</v>
+        <v>764</v>
       </c>
       <c r="F392" t="s">
-        <v>283</v>
+        <v>765</v>
       </c>
       <c r="G392" s="1">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="H392" s="1">
         <v>46314</v>
@@ -13418,7 +13565,7 @@
         <v>0</v>
       </c>
       <c r="B393" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="C393">
         <v>1</v>
@@ -13427,13 +13574,13 @@
         <v>128</v>
       </c>
       <c r="E393" t="s">
-        <v>282</v>
+        <v>340</v>
       </c>
       <c r="F393" t="s">
-        <v>283</v>
+        <v>341</v>
       </c>
       <c r="G393" s="1">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="H393" s="1">
         <v>46314</v>
@@ -13444,7 +13591,7 @@
         <v>0</v>
       </c>
       <c r="B394" t="s">
-        <v>761</v>
+        <v>767</v>
       </c>
       <c r="C394">
         <v>1</v>
@@ -13453,10 +13600,10 @@
         <v>128</v>
       </c>
       <c r="E394" t="s">
-        <v>762</v>
+        <v>45</v>
       </c>
       <c r="F394" t="s">
-        <v>763</v>
+        <v>46</v>
       </c>
       <c r="G394" s="1">
         <v>46312</v>
@@ -13470,7 +13617,7 @@
         <v>0</v>
       </c>
       <c r="B395" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="C395">
         <v>1</v>
@@ -13479,10 +13626,10 @@
         <v>128</v>
       </c>
       <c r="E395" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="F395" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="G395" s="1">
         <v>46312</v>
@@ -13496,7 +13643,7 @@
         <v>0</v>
       </c>
       <c r="B396" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="C396">
         <v>1</v>
@@ -13505,10 +13652,10 @@
         <v>128</v>
       </c>
       <c r="E396" t="s">
-        <v>768</v>
+        <v>496</v>
       </c>
       <c r="F396" t="s">
-        <v>769</v>
+        <v>497</v>
       </c>
       <c r="G396" s="1">
         <v>46312</v>
@@ -13522,7 +13669,7 @@
         <v>0</v>
       </c>
       <c r="B397" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="C397">
         <v>1</v>
@@ -13531,10 +13678,10 @@
         <v>128</v>
       </c>
       <c r="E397" t="s">
-        <v>771</v>
+        <v>282</v>
       </c>
       <c r="F397" t="s">
-        <v>772</v>
+        <v>283</v>
       </c>
       <c r="G397" s="1">
         <v>46312</v>
@@ -13557,10 +13704,10 @@
         <v>128</v>
       </c>
       <c r="E398" t="s">
-        <v>774</v>
+        <v>282</v>
       </c>
       <c r="F398" t="s">
-        <v>775</v>
+        <v>283</v>
       </c>
       <c r="G398" s="1">
         <v>46312</v>
@@ -13574,19 +13721,19 @@
         <v>0</v>
       </c>
       <c r="B399" t="s">
+        <v>774</v>
+      </c>
+      <c r="C399">
+        <v>1</v>
+      </c>
+      <c r="D399" t="s">
+        <v>128</v>
+      </c>
+      <c r="E399" t="s">
+        <v>775</v>
+      </c>
+      <c r="F399" t="s">
         <v>776</v>
-      </c>
-      <c r="C399">
-        <v>1</v>
-      </c>
-      <c r="D399" t="s">
-        <v>128</v>
-      </c>
-      <c r="E399" t="s">
-        <v>777</v>
-      </c>
-      <c r="F399" t="s">
-        <v>778</v>
       </c>
       <c r="G399" s="1">
         <v>46312</v>
@@ -13600,19 +13747,19 @@
         <v>0</v>
       </c>
       <c r="B400" t="s">
+        <v>777</v>
+      </c>
+      <c r="C400">
+        <v>1</v>
+      </c>
+      <c r="D400" t="s">
+        <v>128</v>
+      </c>
+      <c r="E400" t="s">
+        <v>778</v>
+      </c>
+      <c r="F400" t="s">
         <v>779</v>
-      </c>
-      <c r="C400">
-        <v>1</v>
-      </c>
-      <c r="D400" t="s">
-        <v>128</v>
-      </c>
-      <c r="E400" t="s">
-        <v>396</v>
-      </c>
-      <c r="F400" t="s">
-        <v>397</v>
       </c>
       <c r="G400" s="1">
         <v>46312</v>
@@ -13635,10 +13782,10 @@
         <v>128</v>
       </c>
       <c r="E401" t="s">
-        <v>396</v>
+        <v>781</v>
       </c>
       <c r="F401" t="s">
-        <v>397</v>
+        <v>782</v>
       </c>
       <c r="G401" s="1">
         <v>46312</v>
@@ -13652,7 +13799,7 @@
         <v>0</v>
       </c>
       <c r="B402" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="C402">
         <v>1</v>
@@ -13661,10 +13808,10 @@
         <v>128</v>
       </c>
       <c r="E402" t="s">
-        <v>722</v>
+        <v>784</v>
       </c>
       <c r="F402" t="s">
-        <v>723</v>
+        <v>785</v>
       </c>
       <c r="G402" s="1">
         <v>46312</v>
@@ -13678,7 +13825,7 @@
         <v>0</v>
       </c>
       <c r="B403" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="C403">
         <v>1</v>
@@ -13687,10 +13834,10 @@
         <v>128</v>
       </c>
       <c r="E403" t="s">
-        <v>624</v>
+        <v>787</v>
       </c>
       <c r="F403" t="s">
-        <v>625</v>
+        <v>788</v>
       </c>
       <c r="G403" s="1">
         <v>46312</v>
@@ -13704,7 +13851,7 @@
         <v>0</v>
       </c>
       <c r="B404" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="C404">
         <v>1</v>
@@ -13713,13 +13860,13 @@
         <v>128</v>
       </c>
       <c r="E404" t="s">
-        <v>784</v>
+        <v>790</v>
       </c>
       <c r="F404" t="s">
-        <v>785</v>
+        <v>791</v>
       </c>
       <c r="G404" s="1">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="H404" s="1">
         <v>46314</v>
@@ -13730,7 +13877,7 @@
         <v>0</v>
       </c>
       <c r="B405" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
       <c r="C405">
         <v>1</v>
@@ -13739,13 +13886,13 @@
         <v>128</v>
       </c>
       <c r="E405" t="s">
-        <v>57</v>
+        <v>793</v>
       </c>
       <c r="F405" t="s">
-        <v>58</v>
+        <v>794</v>
       </c>
       <c r="G405" s="1">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="H405" s="1">
         <v>46314</v>
@@ -13756,7 +13903,7 @@
         <v>0</v>
       </c>
       <c r="B406" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
       <c r="C406">
         <v>1</v>
@@ -13765,13 +13912,13 @@
         <v>128</v>
       </c>
       <c r="E406" t="s">
-        <v>788</v>
+        <v>396</v>
       </c>
       <c r="F406" t="s">
-        <v>789</v>
+        <v>397</v>
       </c>
       <c r="G406" s="1">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="H406" s="1">
         <v>46314</v>
@@ -13782,7 +13929,7 @@
         <v>0</v>
       </c>
       <c r="B407" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="C407">
         <v>1</v>
@@ -13791,13 +13938,13 @@
         <v>128</v>
       </c>
       <c r="E407" t="s">
-        <v>195</v>
+        <v>396</v>
       </c>
       <c r="F407" t="s">
-        <v>196</v>
+        <v>397</v>
       </c>
       <c r="G407" s="1">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="H407" s="1">
         <v>46314</v>
@@ -13808,7 +13955,7 @@
         <v>0</v>
       </c>
       <c r="B408" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
       <c r="C408">
         <v>1</v>
@@ -13817,13 +13964,13 @@
         <v>128</v>
       </c>
       <c r="E408" t="s">
-        <v>195</v>
+        <v>734</v>
       </c>
       <c r="F408" t="s">
-        <v>196</v>
+        <v>735</v>
       </c>
       <c r="G408" s="1">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="H408" s="1">
         <v>46314</v>
@@ -13834,7 +13981,7 @@
         <v>0</v>
       </c>
       <c r="B409" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
       <c r="C409">
         <v>1</v>
@@ -13843,13 +13990,13 @@
         <v>128</v>
       </c>
       <c r="E409" t="s">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="F409" t="s">
-        <v>93</v>
+        <v>119</v>
       </c>
       <c r="G409" s="1">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="H409" s="1">
         <v>46314</v>
@@ -13860,22 +14007,22 @@
         <v>0</v>
       </c>
       <c r="B410" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="C410">
         <v>1</v>
       </c>
       <c r="D410" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E410" t="s">
-        <v>762</v>
+        <v>624</v>
       </c>
       <c r="F410" t="s">
-        <v>763</v>
+        <v>625</v>
       </c>
       <c r="G410" s="1">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="H410" s="1">
         <v>46314</v>
@@ -13886,7 +14033,7 @@
         <v>0</v>
       </c>
       <c r="B411" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
       <c r="C411">
         <v>1</v>
@@ -13895,10 +14042,10 @@
         <v>128</v>
       </c>
       <c r="E411" t="s">
-        <v>795</v>
+        <v>801</v>
       </c>
       <c r="F411" t="s">
-        <v>796</v>
+        <v>802</v>
       </c>
       <c r="G411" s="1">
         <v>46314</v>
@@ -13912,7 +14059,7 @@
         <v>0</v>
       </c>
       <c r="B412" t="s">
-        <v>797</v>
+        <v>803</v>
       </c>
       <c r="C412">
         <v>1</v>
@@ -13921,10 +14068,10 @@
         <v>128</v>
       </c>
       <c r="E412" t="s">
-        <v>798</v>
+        <v>57</v>
       </c>
       <c r="F412" t="s">
-        <v>799</v>
+        <v>58</v>
       </c>
       <c r="G412" s="1">
         <v>46314</v>
@@ -13938,7 +14085,7 @@
         <v>0</v>
       </c>
       <c r="B413" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C413">
         <v>1</v>
@@ -13947,10 +14094,10 @@
         <v>128</v>
       </c>
       <c r="E413" t="s">
-        <v>41</v>
+        <v>805</v>
       </c>
       <c r="F413" t="s">
-        <v>42</v>
+        <v>806</v>
       </c>
       <c r="G413" s="1">
         <v>46314</v>
@@ -13964,7 +14111,7 @@
         <v>0</v>
       </c>
       <c r="B414" t="s">
-        <v>801</v>
+        <v>807</v>
       </c>
       <c r="C414">
         <v>1</v>
@@ -13973,10 +14120,10 @@
         <v>128</v>
       </c>
       <c r="E414" t="s">
-        <v>802</v>
+        <v>195</v>
       </c>
       <c r="F414" t="s">
-        <v>803</v>
+        <v>196</v>
       </c>
       <c r="G414" s="1">
         <v>46314</v>
@@ -13990,7 +14137,7 @@
         <v>0</v>
       </c>
       <c r="B415" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C415">
         <v>1</v>
@@ -13999,10 +14146,10 @@
         <v>128</v>
       </c>
       <c r="E415" t="s">
-        <v>805</v>
+        <v>195</v>
       </c>
       <c r="F415" t="s">
-        <v>806</v>
+        <v>196</v>
       </c>
       <c r="G415" s="1">
         <v>46314</v>
@@ -14016,7 +14163,7 @@
         <v>0</v>
       </c>
       <c r="B416" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="C416">
         <v>1</v>
@@ -14025,10 +14172,10 @@
         <v>128</v>
       </c>
       <c r="E416" t="s">
-        <v>808</v>
+        <v>92</v>
       </c>
       <c r="F416" t="s">
-        <v>809</v>
+        <v>93</v>
       </c>
       <c r="G416" s="1">
         <v>46314</v>
@@ -14051,10 +14198,10 @@
         <v>128</v>
       </c>
       <c r="E417" t="s">
-        <v>811</v>
+        <v>775</v>
       </c>
       <c r="F417" t="s">
-        <v>812</v>
+        <v>776</v>
       </c>
       <c r="G417" s="1">
         <v>46314</v>
@@ -14068,19 +14215,19 @@
         <v>0</v>
       </c>
       <c r="B418" t="s">
+        <v>811</v>
+      </c>
+      <c r="C418">
+        <v>1</v>
+      </c>
+      <c r="D418" t="s">
+        <v>128</v>
+      </c>
+      <c r="E418" t="s">
+        <v>812</v>
+      </c>
+      <c r="F418" t="s">
         <v>813</v>
-      </c>
-      <c r="C418">
-        <v>1</v>
-      </c>
-      <c r="D418" t="s">
-        <v>128</v>
-      </c>
-      <c r="E418" t="s">
-        <v>80</v>
-      </c>
-      <c r="F418" t="s">
-        <v>81</v>
       </c>
       <c r="G418" s="1">
         <v>46314</v>
@@ -14129,10 +14276,10 @@
         <v>128</v>
       </c>
       <c r="E420" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="F420" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="G420" s="1">
         <v>46314</v>
@@ -14143,62 +14290,62 @@
     </row>
     <row r="421" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A421" t="s">
+        <v>0</v>
+      </c>
+      <c r="B421" t="s">
         <v>818</v>
       </c>
-      <c r="B421" t="s">
+      <c r="C421">
+        <v>1</v>
+      </c>
+      <c r="D421" t="s">
+        <v>128</v>
+      </c>
+      <c r="E421" t="s">
         <v>819</v>
       </c>
-      <c r="C421">
-        <v>1</v>
-      </c>
-      <c r="D421" t="s">
-        <v>2</v>
-      </c>
-      <c r="E421" t="s">
-        <v>160</v>
-      </c>
       <c r="F421" t="s">
-        <v>161</v>
+        <v>820</v>
       </c>
       <c r="G421" s="1">
-        <v>46148</v>
+        <v>46314</v>
       </c>
       <c r="H421" s="1">
-        <v>46149</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="422" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A422" t="s">
-        <v>818</v>
+        <v>0</v>
       </c>
       <c r="B422" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="C422">
         <v>1</v>
       </c>
       <c r="D422" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E422" t="s">
-        <v>408</v>
+        <v>822</v>
       </c>
       <c r="F422" t="s">
-        <v>409</v>
+        <v>823</v>
       </c>
       <c r="G422" s="1">
-        <v>46268</v>
+        <v>46314</v>
       </c>
       <c r="H422" s="1">
-        <v>46268</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="423" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A423" t="s">
-        <v>818</v>
+        <v>0</v>
       </c>
       <c r="B423" t="s">
-        <v>821</v>
+        <v>824</v>
       </c>
       <c r="C423">
         <v>1</v>
@@ -14207,24 +14354,24 @@
         <v>128</v>
       </c>
       <c r="E423" t="s">
-        <v>80</v>
+        <v>825</v>
       </c>
       <c r="F423" t="s">
-        <v>81</v>
+        <v>826</v>
       </c>
       <c r="G423" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="H423" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="424" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A424" t="s">
-        <v>818</v>
+        <v>0</v>
       </c>
       <c r="B424" t="s">
-        <v>822</v>
+        <v>827</v>
       </c>
       <c r="C424">
         <v>1</v>
@@ -14233,24 +14380,24 @@
         <v>128</v>
       </c>
       <c r="E424" t="s">
-        <v>823</v>
+        <v>828</v>
       </c>
       <c r="F424" t="s">
-        <v>824</v>
+        <v>829</v>
       </c>
       <c r="G424" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="H424" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="425" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A425" t="s">
-        <v>825</v>
+        <v>0</v>
       </c>
       <c r="B425" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
       <c r="C425">
         <v>1</v>
@@ -14259,195 +14406,195 @@
         <v>128</v>
       </c>
       <c r="E425" t="s">
-        <v>827</v>
+        <v>80</v>
       </c>
       <c r="F425" t="s">
-        <v>828</v>
+        <v>81</v>
       </c>
       <c r="G425" s="1">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="H425" s="1">
-        <v>46308</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="426" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A426" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B426" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="C426">
         <v>1</v>
       </c>
       <c r="D426" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E426" t="s">
-        <v>41</v>
+        <v>832</v>
       </c>
       <c r="F426" t="s">
-        <v>42</v>
+        <v>833</v>
       </c>
       <c r="G426" s="1">
-        <v>46133</v>
+        <v>46314</v>
       </c>
       <c r="H426" s="1">
-        <v>46134</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="427" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A427" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B427" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
       <c r="C427">
         <v>1</v>
       </c>
       <c r="D427" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E427" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="F427" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="G427" s="1">
-        <v>46134</v>
+        <v>46314</v>
       </c>
       <c r="H427" s="1">
-        <v>46134</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="428" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A428" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B428" t="s">
-        <v>832</v>
+        <v>835</v>
       </c>
       <c r="C428">
         <v>1</v>
       </c>
       <c r="D428" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E428" t="s">
-        <v>19</v>
+        <v>591</v>
       </c>
       <c r="F428" t="s">
-        <v>20</v>
+        <v>592</v>
       </c>
       <c r="G428" s="1">
-        <v>46156</v>
+        <v>46314</v>
       </c>
       <c r="H428" s="1">
-        <v>46156</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="429" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A429" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B429" t="s">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="C429">
         <v>1</v>
       </c>
       <c r="D429" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E429" t="s">
-        <v>834</v>
+        <v>591</v>
       </c>
       <c r="F429" t="s">
-        <v>835</v>
+        <v>592</v>
       </c>
       <c r="G429" s="1">
-        <v>46213</v>
+        <v>46314</v>
       </c>
       <c r="H429" s="1">
-        <v>46213</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="430" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A430" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B430" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="C430">
         <v>1</v>
       </c>
       <c r="D430" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E430" t="s">
-        <v>725</v>
+        <v>514</v>
       </c>
       <c r="F430" t="s">
-        <v>726</v>
+        <v>515</v>
       </c>
       <c r="G430" s="1">
-        <v>46253</v>
+        <v>46314</v>
       </c>
       <c r="H430" s="1">
-        <v>46253</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="431" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A431" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B431" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="C431">
         <v>1</v>
       </c>
       <c r="D431" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E431" t="s">
-        <v>172</v>
+        <v>313</v>
       </c>
       <c r="F431" t="s">
-        <v>173</v>
+        <v>314</v>
       </c>
       <c r="G431" s="1">
-        <v>46273</v>
+        <v>46314</v>
       </c>
       <c r="H431" s="1">
-        <v>46274</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="432" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A432" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B432" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="C432">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D432" t="s">
         <v>128</v>
       </c>
       <c r="E432" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="F432" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="G432" s="1">
-        <v>46300</v>
+        <v>46314</v>
       </c>
       <c r="H432" s="1">
         <v>46314</v>
@@ -14455,181 +14602,181 @@
     </row>
     <row r="433" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A433" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B433" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="C433">
         <v>1</v>
       </c>
       <c r="D433" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E433" t="s">
-        <v>182</v>
+        <v>843</v>
       </c>
       <c r="F433" t="s">
-        <v>183</v>
+        <v>844</v>
       </c>
       <c r="G433" s="1">
-        <v>46300</v>
+        <v>46314</v>
       </c>
       <c r="H433" s="1">
-        <v>46300</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="434" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A434" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B434" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="C434">
         <v>1</v>
       </c>
       <c r="D434" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E434" t="s">
-        <v>823</v>
+        <v>846</v>
       </c>
       <c r="F434" t="s">
-        <v>824</v>
+        <v>847</v>
       </c>
       <c r="G434" s="1">
-        <v>46300</v>
+        <v>46314</v>
       </c>
       <c r="H434" s="1">
-        <v>46301</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="435" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A435" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B435" t="s">
-        <v>843</v>
+        <v>848</v>
       </c>
       <c r="C435">
         <v>1</v>
       </c>
       <c r="D435" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E435" t="s">
-        <v>301</v>
+        <v>215</v>
       </c>
       <c r="F435" t="s">
-        <v>302</v>
+        <v>216</v>
       </c>
       <c r="G435" s="1">
-        <v>46302</v>
+        <v>46314</v>
       </c>
       <c r="H435" s="1">
-        <v>46302</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="436" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A436" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B436" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="C436">
         <v>1</v>
       </c>
       <c r="D436" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E436" t="s">
-        <v>703</v>
+        <v>850</v>
       </c>
       <c r="F436" t="s">
-        <v>704</v>
+        <v>851</v>
       </c>
       <c r="G436" s="1">
-        <v>46303</v>
+        <v>46314</v>
       </c>
       <c r="H436" s="1">
-        <v>46303</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="437" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A437" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B437" t="s">
-        <v>845</v>
+        <v>852</v>
       </c>
       <c r="C437">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D437" t="s">
         <v>128</v>
       </c>
       <c r="E437" t="s">
-        <v>149</v>
+        <v>185</v>
       </c>
       <c r="F437" t="s">
-        <v>150</v>
+        <v>186</v>
       </c>
       <c r="G437" s="1">
-        <v>46303</v>
+        <v>46314</v>
       </c>
       <c r="H437" s="1">
-        <v>46308</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="438" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A438" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B438" t="s">
-        <v>846</v>
+        <v>853</v>
       </c>
       <c r="C438">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D438" t="s">
         <v>128</v>
       </c>
       <c r="E438" t="s">
-        <v>784</v>
+        <v>854</v>
       </c>
       <c r="F438" t="s">
-        <v>785</v>
+        <v>855</v>
       </c>
       <c r="G438" s="1">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="H438" s="1">
-        <v>46309</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="439" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A439" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B439" t="s">
-        <v>847</v>
+        <v>856</v>
       </c>
       <c r="C439">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D439" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E439" t="s">
-        <v>784</v>
+        <v>857</v>
       </c>
       <c r="F439" t="s">
-        <v>785</v>
+        <v>858</v>
       </c>
       <c r="G439" s="1">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="H439" s="1">
         <v>46314</v>
@@ -14637,10 +14784,10 @@
     </row>
     <row r="440" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A440" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B440" t="s">
-        <v>848</v>
+        <v>859</v>
       </c>
       <c r="C440">
         <v>1</v>
@@ -14649,39 +14796,39 @@
         <v>128</v>
       </c>
       <c r="E440" t="s">
-        <v>487</v>
+        <v>83</v>
       </c>
       <c r="F440" t="s">
-        <v>488</v>
+        <v>84</v>
       </c>
       <c r="G440" s="1">
-        <v>46309</v>
+        <v>46314</v>
       </c>
       <c r="H440" s="1">
-        <v>46309</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="441" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A441" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B441" t="s">
-        <v>849</v>
+        <v>860</v>
       </c>
       <c r="C441">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D441" t="s">
         <v>128</v>
       </c>
       <c r="E441" t="s">
-        <v>594</v>
+        <v>83</v>
       </c>
       <c r="F441" t="s">
-        <v>595</v>
+        <v>84</v>
       </c>
       <c r="G441" s="1">
-        <v>46310</v>
+        <v>46314</v>
       </c>
       <c r="H441" s="1">
         <v>46314</v>
@@ -14689,10 +14836,10 @@
     </row>
     <row r="442" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A442" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B442" t="s">
-        <v>850</v>
+        <v>861</v>
       </c>
       <c r="C442">
         <v>1</v>
@@ -14701,24 +14848,24 @@
         <v>128</v>
       </c>
       <c r="E442" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="F442" t="s">
-        <v>150</v>
+        <v>17</v>
       </c>
       <c r="G442" s="1">
-        <v>46310</v>
+        <v>46314</v>
       </c>
       <c r="H442" s="1">
-        <v>46310</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="443" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A443" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B443" t="s">
-        <v>851</v>
+        <v>862</v>
       </c>
       <c r="C443">
         <v>1</v>
@@ -14727,24 +14874,24 @@
         <v>128</v>
       </c>
       <c r="E443" t="s">
-        <v>41</v>
+        <v>405</v>
       </c>
       <c r="F443" t="s">
-        <v>42</v>
+        <v>406</v>
       </c>
       <c r="G443" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="H443" s="1">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="444" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A444" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B444" t="s">
-        <v>852</v>
+        <v>863</v>
       </c>
       <c r="C444">
         <v>1</v>
@@ -14753,10 +14900,10 @@
         <v>128</v>
       </c>
       <c r="E444" t="s">
-        <v>784</v>
+        <v>864</v>
       </c>
       <c r="F444" t="s">
-        <v>785</v>
+        <v>865</v>
       </c>
       <c r="G444" s="1">
         <v>46314</v>
@@ -14767,10 +14914,10 @@
     </row>
     <row r="445" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A445" t="s">
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="B445" t="s">
-        <v>853</v>
+        <v>866</v>
       </c>
       <c r="C445">
         <v>1</v>
@@ -14779,10 +14926,10 @@
         <v>128</v>
       </c>
       <c r="E445" t="s">
-        <v>854</v>
+        <v>16</v>
       </c>
       <c r="F445" t="s">
-        <v>855</v>
+        <v>17</v>
       </c>
       <c r="G445" s="1">
         <v>46314</v>
@@ -14793,88 +14940,88 @@
     </row>
     <row r="446" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A446" t="s">
-        <v>856</v>
+        <v>0</v>
       </c>
       <c r="B446" t="s">
-        <v>857</v>
+        <v>867</v>
       </c>
       <c r="C446">
         <v>1</v>
       </c>
       <c r="D446" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E446" t="s">
-        <v>858</v>
+        <v>16</v>
       </c>
       <c r="F446" t="s">
-        <v>859</v>
+        <v>17</v>
       </c>
       <c r="G446" s="1">
-        <v>46063</v>
+        <v>46314</v>
       </c>
       <c r="H446" s="1">
-        <v>46064</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="447" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A447" t="s">
-        <v>856</v>
+        <v>0</v>
       </c>
       <c r="B447" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
       <c r="C447">
         <v>1</v>
       </c>
       <c r="D447" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E447" t="s">
-        <v>57</v>
+        <v>493</v>
       </c>
       <c r="F447" t="s">
-        <v>58</v>
+        <v>494</v>
       </c>
       <c r="G447" s="1">
-        <v>46113</v>
+        <v>46314</v>
       </c>
       <c r="H447" s="1">
-        <v>46125</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="448" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A448" t="s">
-        <v>856</v>
+        <v>0</v>
       </c>
       <c r="B448" t="s">
-        <v>861</v>
+        <v>869</v>
       </c>
       <c r="C448">
         <v>1</v>
       </c>
       <c r="D448" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E448" t="s">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="F448" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="G448" s="1">
-        <v>46125</v>
+        <v>46314</v>
       </c>
       <c r="H448" s="1">
-        <v>46125</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="449" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A449" t="s">
-        <v>856</v>
+        <v>870</v>
       </c>
       <c r="B449" t="s">
-        <v>862</v>
+        <v>871</v>
       </c>
       <c r="C449">
         <v>1</v>
@@ -14883,24 +15030,24 @@
         <v>2</v>
       </c>
       <c r="E449" t="s">
-        <v>57</v>
+        <v>160</v>
       </c>
       <c r="F449" t="s">
-        <v>58</v>
+        <v>161</v>
       </c>
       <c r="G449" s="1">
-        <v>46126</v>
+        <v>46148</v>
       </c>
       <c r="H449" s="1">
-        <v>46126</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="450" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A450" t="s">
-        <v>856</v>
+        <v>870</v>
       </c>
       <c r="B450" t="s">
-        <v>863</v>
+        <v>872</v>
       </c>
       <c r="C450">
         <v>1</v>
@@ -14909,154 +15056,154 @@
         <v>2</v>
       </c>
       <c r="E450" t="s">
-        <v>57</v>
+        <v>408</v>
       </c>
       <c r="F450" t="s">
-        <v>58</v>
+        <v>409</v>
       </c>
       <c r="G450" s="1">
-        <v>46126</v>
+        <v>46268</v>
       </c>
       <c r="H450" s="1">
-        <v>46126</v>
+        <v>46268</v>
       </c>
     </row>
     <row r="451" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A451" t="s">
-        <v>856</v>
+        <v>870</v>
       </c>
       <c r="B451" t="s">
-        <v>864</v>
+        <v>873</v>
       </c>
       <c r="C451">
         <v>1</v>
       </c>
       <c r="D451" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E451" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="F451" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="G451" s="1">
-        <v>46128</v>
+        <v>46311</v>
       </c>
       <c r="H451" s="1">
-        <v>46128</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="452" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A452" t="s">
-        <v>856</v>
+        <v>870</v>
       </c>
       <c r="B452" t="s">
-        <v>865</v>
+        <v>874</v>
       </c>
       <c r="C452">
         <v>1</v>
       </c>
       <c r="D452" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E452" t="s">
-        <v>57</v>
+        <v>875</v>
       </c>
       <c r="F452" t="s">
-        <v>58</v>
+        <v>876</v>
       </c>
       <c r="G452" s="1">
-        <v>46132</v>
+        <v>46311</v>
       </c>
       <c r="H452" s="1">
-        <v>46132</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="453" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A453" t="s">
-        <v>856</v>
+        <v>877</v>
       </c>
       <c r="B453" t="s">
-        <v>866</v>
+        <v>878</v>
       </c>
       <c r="C453">
         <v>1</v>
       </c>
       <c r="D453" t="s">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="E453" t="s">
-        <v>57</v>
+        <v>879</v>
       </c>
       <c r="F453" t="s">
-        <v>58</v>
+        <v>880</v>
       </c>
       <c r="G453" s="1">
-        <v>46161</v>
+        <v>46308</v>
       </c>
       <c r="H453" s="1">
-        <v>46161</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="454" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A454" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B454" t="s">
-        <v>867</v>
+        <v>882</v>
       </c>
       <c r="C454">
         <v>1</v>
       </c>
       <c r="D454" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E454" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="F454" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="G454" s="1">
-        <v>46174</v>
+        <v>46133</v>
       </c>
       <c r="H454" s="1">
-        <v>46174</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="455" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A455" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B455" t="s">
-        <v>868</v>
+        <v>883</v>
       </c>
       <c r="C455">
         <v>1</v>
       </c>
       <c r="D455" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E455" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="F455" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="G455" s="1">
-        <v>46174</v>
+        <v>46134</v>
       </c>
       <c r="H455" s="1">
-        <v>46174</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="456" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A456" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B456" t="s">
-        <v>869</v>
+        <v>884</v>
       </c>
       <c r="C456">
         <v>1</v>
@@ -15065,24 +15212,24 @@
         <v>6</v>
       </c>
       <c r="E456" t="s">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="F456" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="G456" s="1">
-        <v>46195</v>
+        <v>46156</v>
       </c>
       <c r="H456" s="1">
-        <v>46252</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="457" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A457" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B457" t="s">
-        <v>870</v>
+        <v>885</v>
       </c>
       <c r="C457">
         <v>1</v>
@@ -15091,180 +15238,180 @@
         <v>6</v>
       </c>
       <c r="E457" t="s">
-        <v>57</v>
+        <v>886</v>
       </c>
       <c r="F457" t="s">
-        <v>58</v>
+        <v>887</v>
       </c>
       <c r="G457" s="1">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="H457" s="1">
-        <v>46210</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="458" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A458" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B458" t="s">
-        <v>871</v>
+        <v>888</v>
       </c>
       <c r="C458">
         <v>1</v>
       </c>
       <c r="D458" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E458" t="s">
-        <v>57</v>
+        <v>738</v>
       </c>
       <c r="F458" t="s">
-        <v>58</v>
+        <v>739</v>
       </c>
       <c r="G458" s="1">
-        <v>46213</v>
+        <v>46253</v>
       </c>
       <c r="H458" s="1">
-        <v>46213</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="459" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A459" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B459" t="s">
-        <v>872</v>
+        <v>889</v>
       </c>
       <c r="C459">
         <v>1</v>
       </c>
       <c r="D459" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E459" t="s">
-        <v>57</v>
+        <v>172</v>
       </c>
       <c r="F459" t="s">
-        <v>58</v>
+        <v>173</v>
       </c>
       <c r="G459" s="1">
-        <v>46218</v>
+        <v>46273</v>
       </c>
       <c r="H459" s="1">
-        <v>46252</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="460" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A460" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B460" t="s">
-        <v>873</v>
+        <v>890</v>
       </c>
       <c r="C460">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D460" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E460" t="s">
-        <v>77</v>
+        <v>891</v>
       </c>
       <c r="F460" t="s">
-        <v>78</v>
+        <v>892</v>
       </c>
       <c r="G460" s="1">
-        <v>46226</v>
+        <v>46300</v>
       </c>
       <c r="H460" s="1">
-        <v>46226</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="461" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A461" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B461" t="s">
-        <v>874</v>
+        <v>893</v>
       </c>
       <c r="C461">
         <v>1</v>
       </c>
       <c r="D461" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E461" t="s">
-        <v>57</v>
+        <v>182</v>
       </c>
       <c r="F461" t="s">
-        <v>58</v>
+        <v>183</v>
       </c>
       <c r="G461" s="1">
-        <v>46227</v>
+        <v>46300</v>
       </c>
       <c r="H461" s="1">
-        <v>46252</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="462" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A462" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B462" t="s">
+        <v>894</v>
+      </c>
+      <c r="C462">
+        <v>1</v>
+      </c>
+      <c r="D462" t="s">
+        <v>2</v>
+      </c>
+      <c r="E462" t="s">
         <v>875</v>
       </c>
-      <c r="C462">
-        <v>1</v>
-      </c>
-      <c r="D462" t="s">
-        <v>6</v>
-      </c>
-      <c r="E462" t="s">
-        <v>57</v>
-      </c>
       <c r="F462" t="s">
-        <v>58</v>
+        <v>876</v>
       </c>
       <c r="G462" s="1">
-        <v>46227</v>
+        <v>46300</v>
       </c>
       <c r="H462" s="1">
-        <v>46252</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="463" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A463" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B463" t="s">
-        <v>876</v>
+        <v>895</v>
       </c>
       <c r="C463">
         <v>1</v>
       </c>
       <c r="D463" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E463" t="s">
-        <v>57</v>
+        <v>301</v>
       </c>
       <c r="F463" t="s">
-        <v>58</v>
+        <v>302</v>
       </c>
       <c r="G463" s="1">
-        <v>46227</v>
+        <v>46302</v>
       </c>
       <c r="H463" s="1">
-        <v>46228</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="464" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A464" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B464" t="s">
-        <v>877</v>
+        <v>896</v>
       </c>
       <c r="C464">
         <v>1</v>
@@ -15273,180 +15420,180 @@
         <v>6</v>
       </c>
       <c r="E464" t="s">
-        <v>77</v>
+        <v>706</v>
       </c>
       <c r="F464" t="s">
-        <v>78</v>
+        <v>707</v>
       </c>
       <c r="G464" s="1">
-        <v>46230</v>
+        <v>46303</v>
       </c>
       <c r="H464" s="1">
-        <v>46252</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="465" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A465" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B465" t="s">
-        <v>878</v>
+        <v>897</v>
       </c>
       <c r="C465">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D465" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E465" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="F465" t="s">
-        <v>58</v>
+        <v>150</v>
       </c>
       <c r="G465" s="1">
-        <v>46231</v>
+        <v>46303</v>
       </c>
       <c r="H465" s="1">
-        <v>46231</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="466" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A466" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B466" t="s">
-        <v>879</v>
+        <v>898</v>
       </c>
       <c r="C466">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D466" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E466" t="s">
-        <v>57</v>
+        <v>801</v>
       </c>
       <c r="F466" t="s">
-        <v>58</v>
+        <v>802</v>
       </c>
       <c r="G466" s="1">
-        <v>46254</v>
+        <v>46308</v>
       </c>
       <c r="H466" s="1">
-        <v>46254</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="467" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A467" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B467" t="s">
-        <v>880</v>
+        <v>899</v>
       </c>
       <c r="C467">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D467" t="s">
         <v>2</v>
       </c>
       <c r="E467" t="s">
-        <v>57</v>
+        <v>801</v>
       </c>
       <c r="F467" t="s">
-        <v>58</v>
+        <v>802</v>
       </c>
       <c r="G467" s="1">
-        <v>46255</v>
+        <v>46308</v>
       </c>
       <c r="H467" s="1">
-        <v>46255</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="468" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A468" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B468" t="s">
-        <v>881</v>
+        <v>900</v>
       </c>
       <c r="C468">
         <v>1</v>
       </c>
       <c r="D468" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E468" t="s">
-        <v>57</v>
+        <v>487</v>
       </c>
       <c r="F468" t="s">
-        <v>58</v>
+        <v>488</v>
       </c>
       <c r="G468" s="1">
-        <v>46260</v>
+        <v>46309</v>
       </c>
       <c r="H468" s="1">
-        <v>46260</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="469" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A469" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B469" t="s">
-        <v>882</v>
+        <v>901</v>
       </c>
       <c r="C469">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D469" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E469" t="s">
-        <v>57</v>
+        <v>594</v>
       </c>
       <c r="F469" t="s">
-        <v>58</v>
+        <v>595</v>
       </c>
       <c r="G469" s="1">
-        <v>46289</v>
+        <v>46310</v>
       </c>
       <c r="H469" s="1">
-        <v>46289</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="470" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A470" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B470" t="s">
-        <v>883</v>
+        <v>902</v>
       </c>
       <c r="C470">
         <v>1</v>
       </c>
       <c r="D470" t="s">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="E470" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="F470" t="s">
-        <v>58</v>
+        <v>150</v>
       </c>
       <c r="G470" s="1">
-        <v>46294</v>
+        <v>46310</v>
       </c>
       <c r="H470" s="1">
-        <v>46294</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="471" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A471" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B471" t="s">
-        <v>884</v>
+        <v>903</v>
       </c>
       <c r="C471">
         <v>1</v>
@@ -15455,24 +15602,24 @@
         <v>128</v>
       </c>
       <c r="E471" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="F471" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="G471" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
       <c r="H471" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="472" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A472" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B472" t="s">
-        <v>885</v>
+        <v>904</v>
       </c>
       <c r="C472">
         <v>1</v>
@@ -15481,10 +15628,10 @@
         <v>128</v>
       </c>
       <c r="E472" t="s">
-        <v>57</v>
+        <v>801</v>
       </c>
       <c r="F472" t="s">
-        <v>58</v>
+        <v>802</v>
       </c>
       <c r="G472" s="1">
         <v>46314</v>
@@ -15495,10 +15642,10 @@
     </row>
     <row r="473" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A473" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B473" t="s">
-        <v>886</v>
+        <v>905</v>
       </c>
       <c r="C473">
         <v>1</v>
@@ -15507,10 +15654,10 @@
         <v>128</v>
       </c>
       <c r="E473" t="s">
-        <v>57</v>
+        <v>906</v>
       </c>
       <c r="F473" t="s">
-        <v>58</v>
+        <v>907</v>
       </c>
       <c r="G473" s="1">
         <v>46314</v>
@@ -15521,10 +15668,10 @@
     </row>
     <row r="474" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A474" t="s">
-        <v>856</v>
+        <v>881</v>
       </c>
       <c r="B474" t="s">
-        <v>887</v>
+        <v>908</v>
       </c>
       <c r="C474">
         <v>1</v>
@@ -15533,10 +15680,10 @@
         <v>128</v>
       </c>
       <c r="E474" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="F474" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="G474" s="1">
         <v>46314</v>
@@ -15547,42 +15694,42 @@
     </row>
     <row r="475" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A475" t="s">
-        <v>856</v>
+        <v>909</v>
       </c>
       <c r="B475" t="s">
-        <v>888</v>
+        <v>910</v>
       </c>
       <c r="C475">
         <v>1</v>
       </c>
       <c r="D475" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E475" t="s">
-        <v>57</v>
+        <v>911</v>
       </c>
       <c r="F475" t="s">
-        <v>58</v>
+        <v>912</v>
       </c>
       <c r="G475" s="1">
-        <v>46314</v>
+        <v>46063</v>
       </c>
       <c r="H475" s="1">
-        <v>46314</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="476" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A476" t="s">
-        <v>856</v>
+        <v>909</v>
       </c>
       <c r="B476" t="s">
-        <v>889</v>
+        <v>913</v>
       </c>
       <c r="C476">
         <v>1</v>
       </c>
       <c r="D476" t="s">
-        <v>128</v>
+        <v>6</v>
       </c>
       <c r="E476" t="s">
         <v>57</v>
@@ -15591,24 +15738,24 @@
         <v>58</v>
       </c>
       <c r="G476" s="1">
-        <v>46314</v>
+        <v>46113</v>
       </c>
       <c r="H476" s="1">
-        <v>46314</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="477" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A477" t="s">
-        <v>856</v>
+        <v>909</v>
       </c>
       <c r="B477" t="s">
-        <v>890</v>
+        <v>914</v>
       </c>
       <c r="C477">
         <v>1</v>
       </c>
       <c r="D477" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="E477" t="s">
         <v>57</v>
@@ -15617,18 +15764,18 @@
         <v>58</v>
       </c>
       <c r="G477" s="1">
-        <v>46314</v>
+        <v>46125</v>
       </c>
       <c r="H477" s="1">
-        <v>46314</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="478" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A478" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B478" t="s">
-        <v>892</v>
+        <v>915</v>
       </c>
       <c r="C478">
         <v>1</v>
@@ -15637,24 +15784,24 @@
         <v>2</v>
       </c>
       <c r="E478" t="s">
-        <v>893</v>
+        <v>57</v>
       </c>
       <c r="F478" t="s">
-        <v>894</v>
+        <v>58</v>
       </c>
       <c r="G478" s="1">
-        <v>46157</v>
+        <v>46126</v>
       </c>
       <c r="H478" s="1">
-        <v>46157</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="479" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A479" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B479" t="s">
-        <v>895</v>
+        <v>916</v>
       </c>
       <c r="C479">
         <v>1</v>
@@ -15663,24 +15810,24 @@
         <v>2</v>
       </c>
       <c r="E479" t="s">
-        <v>896</v>
+        <v>57</v>
       </c>
       <c r="F479" t="s">
-        <v>897</v>
+        <v>58</v>
       </c>
       <c r="G479" s="1">
-        <v>46168</v>
+        <v>46126</v>
       </c>
       <c r="H479" s="1">
-        <v>46170</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="480" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A480" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B480" t="s">
-        <v>898</v>
+        <v>917</v>
       </c>
       <c r="C480">
         <v>1</v>
@@ -15689,50 +15836,50 @@
         <v>2</v>
       </c>
       <c r="E480" t="s">
-        <v>893</v>
+        <v>57</v>
       </c>
       <c r="F480" t="s">
-        <v>894</v>
+        <v>58</v>
       </c>
       <c r="G480" s="1">
-        <v>46218</v>
+        <v>46128</v>
       </c>
       <c r="H480" s="1">
-        <v>46218</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="481" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A481" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B481" t="s">
-        <v>899</v>
+        <v>918</v>
       </c>
       <c r="C481">
         <v>1</v>
       </c>
       <c r="D481" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E481" t="s">
-        <v>893</v>
+        <v>57</v>
       </c>
       <c r="F481" t="s">
-        <v>894</v>
+        <v>58</v>
       </c>
       <c r="G481" s="1">
-        <v>46244</v>
+        <v>46132</v>
       </c>
       <c r="H481" s="1">
-        <v>46244</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="482" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A482" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B482" t="s">
-        <v>900</v>
+        <v>919</v>
       </c>
       <c r="C482">
         <v>1</v>
@@ -15741,24 +15888,24 @@
         <v>2</v>
       </c>
       <c r="E482" t="s">
-        <v>893</v>
+        <v>57</v>
       </c>
       <c r="F482" t="s">
-        <v>894</v>
+        <v>58</v>
       </c>
       <c r="G482" s="1">
-        <v>46247</v>
+        <v>46161</v>
       </c>
       <c r="H482" s="1">
-        <v>46247</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="483" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A483" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B483" t="s">
-        <v>901</v>
+        <v>920</v>
       </c>
       <c r="C483">
         <v>1</v>
@@ -15767,24 +15914,24 @@
         <v>2</v>
       </c>
       <c r="E483" t="s">
-        <v>902</v>
+        <v>57</v>
       </c>
       <c r="F483" t="s">
-        <v>903</v>
+        <v>58</v>
       </c>
       <c r="G483" s="1">
-        <v>46247</v>
+        <v>46174</v>
       </c>
       <c r="H483" s="1">
-        <v>46247</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="484" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A484" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B484" t="s">
-        <v>904</v>
+        <v>921</v>
       </c>
       <c r="C484">
         <v>1</v>
@@ -15793,93 +15940,743 @@
         <v>2</v>
       </c>
       <c r="E484" t="s">
-        <v>893</v>
+        <v>57</v>
       </c>
       <c r="F484" t="s">
-        <v>894</v>
+        <v>58</v>
       </c>
       <c r="G484" s="1">
-        <v>46255</v>
+        <v>46174</v>
       </c>
       <c r="H484" s="1">
-        <v>46255</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="485" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A485" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B485" t="s">
-        <v>905</v>
+        <v>922</v>
       </c>
       <c r="C485">
         <v>1</v>
       </c>
       <c r="D485" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E485" t="s">
-        <v>893</v>
+        <v>57</v>
       </c>
       <c r="F485" t="s">
-        <v>894</v>
+        <v>58</v>
       </c>
       <c r="G485" s="1">
-        <v>46258</v>
+        <v>46195</v>
       </c>
       <c r="H485" s="1">
-        <v>46258</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="486" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A486" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B486" t="s">
-        <v>906</v>
+        <v>923</v>
       </c>
       <c r="C486">
         <v>1</v>
       </c>
       <c r="D486" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E486" t="s">
-        <v>893</v>
+        <v>57</v>
       </c>
       <c r="F486" t="s">
-        <v>894</v>
+        <v>58</v>
       </c>
       <c r="G486" s="1">
-        <v>46262</v>
+        <v>46210</v>
       </c>
       <c r="H486" s="1">
-        <v>46265</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="487" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A487" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="B487" t="s">
-        <v>907</v>
+        <v>924</v>
       </c>
       <c r="C487">
         <v>1</v>
       </c>
       <c r="D487" t="s">
+        <v>2</v>
+      </c>
+      <c r="E487" t="s">
+        <v>57</v>
+      </c>
+      <c r="F487" t="s">
+        <v>58</v>
+      </c>
+      <c r="G487" s="1">
+        <v>46213</v>
+      </c>
+      <c r="H487" s="1">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="488" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A488" t="s">
+        <v>909</v>
+      </c>
+      <c r="B488" t="s">
+        <v>925</v>
+      </c>
+      <c r="C488">
+        <v>1</v>
+      </c>
+      <c r="D488" t="s">
         <v>6</v>
       </c>
-      <c r="E487" t="s">
+      <c r="E488" t="s">
+        <v>57</v>
+      </c>
+      <c r="F488" t="s">
+        <v>58</v>
+      </c>
+      <c r="G488" s="1">
+        <v>46218</v>
+      </c>
+      <c r="H488" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="489" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A489" t="s">
+        <v>909</v>
+      </c>
+      <c r="B489" t="s">
+        <v>926</v>
+      </c>
+      <c r="C489">
+        <v>1</v>
+      </c>
+      <c r="D489" t="s">
+        <v>6</v>
+      </c>
+      <c r="E489" t="s">
+        <v>77</v>
+      </c>
+      <c r="F489" t="s">
+        <v>78</v>
+      </c>
+      <c r="G489" s="1">
+        <v>46226</v>
+      </c>
+      <c r="H489" s="1">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="490" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A490" t="s">
+        <v>909</v>
+      </c>
+      <c r="B490" t="s">
+        <v>927</v>
+      </c>
+      <c r="C490">
+        <v>1</v>
+      </c>
+      <c r="D490" t="s">
+        <v>128</v>
+      </c>
+      <c r="E490" t="s">
+        <v>57</v>
+      </c>
+      <c r="F490" t="s">
+        <v>58</v>
+      </c>
+      <c r="G490" s="1">
+        <v>46227</v>
+      </c>
+      <c r="H490" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="491" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A491" t="s">
+        <v>909</v>
+      </c>
+      <c r="B491" t="s">
+        <v>928</v>
+      </c>
+      <c r="C491">
+        <v>1</v>
+      </c>
+      <c r="D491" t="s">
+        <v>6</v>
+      </c>
+      <c r="E491" t="s">
+        <v>57</v>
+      </c>
+      <c r="F491" t="s">
+        <v>58</v>
+      </c>
+      <c r="G491" s="1">
+        <v>46227</v>
+      </c>
+      <c r="H491" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="492" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A492" t="s">
+        <v>909</v>
+      </c>
+      <c r="B492" t="s">
+        <v>929</v>
+      </c>
+      <c r="C492">
+        <v>1</v>
+      </c>
+      <c r="D492" t="s">
+        <v>6</v>
+      </c>
+      <c r="E492" t="s">
+        <v>57</v>
+      </c>
+      <c r="F492" t="s">
+        <v>58</v>
+      </c>
+      <c r="G492" s="1">
+        <v>46227</v>
+      </c>
+      <c r="H492" s="1">
+        <v>46228</v>
+      </c>
+    </row>
+    <row r="493" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A493" t="s">
+        <v>909</v>
+      </c>
+      <c r="B493" t="s">
+        <v>930</v>
+      </c>
+      <c r="C493">
+        <v>1</v>
+      </c>
+      <c r="D493" t="s">
+        <v>6</v>
+      </c>
+      <c r="E493" t="s">
+        <v>77</v>
+      </c>
+      <c r="F493" t="s">
+        <v>78</v>
+      </c>
+      <c r="G493" s="1">
+        <v>46230</v>
+      </c>
+      <c r="H493" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="494" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A494" t="s">
+        <v>909</v>
+      </c>
+      <c r="B494" t="s">
+        <v>931</v>
+      </c>
+      <c r="C494">
+        <v>1</v>
+      </c>
+      <c r="D494" t="s">
+        <v>6</v>
+      </c>
+      <c r="E494" t="s">
+        <v>57</v>
+      </c>
+      <c r="F494" t="s">
+        <v>58</v>
+      </c>
+      <c r="G494" s="1">
+        <v>46231</v>
+      </c>
+      <c r="H494" s="1">
+        <v>46231</v>
+      </c>
+    </row>
+    <row r="495" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A495" t="s">
+        <v>909</v>
+      </c>
+      <c r="B495" t="s">
+        <v>932</v>
+      </c>
+      <c r="C495">
+        <v>1</v>
+      </c>
+      <c r="D495" t="s">
+        <v>6</v>
+      </c>
+      <c r="E495" t="s">
+        <v>57</v>
+      </c>
+      <c r="F495" t="s">
+        <v>58</v>
+      </c>
+      <c r="G495" s="1">
+        <v>46254</v>
+      </c>
+      <c r="H495" s="1">
+        <v>46254</v>
+      </c>
+    </row>
+    <row r="496" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A496" t="s">
+        <v>909</v>
+      </c>
+      <c r="B496" t="s">
+        <v>933</v>
+      </c>
+      <c r="C496">
+        <v>1</v>
+      </c>
+      <c r="D496" t="s">
+        <v>2</v>
+      </c>
+      <c r="E496" t="s">
+        <v>57</v>
+      </c>
+      <c r="F496" t="s">
+        <v>58</v>
+      </c>
+      <c r="G496" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H496" s="1">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="497" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A497" t="s">
+        <v>909</v>
+      </c>
+      <c r="B497" t="s">
+        <v>934</v>
+      </c>
+      <c r="C497">
+        <v>1</v>
+      </c>
+      <c r="D497" t="s">
+        <v>6</v>
+      </c>
+      <c r="E497" t="s">
+        <v>57</v>
+      </c>
+      <c r="F497" t="s">
+        <v>58</v>
+      </c>
+      <c r="G497" s="1">
+        <v>46260</v>
+      </c>
+      <c r="H497" s="1">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="498" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A498" t="s">
+        <v>909</v>
+      </c>
+      <c r="B498" t="s">
+        <v>935</v>
+      </c>
+      <c r="C498">
+        <v>1</v>
+      </c>
+      <c r="D498" t="s">
+        <v>6</v>
+      </c>
+      <c r="E498" t="s">
+        <v>57</v>
+      </c>
+      <c r="F498" t="s">
+        <v>58</v>
+      </c>
+      <c r="G498" s="1">
+        <v>46289</v>
+      </c>
+      <c r="H498" s="1">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="499" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A499" t="s">
+        <v>909</v>
+      </c>
+      <c r="B499" t="s">
+        <v>936</v>
+      </c>
+      <c r="C499">
+        <v>1</v>
+      </c>
+      <c r="D499" t="s">
+        <v>6</v>
+      </c>
+      <c r="E499" t="s">
+        <v>57</v>
+      </c>
+      <c r="F499" t="s">
+        <v>58</v>
+      </c>
+      <c r="G499" s="1">
+        <v>46294</v>
+      </c>
+      <c r="H499" s="1">
+        <v>46294</v>
+      </c>
+    </row>
+    <row r="500" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A500" t="s">
+        <v>909</v>
+      </c>
+      <c r="B500" t="s">
+        <v>937</v>
+      </c>
+      <c r="C500">
+        <v>1</v>
+      </c>
+      <c r="D500" t="s">
+        <v>128</v>
+      </c>
+      <c r="E500" t="s">
+        <v>57</v>
+      </c>
+      <c r="F500" t="s">
+        <v>58</v>
+      </c>
+      <c r="G500" s="1">
+        <v>46314</v>
+      </c>
+      <c r="H500" s="1">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="501" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A501" t="s">
+        <v>909</v>
+      </c>
+      <c r="B501" t="s">
+        <v>938</v>
+      </c>
+      <c r="C501">
+        <v>1</v>
+      </c>
+      <c r="D501" t="s">
+        <v>128</v>
+      </c>
+      <c r="E501" t="s">
+        <v>57</v>
+      </c>
+      <c r="F501" t="s">
+        <v>58</v>
+      </c>
+      <c r="G501" s="1">
+        <v>46314</v>
+      </c>
+      <c r="H501" s="1">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="502" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A502" t="s">
+        <v>909</v>
+      </c>
+      <c r="B502" t="s">
+        <v>939</v>
+      </c>
+      <c r="C502">
+        <v>1</v>
+      </c>
+      <c r="D502" t="s">
+        <v>128</v>
+      </c>
+      <c r="E502" t="s">
+        <v>57</v>
+      </c>
+      <c r="F502" t="s">
+        <v>58</v>
+      </c>
+      <c r="G502" s="1">
+        <v>46314</v>
+      </c>
+      <c r="H502" s="1">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="503" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A503" t="s">
+        <v>940</v>
+      </c>
+      <c r="B503" t="s">
+        <v>941</v>
+      </c>
+      <c r="C503">
+        <v>1</v>
+      </c>
+      <c r="D503" t="s">
+        <v>2</v>
+      </c>
+      <c r="E503" t="s">
+        <v>942</v>
+      </c>
+      <c r="F503" t="s">
+        <v>943</v>
+      </c>
+      <c r="G503" s="1">
+        <v>46157</v>
+      </c>
+      <c r="H503" s="1">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="504" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A504" t="s">
+        <v>940</v>
+      </c>
+      <c r="B504" t="s">
+        <v>944</v>
+      </c>
+      <c r="C504">
+        <v>1</v>
+      </c>
+      <c r="D504" t="s">
+        <v>2</v>
+      </c>
+      <c r="E504" t="s">
+        <v>945</v>
+      </c>
+      <c r="F504" t="s">
+        <v>946</v>
+      </c>
+      <c r="G504" s="1">
+        <v>46168</v>
+      </c>
+      <c r="H504" s="1">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="505" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A505" t="s">
+        <v>940</v>
+      </c>
+      <c r="B505" t="s">
+        <v>947</v>
+      </c>
+      <c r="C505">
+        <v>1</v>
+      </c>
+      <c r="D505" t="s">
+        <v>2</v>
+      </c>
+      <c r="E505" t="s">
+        <v>942</v>
+      </c>
+      <c r="F505" t="s">
+        <v>943</v>
+      </c>
+      <c r="G505" s="1">
+        <v>46218</v>
+      </c>
+      <c r="H505" s="1">
+        <v>46218</v>
+      </c>
+    </row>
+    <row r="506" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A506" t="s">
+        <v>940</v>
+      </c>
+      <c r="B506" t="s">
+        <v>948</v>
+      </c>
+      <c r="C506">
+        <v>1</v>
+      </c>
+      <c r="D506" t="s">
+        <v>2</v>
+      </c>
+      <c r="E506" t="s">
+        <v>942</v>
+      </c>
+      <c r="F506" t="s">
+        <v>943</v>
+      </c>
+      <c r="G506" s="1">
+        <v>46244</v>
+      </c>
+      <c r="H506" s="1">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="507" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A507" t="s">
+        <v>940</v>
+      </c>
+      <c r="B507" t="s">
+        <v>949</v>
+      </c>
+      <c r="C507">
+        <v>1</v>
+      </c>
+      <c r="D507" t="s">
+        <v>2</v>
+      </c>
+      <c r="E507" t="s">
+        <v>942</v>
+      </c>
+      <c r="F507" t="s">
+        <v>943</v>
+      </c>
+      <c r="G507" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H507" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="508" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A508" t="s">
+        <v>940</v>
+      </c>
+      <c r="B508" t="s">
+        <v>950</v>
+      </c>
+      <c r="C508">
+        <v>1</v>
+      </c>
+      <c r="D508" t="s">
+        <v>2</v>
+      </c>
+      <c r="E508" t="s">
+        <v>951</v>
+      </c>
+      <c r="F508" t="s">
+        <v>952</v>
+      </c>
+      <c r="G508" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H508" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="509" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A509" t="s">
+        <v>940</v>
+      </c>
+      <c r="B509" t="s">
+        <v>953</v>
+      </c>
+      <c r="C509">
+        <v>1</v>
+      </c>
+      <c r="D509" t="s">
+        <v>2</v>
+      </c>
+      <c r="E509" t="s">
+        <v>942</v>
+      </c>
+      <c r="F509" t="s">
+        <v>943</v>
+      </c>
+      <c r="G509" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H509" s="1">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="510" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A510" t="s">
+        <v>940</v>
+      </c>
+      <c r="B510" t="s">
+        <v>954</v>
+      </c>
+      <c r="C510">
+        <v>1</v>
+      </c>
+      <c r="D510" t="s">
+        <v>2</v>
+      </c>
+      <c r="E510" t="s">
+        <v>942</v>
+      </c>
+      <c r="F510" t="s">
+        <v>943</v>
+      </c>
+      <c r="G510" s="1">
+        <v>46258</v>
+      </c>
+      <c r="H510" s="1">
+        <v>46258</v>
+      </c>
+    </row>
+    <row r="511" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A511" t="s">
+        <v>940</v>
+      </c>
+      <c r="B511" t="s">
+        <v>955</v>
+      </c>
+      <c r="C511">
+        <v>1</v>
+      </c>
+      <c r="D511" t="s">
+        <v>2</v>
+      </c>
+      <c r="E511" t="s">
+        <v>942</v>
+      </c>
+      <c r="F511" t="s">
+        <v>943</v>
+      </c>
+      <c r="G511" s="1">
+        <v>46262</v>
+      </c>
+      <c r="H511" s="1">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="512" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A512" t="s">
+        <v>940</v>
+      </c>
+      <c r="B512" t="s">
+        <v>956</v>
+      </c>
+      <c r="C512">
+        <v>1</v>
+      </c>
+      <c r="D512" t="s">
+        <v>6</v>
+      </c>
+      <c r="E512" t="s">
         <v>13</v>
       </c>
-      <c r="F487" t="s">
+      <c r="F512" t="s">
         <v>14</v>
       </c>
-      <c r="G487" s="1">
+      <c r="G512" s="1">
         <v>46281</v>
       </c>
-      <c r="H487" s="1">
+      <c r="H512" s="1">
         <v>46283</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 29/10/2026 06:04:19
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DFD5C95-E941-48BD-80A5-57A88E09196D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{41E07371-D54A-4183-B0CF-F5627CD05268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{FBB4A754-8133-4D00-A52E-FE716F7787F8}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F37F80EB-F1F6-412C-B187-271CE8F88977}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2323" uniqueCount="896">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2398" uniqueCount="915">
   <si>
     <t>0001</t>
   </si>
@@ -2365,6 +2365,60 @@
     <t xml:space="preserve">  218445</t>
   </si>
   <si>
+    <t xml:space="preserve">  218446</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218447</t>
+  </si>
+  <si>
+    <t>GO08</t>
+  </si>
+  <si>
+    <t>GOMEZ-OLIVO SRL - HG SANITARIOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218450</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218451</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218452</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218454</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218457</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218458</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218459</t>
+  </si>
+  <si>
+    <t>MA29</t>
+  </si>
+  <si>
+    <t>MULTISANITARIOS Y ACCESORIOS S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218461</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218463</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218464</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  218465</t>
+  </si>
+  <si>
     <t>0004</t>
   </si>
   <si>
@@ -2537,6 +2591,9 @@
   </si>
   <si>
     <t xml:space="preserve">    3090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    3092</t>
   </si>
   <si>
     <t>4444</t>
@@ -3157,34 +3214,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27DFC761-9F0B-4B91-9715-5368ADAF6169}">
-  <dimension ref="A1:H464"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E99DB8D7-1FB1-4BD4-9A31-A8D96DA78E3C}">
+  <dimension ref="A1:H479"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>888</v>
+        <v>907</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>889</v>
+        <v>908</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>890</v>
+        <v>909</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>891</v>
+        <v>910</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>892</v>
+        <v>911</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>893</v>
+        <v>912</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>894</v>
+        <v>913</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>895</v>
+        <v>914</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -8577,10 +8634,10 @@
         <v>457</v>
       </c>
       <c r="C209">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D209" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E209" t="s">
         <v>458</v>
@@ -8592,7 +8649,7 @@
         <v>46317</v>
       </c>
       <c r="H209" s="1">
-        <v>46317</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.2">
@@ -9464,7 +9521,7 @@
         <v>1</v>
       </c>
       <c r="D243" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E243" t="s">
         <v>127</v>
@@ -10764,7 +10821,7 @@
         <v>1</v>
       </c>
       <c r="D293" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E293" t="s">
         <v>616</v>
@@ -13303,88 +13360,88 @@
     </row>
     <row r="391" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A391" t="s">
+        <v>0</v>
+      </c>
+      <c r="B391" t="s">
         <v>781</v>
       </c>
-      <c r="B391" t="s">
-        <v>782</v>
-      </c>
       <c r="C391">
         <v>1</v>
       </c>
       <c r="D391" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E391" t="s">
-        <v>157</v>
+        <v>16</v>
       </c>
       <c r="F391" t="s">
-        <v>158</v>
+        <v>17</v>
       </c>
       <c r="G391" s="1">
-        <v>46148</v>
+        <v>46323</v>
       </c>
       <c r="H391" s="1">
-        <v>46149</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="392" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A392" t="s">
-        <v>781</v>
+        <v>0</v>
       </c>
       <c r="B392" t="s">
+        <v>782</v>
+      </c>
+      <c r="C392">
+        <v>1</v>
+      </c>
+      <c r="D392" t="s">
+        <v>125</v>
+      </c>
+      <c r="E392" t="s">
         <v>783</v>
       </c>
-      <c r="C392">
-        <v>1</v>
-      </c>
-      <c r="D392" t="s">
-        <v>2</v>
-      </c>
-      <c r="E392" t="s">
-        <v>311</v>
-      </c>
       <c r="F392" t="s">
-        <v>312</v>
+        <v>784</v>
       </c>
       <c r="G392" s="1">
-        <v>46268</v>
+        <v>46323</v>
       </c>
       <c r="H392" s="1">
-        <v>46268</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="393" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A393" t="s">
-        <v>781</v>
+        <v>0</v>
       </c>
       <c r="B393" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="C393">
         <v>1</v>
       </c>
       <c r="D393" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E393" t="s">
-        <v>336</v>
+        <v>721</v>
       </c>
       <c r="F393" t="s">
-        <v>337</v>
+        <v>722</v>
       </c>
       <c r="G393" s="1">
-        <v>46315</v>
+        <v>46323</v>
       </c>
       <c r="H393" s="1">
-        <v>46315</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="394" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A394" t="s">
-        <v>781</v>
+        <v>0</v>
       </c>
       <c r="B394" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="C394">
         <v>1</v>
@@ -13393,24 +13450,24 @@
         <v>125</v>
       </c>
       <c r="E394" t="s">
-        <v>786</v>
+        <v>402</v>
       </c>
       <c r="F394" t="s">
-        <v>787</v>
+        <v>403</v>
       </c>
       <c r="G394" s="1">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="H394" s="1">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="395" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A395" t="s">
-        <v>781</v>
+        <v>0</v>
       </c>
       <c r="B395" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="C395">
         <v>1</v>
@@ -13419,24 +13476,24 @@
         <v>125</v>
       </c>
       <c r="E395" t="s">
-        <v>789</v>
+        <v>37</v>
       </c>
       <c r="F395" t="s">
-        <v>790</v>
+        <v>38</v>
       </c>
       <c r="G395" s="1">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="H395" s="1">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="396" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A396" t="s">
-        <v>781</v>
+        <v>0</v>
       </c>
       <c r="B396" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="C396">
         <v>1</v>
@@ -13445,10 +13502,10 @@
         <v>125</v>
       </c>
       <c r="E396" t="s">
-        <v>471</v>
+        <v>37</v>
       </c>
       <c r="F396" t="s">
-        <v>472</v>
+        <v>38</v>
       </c>
       <c r="G396" s="1">
         <v>46323</v>
@@ -13459,218 +13516,218 @@
     </row>
     <row r="397" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A397" t="s">
-        <v>792</v>
+        <v>0</v>
       </c>
       <c r="B397" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
       <c r="C397">
         <v>1</v>
       </c>
       <c r="D397" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E397" t="s">
-        <v>794</v>
+        <v>37</v>
       </c>
       <c r="F397" t="s">
-        <v>795</v>
+        <v>38</v>
       </c>
       <c r="G397" s="1">
-        <v>46308</v>
+        <v>46323</v>
       </c>
       <c r="H397" s="1">
-        <v>46308</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="398" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A398" t="s">
-        <v>796</v>
+        <v>0</v>
       </c>
       <c r="B398" t="s">
-        <v>797</v>
+        <v>790</v>
       </c>
       <c r="C398">
         <v>1</v>
       </c>
       <c r="D398" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="E398" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F398" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G398" s="1">
-        <v>46133</v>
+        <v>46323</v>
       </c>
       <c r="H398" s="1">
-        <v>46134</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="399" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A399" t="s">
-        <v>796</v>
+        <v>0</v>
       </c>
       <c r="B399" t="s">
-        <v>798</v>
+        <v>791</v>
       </c>
       <c r="C399">
         <v>1</v>
       </c>
       <c r="D399" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="E399" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F399" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G399" s="1">
-        <v>46134</v>
+        <v>46323</v>
       </c>
       <c r="H399" s="1">
-        <v>46134</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="400" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A400" t="s">
-        <v>796</v>
+        <v>0</v>
       </c>
       <c r="B400" t="s">
-        <v>799</v>
+        <v>792</v>
       </c>
       <c r="C400">
         <v>1</v>
       </c>
       <c r="D400" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="E400" t="s">
-        <v>19</v>
+        <v>793</v>
       </c>
       <c r="F400" t="s">
-        <v>20</v>
+        <v>794</v>
       </c>
       <c r="G400" s="1">
-        <v>46156</v>
+        <v>46323</v>
       </c>
       <c r="H400" s="1">
-        <v>46156</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="401" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A401" t="s">
-        <v>796</v>
+        <v>0</v>
       </c>
       <c r="B401" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="C401">
         <v>1</v>
       </c>
       <c r="D401" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="E401" t="s">
-        <v>801</v>
+        <v>37</v>
       </c>
       <c r="F401" t="s">
-        <v>802</v>
+        <v>38</v>
       </c>
       <c r="G401" s="1">
-        <v>46213</v>
+        <v>46323</v>
       </c>
       <c r="H401" s="1">
-        <v>46213</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="402" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A402" t="s">
+        <v>0</v>
+      </c>
+      <c r="B402" t="s">
         <v>796</v>
       </c>
-      <c r="B402" t="s">
-        <v>803</v>
-      </c>
       <c r="C402">
         <v>1</v>
       </c>
       <c r="D402" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="E402" t="s">
-        <v>804</v>
+        <v>37</v>
       </c>
       <c r="F402" t="s">
-        <v>805</v>
+        <v>38</v>
       </c>
       <c r="G402" s="1">
-        <v>46253</v>
+        <v>46323</v>
       </c>
       <c r="H402" s="1">
-        <v>46253</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="403" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A403" t="s">
-        <v>796</v>
+        <v>0</v>
       </c>
       <c r="B403" t="s">
-        <v>806</v>
+        <v>797</v>
       </c>
       <c r="C403">
         <v>1</v>
       </c>
       <c r="D403" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E403" t="s">
-        <v>169</v>
+        <v>37</v>
       </c>
       <c r="F403" t="s">
-        <v>170</v>
+        <v>38</v>
       </c>
       <c r="G403" s="1">
-        <v>46273</v>
+        <v>46323</v>
       </c>
       <c r="H403" s="1">
-        <v>46274</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="404" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A404" t="s">
-        <v>796</v>
+        <v>0</v>
       </c>
       <c r="B404" t="s">
-        <v>807</v>
+        <v>798</v>
       </c>
       <c r="C404">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D404" t="s">
         <v>125</v>
       </c>
       <c r="E404" t="s">
-        <v>808</v>
+        <v>37</v>
       </c>
       <c r="F404" t="s">
-        <v>809</v>
+        <v>38</v>
       </c>
       <c r="G404" s="1">
-        <v>46300</v>
+        <v>46323</v>
       </c>
       <c r="H404" s="1">
-        <v>46318</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="405" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A405" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="B405" t="s">
-        <v>810</v>
+        <v>800</v>
       </c>
       <c r="C405">
         <v>1</v>
@@ -13679,24 +13736,24 @@
         <v>2</v>
       </c>
       <c r="E405" t="s">
-        <v>179</v>
+        <v>157</v>
       </c>
       <c r="F405" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
       <c r="G405" s="1">
-        <v>46300</v>
+        <v>46148</v>
       </c>
       <c r="H405" s="1">
-        <v>46300</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="406" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A406" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="B406" t="s">
-        <v>811</v>
+        <v>801</v>
       </c>
       <c r="C406">
         <v>1</v>
@@ -13705,128 +13762,128 @@
         <v>2</v>
       </c>
       <c r="E406" t="s">
-        <v>812</v>
+        <v>311</v>
       </c>
       <c r="F406" t="s">
-        <v>813</v>
+        <v>312</v>
       </c>
       <c r="G406" s="1">
-        <v>46300</v>
+        <v>46268</v>
       </c>
       <c r="H406" s="1">
-        <v>46301</v>
+        <v>46268</v>
       </c>
     </row>
     <row r="407" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A407" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="B407" t="s">
-        <v>814</v>
+        <v>802</v>
       </c>
       <c r="C407">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D407" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E407" t="s">
-        <v>278</v>
+        <v>336</v>
       </c>
       <c r="F407" t="s">
-        <v>279</v>
+        <v>337</v>
       </c>
       <c r="G407" s="1">
-        <v>46302</v>
+        <v>46315</v>
       </c>
       <c r="H407" s="1">
-        <v>46321</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="408" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A408" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="B408" t="s">
-        <v>815</v>
+        <v>803</v>
       </c>
       <c r="C408">
         <v>1</v>
       </c>
       <c r="D408" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="E408" t="s">
-        <v>816</v>
+        <v>804</v>
       </c>
       <c r="F408" t="s">
-        <v>817</v>
+        <v>805</v>
       </c>
       <c r="G408" s="1">
-        <v>46303</v>
+        <v>46321</v>
       </c>
       <c r="H408" s="1">
-        <v>46303</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="409" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A409" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="B409" t="s">
-        <v>818</v>
+        <v>806</v>
       </c>
       <c r="C409">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D409" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E409" t="s">
-        <v>505</v>
+        <v>807</v>
       </c>
       <c r="F409" t="s">
-        <v>506</v>
+        <v>808</v>
       </c>
       <c r="G409" s="1">
-        <v>46308</v>
+        <v>46321</v>
       </c>
       <c r="H409" s="1">
-        <v>46316</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="410" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A410" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="B410" t="s">
-        <v>819</v>
+        <v>809</v>
       </c>
       <c r="C410">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D410" t="s">
         <v>125</v>
       </c>
       <c r="E410" t="s">
-        <v>593</v>
+        <v>471</v>
       </c>
       <c r="F410" t="s">
-        <v>594</v>
+        <v>472</v>
       </c>
       <c r="G410" s="1">
-        <v>46310</v>
+        <v>46323</v>
       </c>
       <c r="H410" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="411" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A411" t="s">
-        <v>796</v>
+        <v>810</v>
       </c>
       <c r="B411" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
       <c r="C411">
         <v>1</v>
@@ -13835,258 +13892,258 @@
         <v>2</v>
       </c>
       <c r="E411" t="s">
-        <v>41</v>
+        <v>812</v>
       </c>
       <c r="F411" t="s">
-        <v>42</v>
+        <v>813</v>
       </c>
       <c r="G411" s="1">
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="H411" s="1">
-        <v>46311</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="412" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A412" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B412" t="s">
-        <v>821</v>
+        <v>815</v>
       </c>
       <c r="C412">
         <v>1</v>
       </c>
       <c r="D412" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E412" t="s">
-        <v>812</v>
+        <v>41</v>
       </c>
       <c r="F412" t="s">
-        <v>813</v>
+        <v>42</v>
       </c>
       <c r="G412" s="1">
-        <v>46315</v>
+        <v>46133</v>
       </c>
       <c r="H412" s="1">
-        <v>46315</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="413" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A413" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B413" t="s">
-        <v>822</v>
+        <v>816</v>
       </c>
       <c r="C413">
         <v>1</v>
       </c>
       <c r="D413" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E413" t="s">
-        <v>823</v>
+        <v>41</v>
       </c>
       <c r="F413" t="s">
-        <v>824</v>
+        <v>42</v>
       </c>
       <c r="G413" s="1">
-        <v>46317</v>
+        <v>46134</v>
       </c>
       <c r="H413" s="1">
-        <v>46318</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="414" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A414" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B414" t="s">
-        <v>825</v>
+        <v>817</v>
       </c>
       <c r="C414">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D414" t="s">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="E414" t="s">
-        <v>146</v>
+        <v>19</v>
       </c>
       <c r="F414" t="s">
-        <v>147</v>
+        <v>20</v>
       </c>
       <c r="G414" s="1">
-        <v>46317</v>
+        <v>46156</v>
       </c>
       <c r="H414" s="1">
-        <v>46323</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="415" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A415" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B415" t="s">
-        <v>826</v>
+        <v>818</v>
       </c>
       <c r="C415">
         <v>1</v>
       </c>
       <c r="D415" t="s">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="E415" t="s">
-        <v>16</v>
+        <v>819</v>
       </c>
       <c r="F415" t="s">
-        <v>17</v>
+        <v>820</v>
       </c>
       <c r="G415" s="1">
-        <v>46318</v>
+        <v>46213</v>
       </c>
       <c r="H415" s="1">
-        <v>46318</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="416" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A416" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B416" t="s">
-        <v>827</v>
+        <v>821</v>
       </c>
       <c r="C416">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D416" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E416" t="s">
-        <v>505</v>
+        <v>822</v>
       </c>
       <c r="F416" t="s">
-        <v>506</v>
+        <v>823</v>
       </c>
       <c r="G416" s="1">
-        <v>46321</v>
+        <v>46253</v>
       </c>
       <c r="H416" s="1">
-        <v>46323</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="417" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A417" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B417" t="s">
-        <v>828</v>
+        <v>824</v>
       </c>
       <c r="C417">
         <v>1</v>
       </c>
       <c r="D417" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E417" t="s">
-        <v>278</v>
+        <v>169</v>
       </c>
       <c r="F417" t="s">
-        <v>279</v>
+        <v>170</v>
       </c>
       <c r="G417" s="1">
-        <v>46321</v>
+        <v>46273</v>
       </c>
       <c r="H417" s="1">
-        <v>46321</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="418" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A418" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B418" t="s">
-        <v>829</v>
+        <v>825</v>
       </c>
       <c r="C418">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D418" t="s">
         <v>125</v>
       </c>
       <c r="E418" t="s">
-        <v>830</v>
+        <v>826</v>
       </c>
       <c r="F418" t="s">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="G418" s="1">
-        <v>46321</v>
+        <v>46300</v>
       </c>
       <c r="H418" s="1">
-        <v>46323</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="419" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A419" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B419" t="s">
-        <v>832</v>
+        <v>828</v>
       </c>
       <c r="C419">
         <v>1</v>
       </c>
       <c r="D419" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E419" t="s">
-        <v>278</v>
+        <v>179</v>
       </c>
       <c r="F419" t="s">
-        <v>279</v>
+        <v>180</v>
       </c>
       <c r="G419" s="1">
-        <v>46321</v>
+        <v>46300</v>
       </c>
       <c r="H419" s="1">
-        <v>46322</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="420" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A420" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B420" t="s">
-        <v>833</v>
+        <v>829</v>
       </c>
       <c r="C420">
         <v>1</v>
       </c>
       <c r="D420" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E420" t="s">
-        <v>808</v>
+        <v>830</v>
       </c>
       <c r="F420" t="s">
-        <v>809</v>
+        <v>831</v>
       </c>
       <c r="G420" s="1">
-        <v>46322</v>
+        <v>46300</v>
       </c>
       <c r="H420" s="1">
-        <v>46322</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="421" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A421" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B421" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="C421">
         <v>2</v>
@@ -14095,99 +14152,99 @@
         <v>125</v>
       </c>
       <c r="E421" t="s">
-        <v>812</v>
+        <v>278</v>
       </c>
       <c r="F421" t="s">
-        <v>813</v>
+        <v>279</v>
       </c>
       <c r="G421" s="1">
-        <v>46322</v>
+        <v>46302</v>
       </c>
       <c r="H421" s="1">
-        <v>46323</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="422" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A422" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B422" t="s">
+        <v>833</v>
+      </c>
+      <c r="C422">
+        <v>1</v>
+      </c>
+      <c r="D422" t="s">
+        <v>6</v>
+      </c>
+      <c r="E422" t="s">
+        <v>834</v>
+      </c>
+      <c r="F422" t="s">
         <v>835</v>
       </c>
-      <c r="C422">
-        <v>1</v>
-      </c>
-      <c r="D422" t="s">
-        <v>2</v>
-      </c>
-      <c r="E422" t="s">
-        <v>812</v>
-      </c>
-      <c r="F422" t="s">
-        <v>813</v>
-      </c>
       <c r="G422" s="1">
-        <v>46322</v>
+        <v>46303</v>
       </c>
       <c r="H422" s="1">
-        <v>46322</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="423" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A423" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B423" t="s">
         <v>836</v>
       </c>
       <c r="C423">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D423" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E423" t="s">
-        <v>812</v>
+        <v>505</v>
       </c>
       <c r="F423" t="s">
-        <v>813</v>
+        <v>506</v>
       </c>
       <c r="G423" s="1">
-        <v>46322</v>
+        <v>46308</v>
       </c>
       <c r="H423" s="1">
-        <v>46323</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="424" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A424" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B424" t="s">
         <v>837</v>
       </c>
       <c r="C424">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D424" t="s">
         <v>125</v>
       </c>
       <c r="E424" t="s">
-        <v>492</v>
+        <v>593</v>
       </c>
       <c r="F424" t="s">
-        <v>493</v>
+        <v>594</v>
       </c>
       <c r="G424" s="1">
+        <v>46310</v>
+      </c>
+      <c r="H424" s="1">
         <v>46322</v>
-      </c>
-      <c r="H424" s="1">
-        <v>46323</v>
       </c>
     </row>
     <row r="425" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A425" t="s">
-        <v>796</v>
+        <v>814</v>
       </c>
       <c r="B425" t="s">
         <v>838</v>
@@ -14196,28 +14253,28 @@
         <v>1</v>
       </c>
       <c r="D425" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E425" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="F425" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="G425" s="1">
-        <v>46323</v>
+        <v>46311</v>
       </c>
       <c r="H425" s="1">
-        <v>46323</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="426" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A426" t="s">
+        <v>814</v>
+      </c>
+      <c r="B426" t="s">
         <v>839</v>
       </c>
-      <c r="B426" t="s">
-        <v>840</v>
-      </c>
       <c r="C426">
         <v>1</v>
       </c>
@@ -14225,414 +14282,414 @@
         <v>2</v>
       </c>
       <c r="E426" t="s">
-        <v>841</v>
+        <v>830</v>
       </c>
       <c r="F426" t="s">
-        <v>842</v>
+        <v>831</v>
       </c>
       <c r="G426" s="1">
-        <v>46063</v>
+        <v>46315</v>
       </c>
       <c r="H426" s="1">
-        <v>46064</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="427" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A427" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B427" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="C427">
         <v>1</v>
       </c>
       <c r="D427" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E427" t="s">
-        <v>57</v>
+        <v>841</v>
       </c>
       <c r="F427" t="s">
-        <v>58</v>
+        <v>842</v>
       </c>
       <c r="G427" s="1">
-        <v>46113</v>
+        <v>46317</v>
       </c>
       <c r="H427" s="1">
-        <v>46125</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="428" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A428" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B428" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="C428">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D428" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E428" t="s">
-        <v>57</v>
+        <v>146</v>
       </c>
       <c r="F428" t="s">
-        <v>58</v>
+        <v>147</v>
       </c>
       <c r="G428" s="1">
-        <v>46125</v>
+        <v>46317</v>
       </c>
       <c r="H428" s="1">
-        <v>46125</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="429" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A429" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B429" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="C429">
         <v>1</v>
       </c>
       <c r="D429" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E429" t="s">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="F429" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="G429" s="1">
-        <v>46126</v>
+        <v>46318</v>
       </c>
       <c r="H429" s="1">
-        <v>46126</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="430" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A430" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B430" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="C430">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D430" t="s">
         <v>2</v>
       </c>
       <c r="E430" t="s">
-        <v>57</v>
+        <v>505</v>
       </c>
       <c r="F430" t="s">
-        <v>58</v>
+        <v>506</v>
       </c>
       <c r="G430" s="1">
-        <v>46126</v>
+        <v>46321</v>
       </c>
       <c r="H430" s="1">
-        <v>46126</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="431" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A431" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B431" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="C431">
         <v>1</v>
       </c>
       <c r="D431" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E431" t="s">
-        <v>57</v>
+        <v>278</v>
       </c>
       <c r="F431" t="s">
-        <v>58</v>
+        <v>279</v>
       </c>
       <c r="G431" s="1">
-        <v>46128</v>
+        <v>46321</v>
       </c>
       <c r="H431" s="1">
-        <v>46128</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="432" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A432" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B432" t="s">
+        <v>847</v>
+      </c>
+      <c r="C432">
+        <v>1</v>
+      </c>
+      <c r="D432" t="s">
+        <v>125</v>
+      </c>
+      <c r="E432" t="s">
         <v>848</v>
       </c>
-      <c r="C432">
-        <v>1</v>
-      </c>
-      <c r="D432" t="s">
-        <v>6</v>
-      </c>
-      <c r="E432" t="s">
-        <v>57</v>
-      </c>
       <c r="F432" t="s">
-        <v>58</v>
+        <v>849</v>
       </c>
       <c r="G432" s="1">
-        <v>46132</v>
+        <v>46321</v>
       </c>
       <c r="H432" s="1">
-        <v>46132</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="433" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A433" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B433" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="C433">
         <v>1</v>
       </c>
       <c r="D433" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E433" t="s">
-        <v>57</v>
+        <v>278</v>
       </c>
       <c r="F433" t="s">
-        <v>58</v>
+        <v>279</v>
       </c>
       <c r="G433" s="1">
-        <v>46161</v>
+        <v>46321</v>
       </c>
       <c r="H433" s="1">
-        <v>46161</v>
+        <v>46322</v>
       </c>
     </row>
     <row r="434" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A434" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B434" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="C434">
         <v>1</v>
       </c>
       <c r="D434" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E434" t="s">
-        <v>57</v>
+        <v>826</v>
       </c>
       <c r="F434" t="s">
-        <v>58</v>
+        <v>827</v>
       </c>
       <c r="G434" s="1">
-        <v>46174</v>
+        <v>46322</v>
       </c>
       <c r="H434" s="1">
-        <v>46174</v>
+        <v>46322</v>
       </c>
     </row>
     <row r="435" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A435" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B435" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="C435">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D435" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E435" t="s">
-        <v>57</v>
+        <v>830</v>
       </c>
       <c r="F435" t="s">
-        <v>58</v>
+        <v>831</v>
       </c>
       <c r="G435" s="1">
-        <v>46174</v>
+        <v>46322</v>
       </c>
       <c r="H435" s="1">
-        <v>46174</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="436" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A436" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B436" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="C436">
         <v>1</v>
       </c>
       <c r="D436" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E436" t="s">
-        <v>57</v>
+        <v>830</v>
       </c>
       <c r="F436" t="s">
-        <v>58</v>
+        <v>831</v>
       </c>
       <c r="G436" s="1">
-        <v>46195</v>
+        <v>46322</v>
       </c>
       <c r="H436" s="1">
-        <v>46252</v>
+        <v>46322</v>
       </c>
     </row>
     <row r="437" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A437" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B437" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="C437">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D437" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="E437" t="s">
-        <v>57</v>
+        <v>830</v>
       </c>
       <c r="F437" t="s">
-        <v>58</v>
+        <v>831</v>
       </c>
       <c r="G437" s="1">
-        <v>46210</v>
+        <v>46322</v>
       </c>
       <c r="H437" s="1">
-        <v>46210</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="438" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A438" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B438" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C438">
         <v>1</v>
       </c>
       <c r="D438" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E438" t="s">
-        <v>57</v>
+        <v>492</v>
       </c>
       <c r="F438" t="s">
-        <v>58</v>
+        <v>493</v>
       </c>
       <c r="G438" s="1">
-        <v>46213</v>
+        <v>46322</v>
       </c>
       <c r="H438" s="1">
-        <v>46213</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="439" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A439" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B439" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="C439">
         <v>1</v>
       </c>
       <c r="D439" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="E439" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="F439" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G439" s="1">
-        <v>46218</v>
+        <v>46323</v>
       </c>
       <c r="H439" s="1">
-        <v>46252</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="440" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A440" t="s">
-        <v>839</v>
+        <v>814</v>
       </c>
       <c r="B440" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="C440">
         <v>1</v>
       </c>
       <c r="D440" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="E440" t="s">
-        <v>77</v>
+        <v>505</v>
       </c>
       <c r="F440" t="s">
-        <v>78</v>
+        <v>506</v>
       </c>
       <c r="G440" s="1">
-        <v>46226</v>
+        <v>46323</v>
       </c>
       <c r="H440" s="1">
-        <v>46226</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="441" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A441" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B441" t="s">
-        <v>857</v>
+        <v>859</v>
       </c>
       <c r="C441">
         <v>1</v>
       </c>
       <c r="D441" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E441" t="s">
-        <v>57</v>
+        <v>860</v>
       </c>
       <c r="F441" t="s">
-        <v>58</v>
+        <v>861</v>
       </c>
       <c r="G441" s="1">
-        <v>46227</v>
+        <v>46063</v>
       </c>
       <c r="H441" s="1">
-        <v>46252</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="442" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A442" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B442" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
       <c r="C442">
         <v>1</v>
@@ -14647,24 +14704,24 @@
         <v>58</v>
       </c>
       <c r="G442" s="1">
-        <v>46227</v>
+        <v>46113</v>
       </c>
       <c r="H442" s="1">
-        <v>46252</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="443" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A443" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B443" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
       <c r="C443">
         <v>1</v>
       </c>
       <c r="D443" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E443" t="s">
         <v>57</v>
@@ -14673,50 +14730,50 @@
         <v>58</v>
       </c>
       <c r="G443" s="1">
-        <v>46227</v>
+        <v>46125</v>
       </c>
       <c r="H443" s="1">
-        <v>46228</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="444" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A444" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B444" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C444">
         <v>1</v>
       </c>
       <c r="D444" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E444" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="F444" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G444" s="1">
-        <v>46230</v>
+        <v>46126</v>
       </c>
       <c r="H444" s="1">
-        <v>46252</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="445" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A445" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B445" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="C445">
         <v>1</v>
       </c>
       <c r="D445" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E445" t="s">
         <v>57</v>
@@ -14725,24 +14782,24 @@
         <v>58</v>
       </c>
       <c r="G445" s="1">
-        <v>46231</v>
+        <v>46126</v>
       </c>
       <c r="H445" s="1">
-        <v>46231</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="446" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A446" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B446" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
       <c r="C446">
         <v>1</v>
       </c>
       <c r="D446" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E446" t="s">
         <v>57</v>
@@ -14751,24 +14808,24 @@
         <v>58</v>
       </c>
       <c r="G446" s="1">
-        <v>46254</v>
+        <v>46128</v>
       </c>
       <c r="H446" s="1">
-        <v>46254</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="447" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A447" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B447" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
       <c r="C447">
         <v>1</v>
       </c>
       <c r="D447" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E447" t="s">
         <v>57</v>
@@ -14777,24 +14834,24 @@
         <v>58</v>
       </c>
       <c r="G447" s="1">
-        <v>46255</v>
+        <v>46132</v>
       </c>
       <c r="H447" s="1">
-        <v>46255</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="448" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A448" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B448" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C448">
         <v>1</v>
       </c>
       <c r="D448" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E448" t="s">
         <v>57</v>
@@ -14803,24 +14860,24 @@
         <v>58</v>
       </c>
       <c r="G448" s="1">
-        <v>46260</v>
+        <v>46161</v>
       </c>
       <c r="H448" s="1">
-        <v>46260</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="449" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A449" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B449" t="s">
-        <v>865</v>
+        <v>869</v>
       </c>
       <c r="C449">
         <v>1</v>
       </c>
       <c r="D449" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E449" t="s">
         <v>57</v>
@@ -14829,24 +14886,24 @@
         <v>58</v>
       </c>
       <c r="G449" s="1">
-        <v>46289</v>
+        <v>46174</v>
       </c>
       <c r="H449" s="1">
-        <v>46289</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="450" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A450" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B450" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
       <c r="C450">
         <v>1</v>
       </c>
       <c r="D450" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E450" t="s">
         <v>57</v>
@@ -14855,24 +14912,24 @@
         <v>58</v>
       </c>
       <c r="G450" s="1">
-        <v>46294</v>
+        <v>46174</v>
       </c>
       <c r="H450" s="1">
-        <v>46294</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="451" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A451" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B451" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="C451">
         <v>1</v>
       </c>
       <c r="D451" t="s">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="E451" t="s">
         <v>57</v>
@@ -14881,24 +14938,24 @@
         <v>58</v>
       </c>
       <c r="G451" s="1">
-        <v>46302</v>
+        <v>46195</v>
       </c>
       <c r="H451" s="1">
-        <v>46323</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="452" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A452" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B452" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="C452">
         <v>1</v>
       </c>
       <c r="D452" t="s">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="E452" t="s">
         <v>57</v>
@@ -14907,24 +14964,24 @@
         <v>58</v>
       </c>
       <c r="G452" s="1">
-        <v>46323</v>
+        <v>46210</v>
       </c>
       <c r="H452" s="1">
-        <v>46323</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="453" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A453" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B453" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="C453">
         <v>1</v>
       </c>
       <c r="D453" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
       <c r="E453" t="s">
         <v>57</v>
@@ -14933,24 +14990,24 @@
         <v>58</v>
       </c>
       <c r="G453" s="1">
-        <v>46323</v>
+        <v>46213</v>
       </c>
       <c r="H453" s="1">
-        <v>46323</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="454" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A454" t="s">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="B454" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="C454">
         <v>1</v>
       </c>
       <c r="D454" t="s">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="E454" t="s">
         <v>57</v>
@@ -14959,200 +15016,200 @@
         <v>58</v>
       </c>
       <c r="G454" s="1">
-        <v>46323</v>
+        <v>46218</v>
       </c>
       <c r="H454" s="1">
-        <v>46323</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="455" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A455" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B455" t="s">
-        <v>872</v>
+        <v>875</v>
       </c>
       <c r="C455">
         <v>1</v>
       </c>
       <c r="D455" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E455" t="s">
-        <v>873</v>
+        <v>77</v>
       </c>
       <c r="F455" t="s">
-        <v>874</v>
+        <v>78</v>
       </c>
       <c r="G455" s="1">
-        <v>46157</v>
+        <v>46226</v>
       </c>
       <c r="H455" s="1">
-        <v>46157</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="456" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A456" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B456" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="C456">
         <v>1</v>
       </c>
       <c r="D456" t="s">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E456" t="s">
-        <v>876</v>
+        <v>57</v>
       </c>
       <c r="F456" t="s">
-        <v>877</v>
+        <v>58</v>
       </c>
       <c r="G456" s="1">
-        <v>46168</v>
+        <v>46227</v>
       </c>
       <c r="H456" s="1">
-        <v>46170</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="457" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A457" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B457" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="C457">
         <v>1</v>
       </c>
       <c r="D457" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E457" t="s">
-        <v>873</v>
+        <v>57</v>
       </c>
       <c r="F457" t="s">
-        <v>874</v>
+        <v>58</v>
       </c>
       <c r="G457" s="1">
-        <v>46218</v>
+        <v>46227</v>
       </c>
       <c r="H457" s="1">
-        <v>46218</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="458" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A458" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B458" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="C458">
         <v>1</v>
       </c>
       <c r="D458" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E458" t="s">
-        <v>873</v>
+        <v>57</v>
       </c>
       <c r="F458" t="s">
-        <v>874</v>
+        <v>58</v>
       </c>
       <c r="G458" s="1">
-        <v>46244</v>
+        <v>46227</v>
       </c>
       <c r="H458" s="1">
-        <v>46244</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="459" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A459" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B459" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="C459">
         <v>1</v>
       </c>
       <c r="D459" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E459" t="s">
-        <v>873</v>
+        <v>77</v>
       </c>
       <c r="F459" t="s">
-        <v>874</v>
+        <v>78</v>
       </c>
       <c r="G459" s="1">
-        <v>46247</v>
+        <v>46230</v>
       </c>
       <c r="H459" s="1">
-        <v>46247</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="460" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A460" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B460" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="C460">
         <v>1</v>
       </c>
       <c r="D460" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E460" t="s">
-        <v>882</v>
+        <v>57</v>
       </c>
       <c r="F460" t="s">
-        <v>883</v>
+        <v>58</v>
       </c>
       <c r="G460" s="1">
-        <v>46247</v>
+        <v>46231</v>
       </c>
       <c r="H460" s="1">
-        <v>46247</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="461" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A461" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B461" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="C461">
         <v>1</v>
       </c>
       <c r="D461" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E461" t="s">
-        <v>873</v>
+        <v>57</v>
       </c>
       <c r="F461" t="s">
-        <v>874</v>
+        <v>58</v>
       </c>
       <c r="G461" s="1">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="H461" s="1">
-        <v>46255</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="462" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A462" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B462" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="C462">
         <v>1</v>
@@ -15161,50 +15218,50 @@
         <v>2</v>
       </c>
       <c r="E462" t="s">
-        <v>873</v>
+        <v>57</v>
       </c>
       <c r="F462" t="s">
-        <v>874</v>
+        <v>58</v>
       </c>
       <c r="G462" s="1">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="H462" s="1">
-        <v>46258</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="463" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A463" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B463" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="C463">
         <v>1</v>
       </c>
       <c r="D463" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E463" t="s">
-        <v>873</v>
+        <v>57</v>
       </c>
       <c r="F463" t="s">
-        <v>874</v>
+        <v>58</v>
       </c>
       <c r="G463" s="1">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="H463" s="1">
-        <v>46265</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="464" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A464" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="B464" t="s">
-        <v>887</v>
+        <v>884</v>
       </c>
       <c r="C464">
         <v>1</v>
@@ -15213,15 +15270,405 @@
         <v>6</v>
       </c>
       <c r="E464" t="s">
+        <v>57</v>
+      </c>
+      <c r="F464" t="s">
+        <v>58</v>
+      </c>
+      <c r="G464" s="1">
+        <v>46289</v>
+      </c>
+      <c r="H464" s="1">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="465" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A465" t="s">
+        <v>858</v>
+      </c>
+      <c r="B465" t="s">
+        <v>885</v>
+      </c>
+      <c r="C465">
+        <v>1</v>
+      </c>
+      <c r="D465" t="s">
+        <v>6</v>
+      </c>
+      <c r="E465" t="s">
+        <v>57</v>
+      </c>
+      <c r="F465" t="s">
+        <v>58</v>
+      </c>
+      <c r="G465" s="1">
+        <v>46294</v>
+      </c>
+      <c r="H465" s="1">
+        <v>46294</v>
+      </c>
+    </row>
+    <row r="466" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A466" t="s">
+        <v>858</v>
+      </c>
+      <c r="B466" t="s">
+        <v>886</v>
+      </c>
+      <c r="C466">
+        <v>1</v>
+      </c>
+      <c r="D466" t="s">
+        <v>125</v>
+      </c>
+      <c r="E466" t="s">
+        <v>57</v>
+      </c>
+      <c r="F466" t="s">
+        <v>58</v>
+      </c>
+      <c r="G466" s="1">
+        <v>46302</v>
+      </c>
+      <c r="H466" s="1">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="467" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A467" t="s">
+        <v>858</v>
+      </c>
+      <c r="B467" t="s">
+        <v>887</v>
+      </c>
+      <c r="C467">
+        <v>1</v>
+      </c>
+      <c r="D467" t="s">
+        <v>125</v>
+      </c>
+      <c r="E467" t="s">
+        <v>57</v>
+      </c>
+      <c r="F467" t="s">
+        <v>58</v>
+      </c>
+      <c r="G467" s="1">
+        <v>46323</v>
+      </c>
+      <c r="H467" s="1">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="468" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A468" t="s">
+        <v>858</v>
+      </c>
+      <c r="B468" t="s">
+        <v>888</v>
+      </c>
+      <c r="C468">
+        <v>1</v>
+      </c>
+      <c r="D468" t="s">
+        <v>125</v>
+      </c>
+      <c r="E468" t="s">
+        <v>57</v>
+      </c>
+      <c r="F468" t="s">
+        <v>58</v>
+      </c>
+      <c r="G468" s="1">
+        <v>46323</v>
+      </c>
+      <c r="H468" s="1">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="469" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A469" t="s">
+        <v>858</v>
+      </c>
+      <c r="B469" t="s">
+        <v>889</v>
+      </c>
+      <c r="C469">
+        <v>1</v>
+      </c>
+      <c r="D469" t="s">
+        <v>125</v>
+      </c>
+      <c r="E469" t="s">
+        <v>57</v>
+      </c>
+      <c r="F469" t="s">
+        <v>58</v>
+      </c>
+      <c r="G469" s="1">
+        <v>46323</v>
+      </c>
+      <c r="H469" s="1">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="470" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A470" t="s">
+        <v>890</v>
+      </c>
+      <c r="B470" t="s">
+        <v>891</v>
+      </c>
+      <c r="C470">
+        <v>1</v>
+      </c>
+      <c r="D470" t="s">
+        <v>2</v>
+      </c>
+      <c r="E470" t="s">
+        <v>892</v>
+      </c>
+      <c r="F470" t="s">
+        <v>893</v>
+      </c>
+      <c r="G470" s="1">
+        <v>46157</v>
+      </c>
+      <c r="H470" s="1">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="471" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A471" t="s">
+        <v>890</v>
+      </c>
+      <c r="B471" t="s">
+        <v>894</v>
+      </c>
+      <c r="C471">
+        <v>1</v>
+      </c>
+      <c r="D471" t="s">
+        <v>2</v>
+      </c>
+      <c r="E471" t="s">
+        <v>895</v>
+      </c>
+      <c r="F471" t="s">
+        <v>896</v>
+      </c>
+      <c r="G471" s="1">
+        <v>46168</v>
+      </c>
+      <c r="H471" s="1">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="472" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A472" t="s">
+        <v>890</v>
+      </c>
+      <c r="B472" t="s">
+        <v>897</v>
+      </c>
+      <c r="C472">
+        <v>1</v>
+      </c>
+      <c r="D472" t="s">
+        <v>2</v>
+      </c>
+      <c r="E472" t="s">
+        <v>892</v>
+      </c>
+      <c r="F472" t="s">
+        <v>893</v>
+      </c>
+      <c r="G472" s="1">
+        <v>46218</v>
+      </c>
+      <c r="H472" s="1">
+        <v>46218</v>
+      </c>
+    </row>
+    <row r="473" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A473" t="s">
+        <v>890</v>
+      </c>
+      <c r="B473" t="s">
+        <v>898</v>
+      </c>
+      <c r="C473">
+        <v>1</v>
+      </c>
+      <c r="D473" t="s">
+        <v>2</v>
+      </c>
+      <c r="E473" t="s">
+        <v>892</v>
+      </c>
+      <c r="F473" t="s">
+        <v>893</v>
+      </c>
+      <c r="G473" s="1">
+        <v>46244</v>
+      </c>
+      <c r="H473" s="1">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="474" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A474" t="s">
+        <v>890</v>
+      </c>
+      <c r="B474" t="s">
+        <v>899</v>
+      </c>
+      <c r="C474">
+        <v>1</v>
+      </c>
+      <c r="D474" t="s">
+        <v>2</v>
+      </c>
+      <c r="E474" t="s">
+        <v>892</v>
+      </c>
+      <c r="F474" t="s">
+        <v>893</v>
+      </c>
+      <c r="G474" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H474" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="475" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A475" t="s">
+        <v>890</v>
+      </c>
+      <c r="B475" t="s">
+        <v>900</v>
+      </c>
+      <c r="C475">
+        <v>1</v>
+      </c>
+      <c r="D475" t="s">
+        <v>2</v>
+      </c>
+      <c r="E475" t="s">
+        <v>901</v>
+      </c>
+      <c r="F475" t="s">
+        <v>902</v>
+      </c>
+      <c r="G475" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H475" s="1">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="476" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A476" t="s">
+        <v>890</v>
+      </c>
+      <c r="B476" t="s">
+        <v>903</v>
+      </c>
+      <c r="C476">
+        <v>1</v>
+      </c>
+      <c r="D476" t="s">
+        <v>2</v>
+      </c>
+      <c r="E476" t="s">
+        <v>892</v>
+      </c>
+      <c r="F476" t="s">
+        <v>893</v>
+      </c>
+      <c r="G476" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H476" s="1">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="477" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A477" t="s">
+        <v>890</v>
+      </c>
+      <c r="B477" t="s">
+        <v>904</v>
+      </c>
+      <c r="C477">
+        <v>1</v>
+      </c>
+      <c r="D477" t="s">
+        <v>2</v>
+      </c>
+      <c r="E477" t="s">
+        <v>892</v>
+      </c>
+      <c r="F477" t="s">
+        <v>893</v>
+      </c>
+      <c r="G477" s="1">
+        <v>46258</v>
+      </c>
+      <c r="H477" s="1">
+        <v>46258</v>
+      </c>
+    </row>
+    <row r="478" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A478" t="s">
+        <v>890</v>
+      </c>
+      <c r="B478" t="s">
+        <v>905</v>
+      </c>
+      <c r="C478">
+        <v>1</v>
+      </c>
+      <c r="D478" t="s">
+        <v>2</v>
+      </c>
+      <c r="E478" t="s">
+        <v>892</v>
+      </c>
+      <c r="F478" t="s">
+        <v>893</v>
+      </c>
+      <c r="G478" s="1">
+        <v>46262</v>
+      </c>
+      <c r="H478" s="1">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="479" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A479" t="s">
+        <v>890</v>
+      </c>
+      <c r="B479" t="s">
+        <v>906</v>
+      </c>
+      <c r="C479">
+        <v>1</v>
+      </c>
+      <c r="D479" t="s">
+        <v>6</v>
+      </c>
+      <c r="E479" t="s">
         <v>13</v>
       </c>
-      <c r="F464" t="s">
+      <c r="F479" t="s">
         <v>14</v>
       </c>
-      <c r="G464" s="1">
+      <c r="G479" s="1">
         <v>46281</v>
       </c>
-      <c r="H464" s="1">
+      <c r="H479" s="1">
         <v>46283</v>
       </c>
     </row>

</xml_diff>